<commit_message>
Refresh daily stock Quote prices
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -9441,10 +9441,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P14" s="472">
-        <v>155.04123</v>
+        <v>155.04118</v>
       </c>
       <c r="Q14" s="4">
-        <v>46283.22280930555</v>
+        <v>46283.225819375</v>
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
@@ -9498,10 +9498,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P15" s="472">
-        <v>185.8024</v>
+        <v>185.7996</v>
       </c>
       <c r="Q15" s="4">
-        <v>46283.22281232639</v>
+        <v>46283.22582570602</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
@@ -9555,10 +9555,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P16" s="472">
-        <v>763.8404</v>
+        <v>763.6584</v>
       </c>
       <c r="Q16" s="4">
-        <v>46283.22282163194</v>
+        <v>46283.22583083333</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
@@ -9612,10 +9612,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P17" s="472">
-        <v>4365.8247</v>
+        <v>4365.8708</v>
       </c>
       <c r="Q17" s="4">
-        <v>46283.2228275</v>
+        <v>46283.225837060185</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -9669,10 +9669,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P18" s="472">
-        <v>718.903</v>
+        <v>719.01659</v>
       </c>
       <c r="Q18" s="4">
-        <v>46283.22282976852</v>
+        <v>46283.225842465275</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -9726,10 +9726,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P19" s="472">
-        <v>220.3737</v>
+        <v>220.3786</v>
       </c>
       <c r="Q19" s="4">
-        <v>46283.22283550926</v>
+        <v>46283.22584795139</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
@@ -9783,10 +9783,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P20" s="472">
-        <v>336.9207</v>
+        <v>336.9242</v>
       </c>
       <c r="Q20" s="4">
-        <v>46283.222844965276</v>
+        <v>46283.22585391204</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
@@ -9840,10 +9840,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P21" s="472">
-        <v>367.2201</v>
+        <v>367.2234</v>
       </c>
       <c r="Q21" s="4">
-        <v>46283.22284712963</v>
+        <v>46283.22585956018</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
@@ -9900,7 +9900,7 @@
         <v>497.3293</v>
       </c>
       <c r="Q22" s="4">
-        <v>46283.222853576386</v>
+        <v>46283.225865567125</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
@@ -9954,10 +9954,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P23" s="472">
-        <v>353.1791</v>
+        <v>353.1767</v>
       </c>
       <c r="Q23" s="4">
-        <v>46283.22285954861</v>
+        <v>46283.22587113426</v>
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
@@ -10011,10 +10011,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P24" s="472">
-        <v>112.1588</v>
+        <v>112.2211</v>
       </c>
       <c r="Q24" s="4">
-        <v>46283.22286451389</v>
+        <v>46283.22587689815</v>
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
@@ -10068,10 +10068,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P25" s="472">
-        <v>111.7174</v>
+        <v>111.717</v>
       </c>
       <c r="Q25" s="4">
-        <v>46283.222870289355</v>
+        <v>46283.225883148145</v>
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
@@ -10128,7 +10128,7 @@
         <v>22.8523</v>
       </c>
       <c r="Q26" s="4">
-        <v>46283.22287981481</v>
+        <v>46283.22588871528</v>
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
@@ -10185,7 +10185,7 @@
         <v>75.6531</v>
       </c>
       <c r="Q27" s="4">
-        <v>46283.22288184028</v>
+        <v>46283.22589429398</v>
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
@@ -10242,7 +10242,7 @@
         <v>135.5947</v>
       </c>
       <c r="Q28" s="4">
-        <v>46283.22289123842</v>
+        <v>46283.225900405094</v>
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
@@ -10299,7 +10299,7 @@
         <v>8.7421</v>
       </c>
       <c r="Q29" s="4">
-        <v>46283.22289350694</v>
+        <v>46283.225906203705</v>
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
@@ -10353,10 +10353,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P30" s="472">
-        <v>44.4966</v>
+        <v>44.5233</v>
       </c>
       <c r="Q30" s="4">
-        <v>46283.22289924768</v>
+        <v>46283.22591173611</v>
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
@@ -10413,7 +10413,7 @@
         <v>115.8148</v>
       </c>
       <c r="Q31" s="4">
-        <v>46283.22290569444</v>
+        <v>46283.225918171294</v>
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
@@ -10470,7 +10470,7 @@
         <v>160.38</v>
       </c>
       <c r="Q32" s="4">
-        <v>46283.222911689816</v>
+        <v>46283.22592355324</v>
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
@@ -10524,10 +10524,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P33" s="472">
-        <v>7.7979</v>
+        <v>7.8072</v>
       </c>
       <c r="Q33" s="4">
-        <v>46283.222919687505</v>
+        <v>46283.22592967592</v>
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
@@ -10581,10 +10581,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P34" s="472">
-        <v>34.5741</v>
+        <v>34.5733</v>
       </c>
       <c r="Q34" s="4">
-        <v>46283.22292342593</v>
+        <v>46283.22593542824</v>
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
@@ -10638,10 +10638,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P35" s="472">
-        <v>24.4487</v>
+        <v>24.4175</v>
       </c>
       <c r="Q35" s="4">
-        <v>46283.22293134259</v>
+        <v>46283.22594123842</v>
       </c>
       <c r="R35" s="4" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="P36" s="472"/>
       <c r="Q36" s="4">
-        <v>46283.2229340625</v>
+        <v>46283.22594729167</v>
       </c>
       <c r="R36" s="4"/>
       <c r="S36" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Keep daily price dates readable and missing prices blank
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Rd8343663e6f14fe8"/>
-    <sheet name="单币测算" sheetId="2" r:id="Rd15010c2fbee456b"/>
-    <sheet name="全RWA预算" sheetId="3" r:id="R3d35aa659a134bb8"/>
-    <sheet name="选中Quote曲线" sheetId="4" r:id="Rbd71d72a627542fe"/>
-    <sheet name="Quote参数" sheetId="5" r:id="Rfc20555e564e4181"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R07960734c4244702"/>
+    <sheet name="单币测算" sheetId="2" r:id="R790cfe9196f04fe7"/>
+    <sheet name="全RWA预算" sheetId="3" r:id="Rd4c0c5c45eae4e9c"/>
+    <sheet name="选中Quote曲线" sheetId="4" r:id="R86f2a228e9f9400c"/>
+    <sheet name="Quote参数" sheetId="5" r:id="R1cc01e53c52e4152"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -18,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="11">
+  <x:numFmts count="12">
     <x:numFmt numFmtId="200" formatCode="#,##0.00000000"/>
     <x:numFmt numFmtId="201" formatCode="0.00%"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
@@ -30,6 +30,7 @@
     <x:numFmt numFmtId="208" formatCode="0.0000000000"/>
     <x:numFmt numFmtId="209" formatCode="General"/>
     <x:numFmt numFmtId="210" formatCode="0.000000"/>
+    <x:numFmt numFmtId="211" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
   <x:fonts count="28">
     <x:font>
@@ -628,7 +629,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="473">
+  <x:cellXfs count="475">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1900,6 +1901,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="210" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -9400,7 +9405,7 @@
         <v>说明</v>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="C14" s="24" t="n">
         <v>1</v>
       </c>
@@ -9443,21 +9448,21 @@
       <c r="P14" s="472">
         <v>155.04118</v>
       </c>
-      <c r="Q14" s="4">
+      <c r="Q14" s="473">
         <v>46283.225819375</v>
       </c>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R14" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x977daffc095b33872e2741c19568925015c35b4d</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S14" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="C15" s="25" t="n">
         <v>2</v>
       </c>
@@ -9500,21 +9505,21 @@
       <c r="P15" s="472">
         <v>185.7996</v>
       </c>
-      <c r="Q15" s="4">
+      <c r="Q15" s="473">
         <v>46283.22582570602</v>
       </c>
-      <c r="R15" s="4" t="inlineStr">
+      <c r="R15" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xd7d30f434b12f7ed9b0ae11ff1c754745a10ad52</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr">
+      <c r="S15" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="C16" s="25" t="n">
         <v>3</v>
       </c>
@@ -9557,21 +9562,21 @@
       <c r="P16" s="472">
         <v>763.6584</v>
       </c>
-      <c r="Q16" s="4">
+      <c r="Q16" s="473">
         <v>46283.22583083333</v>
       </c>
-      <c r="R16" s="4" t="inlineStr">
+      <c r="R16" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x7aa6d92fc369a8c1edc631a3aac44efb0808ddbf</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
+      <c r="S16" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="C17" s="25" t="n">
         <v>4</v>
       </c>
@@ -9614,21 +9619,21 @@
       <c r="P17" s="472">
         <v>4365.8708</v>
       </c>
-      <c r="Q17" s="4">
+      <c r="Q17" s="473">
         <v>46283.225837060185</v>
       </c>
-      <c r="R17" s="4" t="inlineStr">
+      <c r="R17" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x83a0a8a723262651ae9c54bbba929f167443bc59</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
+      <c r="S17" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="C18" s="25" t="n">
         <v>5</v>
       </c>
@@ -9671,21 +9676,21 @@
       <c r="P18" s="472">
         <v>719.01659</v>
       </c>
-      <c r="Q18" s="4">
+      <c r="Q18" s="473">
         <v>46283.225842465275</v>
       </c>
-      <c r="R18" s="4" t="inlineStr">
+      <c r="R18" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xe531fcb1f5a195de7608b9f4f9518544c2cdb693</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
+      <c r="S18" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="C19" s="25" t="n">
         <v>6</v>
       </c>
@@ -9728,21 +9733,21 @@
       <c r="P19" s="472">
         <v>220.3786</v>
       </c>
-      <c r="Q19" s="4">
+      <c r="Q19" s="473">
         <v>46283.22584795139</v>
       </c>
-      <c r="R19" s="4" t="inlineStr">
+      <c r="R19" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x8fb4243b553ac29ba088acf00b9b7da24bd6690c</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
+      <c r="S19" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="C20" s="25" t="n">
         <v>7</v>
       </c>
@@ -9785,21 +9790,21 @@
       <c r="P20" s="472">
         <v>336.9242</v>
       </c>
-      <c r="Q20" s="4">
+      <c r="Q20" s="473">
         <v>46283.22585391204</v>
       </c>
-      <c r="R20" s="4" t="inlineStr">
+      <c r="R20" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xe9b9998b2ec5430d2246c7f1f8d9f298c97d7365</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
+      <c r="S20" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="C21" s="25" t="n">
         <v>8</v>
       </c>
@@ -9842,21 +9847,21 @@
       <c r="P21" s="472">
         <v>367.2234</v>
       </c>
-      <c r="Q21" s="4">
+      <c r="Q21" s="473">
         <v>46283.22585956018</v>
       </c>
-      <c r="R21" s="4" t="inlineStr">
+      <c r="R21" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xb0f5e5400e8f0f7c242f2b7740c004f020579c41</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
+      <c r="S21" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="C22" s="25" t="n">
         <v>9</v>
       </c>
@@ -9899,21 +9904,21 @@
       <c r="P22" s="472">
         <v>497.3293</v>
       </c>
-      <c r="Q22" s="4">
+      <c r="Q22" s="473">
         <v>46283.225865567125</v>
       </c>
-      <c r="R22" s="4" t="inlineStr">
+      <c r="R22" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x5018b018ceb7645c927c5cf246786f89ebcbe7ea</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
+      <c r="S22" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="36" customHeight="1">
       <c r="C23" s="25" t="n">
         <v>10</v>
       </c>
@@ -9956,21 +9961,21 @@
       <c r="P23" s="472">
         <v>353.1767</v>
       </c>
-      <c r="Q23" s="4">
+      <c r="Q23" s="473">
         <v>46283.22587113426</v>
       </c>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="R23" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x89001d846f7ca36ee089f73eefc25657e1798144</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S23" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="C24" s="25" t="n">
         <v>11</v>
       </c>
@@ -10013,21 +10018,21 @@
       <c r="P24" s="472">
         <v>112.2211</v>
       </c>
-      <c r="Q24" s="4">
+      <c r="Q24" s="473">
         <v>46283.22587689815</v>
       </c>
-      <c r="R24" s="4" t="inlineStr">
+      <c r="R24" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xfeef70ff6f58f0a900e28a77e5a8945afb343923</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr">
+      <c r="S24" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="C25" s="25" t="n">
         <v>12</v>
       </c>
@@ -10070,21 +10075,21 @@
       <c r="P25" s="472">
         <v>111.717</v>
       </c>
-      <c r="Q25" s="4">
+      <c r="Q25" s="473">
         <v>46283.225883148145</v>
       </c>
-      <c r="R25" s="4" t="inlineStr">
+      <c r="R25" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xfd95cb1391999006eb91797a7c62acfe88b20292</t>
         </is>
       </c>
-      <c r="S25" s="4" t="inlineStr">
+      <c r="S25" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="20" customHeight="1">
+    <row r="26" ht="36" customHeight="1">
       <c r="C26" s="25" t="n">
         <v>13</v>
       </c>
@@ -10127,21 +10132,21 @@
       <c r="P26" s="472">
         <v>22.8523</v>
       </c>
-      <c r="Q26" s="4">
+      <c r="Q26" s="473">
         <v>46283.22588871528</v>
       </c>
-      <c r="R26" s="4" t="inlineStr">
+      <c r="R26" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x908d49048eb3a7bedfd238972403842805eaf2be</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr">
+      <c r="S26" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
+    <row r="27" ht="36" customHeight="1">
       <c r="C27" s="25" t="n">
         <v>14</v>
       </c>
@@ -10184,21 +10189,21 @@
       <c r="P27" s="472">
         <v>75.6531</v>
       </c>
-      <c r="Q27" s="4">
+      <c r="Q27" s="473">
         <v>46283.22589429398</v>
       </c>
-      <c r="R27" s="4" t="inlineStr">
+      <c r="R27" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xafab4441d8b354bba790229c0e235e7e6187b3d0</t>
         </is>
       </c>
-      <c r="S27" s="4" t="inlineStr">
+      <c r="S27" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
+    <row r="28" ht="36" customHeight="1">
       <c r="C28" s="25" t="n">
         <v>15</v>
       </c>
@@ -10241,21 +10246,21 @@
       <c r="P28" s="472">
         <v>135.5947</v>
       </c>
-      <c r="Q28" s="4">
+      <c r="Q28" s="473">
         <v>46283.225900405094</v>
       </c>
-      <c r="R28" s="4" t="inlineStr">
+      <c r="R28" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x692081209619735f25700557078ab084d3e5d007</t>
         </is>
       </c>
-      <c r="S28" s="4" t="inlineStr">
+      <c r="S28" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="20" customHeight="1">
+    <row r="29" ht="36" customHeight="1">
       <c r="C29" s="25" t="n">
         <v>16</v>
       </c>
@@ -10298,21 +10303,21 @@
       <c r="P29" s="472">
         <v>8.7421</v>
       </c>
-      <c r="Q29" s="4">
+      <c r="Q29" s="473">
         <v>46283.225906203705</v>
       </c>
-      <c r="R29" s="4" t="inlineStr">
+      <c r="R29" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x9aadbd51515432dbb77c0a7f69c2b2c211f0c837</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr">
+      <c r="S29" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="20" customHeight="1">
+    <row r="30" ht="36" customHeight="1">
       <c r="C30" s="25" t="n">
         <v>17</v>
       </c>
@@ -10355,21 +10360,21 @@
       <c r="P30" s="472">
         <v>44.5233</v>
       </c>
-      <c r="Q30" s="4">
+      <c r="Q30" s="473">
         <v>46283.22591173611</v>
       </c>
-      <c r="R30" s="4" t="inlineStr">
+      <c r="R30" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xd5c0572126a707196aaba2b6952d67fc2a140651</t>
         </is>
       </c>
-      <c r="S30" s="4" t="inlineStr">
+      <c r="S30" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
+    <row r="31" ht="36" customHeight="1">
       <c r="C31" s="25" t="n">
         <v>18</v>
       </c>
@@ -10412,21 +10417,21 @@
       <c r="P31" s="472">
         <v>115.8148</v>
       </c>
-      <c r="Q31" s="4">
+      <c r="Q31" s="473">
         <v>46283.225918171294</v>
       </c>
-      <c r="R31" s="4" t="inlineStr">
+      <c r="R31" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x3d7d950377eca7b4af7233716ff17def00ab2045</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr">
+      <c r="S31" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
+    <row r="32" ht="36" customHeight="1">
       <c r="C32" s="25" t="n">
         <v>19</v>
       </c>
@@ -10469,21 +10474,21 @@
       <c r="P32" s="472">
         <v>160.38</v>
       </c>
-      <c r="Q32" s="4">
+      <c r="Q32" s="473">
         <v>46283.22592355324</v>
       </c>
-      <c r="R32" s="4" t="inlineStr">
+      <c r="R32" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0xcc992887e9cee37a698541e2f6d1675453fbcfcc</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr">
+      <c r="S32" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
+    <row r="33" ht="36" customHeight="1">
       <c r="C33" s="25" t="n">
         <v>20</v>
       </c>
@@ -10526,21 +10531,21 @@
       <c r="P33" s="472">
         <v>7.8072</v>
       </c>
-      <c r="Q33" s="4">
+      <c r="Q33" s="473">
         <v>46283.22592967592</v>
       </c>
-      <c r="R33" s="4" t="inlineStr">
+      <c r="R33" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x1f7083a138f980b60eb1582f01ca3b1d6c46ad10</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr">
+      <c r="S33" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
+    <row r="34" ht="36" customHeight="1">
       <c r="C34" s="25" t="n">
         <v>21</v>
       </c>
@@ -10583,21 +10588,21 @@
       <c r="P34" s="472">
         <v>34.5733</v>
       </c>
-      <c r="Q34" s="4">
+      <c r="Q34" s="473">
         <v>46283.22593542824</v>
       </c>
-      <c r="R34" s="4" t="inlineStr">
+      <c r="R34" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x8768c8969e177575e37435b8295afa2dfb231c86</t>
         </is>
       </c>
-      <c r="S34" s="4" t="inlineStr">
+      <c r="S34" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
+    <row r="35" ht="36" customHeight="1">
       <c r="C35" s="25" t="n">
         <v>22</v>
       </c>
@@ -10640,21 +10645,21 @@
       <c r="P35" s="472">
         <v>24.4175</v>
       </c>
-      <c r="Q35" s="4">
+      <c r="Q35" s="473">
         <v>46283.22594123842</v>
       </c>
-      <c r="R35" s="4" t="inlineStr">
+      <c r="R35" s="474" t="inlineStr">
         <is>
           <t>https://dexscreener.com/bsc/0x52a427db0b2d9154a5f4ad09d22f3792f754b6fc</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr">
+      <c r="S35" s="474" t="inlineStr">
         <is>
           <t>每日 Quote 代币池价；本地可手动更新</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
+    <row r="36" ht="36" customHeight="1">
       <c r="C36" s="26" t="n">
         <v>23</v>
       </c>
@@ -10694,12 +10699,20 @@
       <c r="O36" s="34" t="str">
         <v>2026-09-10</v>
       </c>
-      <c r="P36" s="472"/>
-      <c r="Q36" s="4">
+      <c r="P36" s="472" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q36" s="473">
         <v>46283.22594729167</v>
       </c>
-      <c r="R36" s="4"/>
-      <c r="S36" s="4" t="inlineStr">
+      <c r="R36" s="474" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S36" s="474" t="inlineStr">
         <is>
           <t>暂无合格池价；可手动输入</t>
         </is>

</xml_diff>

<commit_message>
Compact Excel layout and expose tax-inclusive budget fees
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Re00aa08619b444e4"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R9873abdba5834a61"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R2719262e5d164f66"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R782263309ec44554"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -27,7 +27,7 @@
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0.0000000000"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -79,8 +79,13 @@
       <x:name val="Arial"/>
     </x:font>
     <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF667085"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:b/>
-      <x:sz val="13"/>
+      <x:sz val="12"/>
       <x:color rgb="FF365F20"/>
       <x:name val="Arial"/>
     </x:font>
@@ -110,12 +115,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE8F3DD"/>
+        <x:fgColor rgb="FFEAF3FA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEAF3FA"/>
+        <x:fgColor rgb="FFE8F3DD"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -153,7 +158,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -303,10 +308,19 @@
     <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -342,19 +356,16 @@
     <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -384,22 +395,22 @@
     <x:xf numFmtId="209" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="10" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="10" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="11" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="11" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="11" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -681,7 +692,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetPr>
+    <outlinePr summaryBelow="0" showOutlineSymbols="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="2" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="2" hidden="0" customWidth="1"/>
@@ -697,7 +711,7 @@
     <col min="12" max="12" width="17" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="6" customHeight="1">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -711,7 +725,7 @@
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
-    <row r="2" ht="26" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="4" t="str">
@@ -727,7 +741,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="5" t="str">
@@ -743,7 +757,7 @@
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="6" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -757,7 +771,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" ht="27" customHeight="1">
+    <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="8" t="str">
@@ -773,7 +787,7 @@
       <c r="K5" s="8"/>
       <c r="L5" s="8"/>
     </row>
-    <row r="6" ht="26" customHeight="1">
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="42" t="str">
@@ -793,7 +807,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" ht="26" customHeight="1">
+    <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="35" t="str">
@@ -819,7 +833,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
     </row>
-    <row r="8" ht="26" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="35" t="str">
@@ -847,7 +861,7 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
     </row>
-    <row r="9" ht="26" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="35" t="str">
@@ -869,15 +883,11 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
     </row>
-    <row r="10" ht="26" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="35" t="str">
-        <v>资金预留 / Quote</v>
-      </c>
-      <c r="D10" s="47" t="n">
-        <v>0</v>
-      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="35" t="str">
         <v>Holder 地址数</v>
@@ -891,7 +901,7 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
     </row>
-    <row r="11" ht="26" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -909,21 +919,25 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
     </row>
-    <row r="12" ht="26" customHeight="1">
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="F12" s="35" t="str">
+        <v>资金预留 / Quote</v>
+      </c>
+      <c r="G12" s="47" t="n">
+        <v>0</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
     </row>
-    <row r="13" ht="26" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="48" t="str">
@@ -939,7 +953,7 @@
       <c r="K13" s="48"/>
       <c r="L13" s="48"/>
     </row>
-    <row r="14" ht="26" customHeight="1">
+    <row r="14" ht="6" customHeight="1">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -953,7 +967,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
     </row>
-    <row r="15" ht="26" customHeight="1">
+    <row r="15" ht="6" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -967,7 +981,7 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
     </row>
-    <row r="16" ht="26" customHeight="1">
+    <row r="16" ht="6" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -981,7 +995,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" ht="27" customHeight="1">
+    <row r="17" ht="24" customHeight="1">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="8" t="str">
@@ -997,53 +1011,55 @@
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
     </row>
-    <row r="18" ht="38" customHeight="1">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="35" t="str">
         <v>建议总资金 / Quote</v>
       </c>
-      <c r="D18" s="64">
+      <c r="D18" s="67">
         <f>IF(LEFT($D$23,2)&lt;&gt;"可达","",IF($D$21="","",SUM($D$21,$G$21,$J$21,$D$22)))</f>
       </c>
-      <c r="E18" s="50">
+      <c r="E18" s="55">
         <f>$D$7</f>
       </c>
       <c r="F18" s="35" t="str">
         <v>折合 USDT（不含 Gas）</v>
       </c>
-      <c r="G18" s="64">
+      <c r="G18" s="67">
         <f>IF(OR($D$18="",$D$24=""),"",$D$18*$D$24)</f>
       </c>
-      <c r="H18" s="50" t="str">
+      <c r="H18" s="55" t="str">
         <v>USDT</v>
       </c>
       <c r="I18" s="35" t="str">
         <v>Gas 储备 / BNB</v>
       </c>
-      <c r="J18" s="64">
+      <c r="J18" s="67">
         <f>$G$22*MAX(0,$G$11)</f>
       </c>
-      <c r="K18" s="50" t="str">
+      <c r="K18" s="55" t="str">
         <v>BNB</v>
       </c>
-      <c r="L18" s="50"/>
-    </row>
-    <row r="19" ht="26" customHeight="1">
+      <c r="L18" s="55"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-    </row>
-    <row r="20" ht="26" customHeight="1">
+      <c r="C19" s="50" t="str">
+        <v>Quote 资金构成：预算控筹率理论资金 + 额外内盘资金 + 资金预留 + 洗筹损耗</v>
+      </c>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+    </row>
+    <row r="20" ht="6" customHeight="1">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1057,46 +1073,46 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" ht="26" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="35" t="str">
-        <v>理论累计投入 / Quote</v>
-      </c>
-      <c r="D21" s="51">
+      <c r="C21" s="35">
+        <f>"预算 "&amp;TEXT($J$22,"0%")&amp;" 理论资金 / Quote"</f>
+      </c>
+      <c r="D21" s="53">
         <f>IF(LEFT($D$23,2)&lt;&gt;"可达","",IF($J$35="","",$J$31+$J$35))</f>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="35" t="str">
         <v>额外内盘资金 / Quote</v>
       </c>
-      <c r="G21" s="51">
+      <c r="G21" s="53">
         <f>IF(LEFT($D$23,2)&lt;&gt;"可达","",$J$31*MAX(0,$G$7-1))</f>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="35" t="str">
-        <v>洗筹预算 / Quote</v>
-      </c>
-      <c r="J21" s="51">
+        <v>洗筹损耗 / Quote</v>
+      </c>
+      <c r="J21" s="53">
         <f>IF(LEFT($D$23,2)&lt;&gt;"可达","",IF($J$36="","",$J$36*$J$37))</f>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" ht="26" customHeight="1">
+    <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="35" t="str">
         <v>资金预留 / Quote</v>
       </c>
-      <c r="D22" s="51">
-        <f>MAX(0,$D$10)</f>
+      <c r="D22" s="53">
+        <f>MAX(0,$G$12)</f>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="35" t="str">
         <v>地址总数</v>
       </c>
-      <c r="G22" s="54">
+      <c r="G22" s="57">
         <f>MAX(0,$G$8)*MAX(0,$G$7)+MAX(0,$G$9)+MAX(0,$G$10)</f>
       </c>
       <c r="H22" s="2"/>
@@ -1109,125 +1125,159 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" ht="40" customHeight="1">
+    <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="35" t="str">
         <v>目标是否可达</v>
       </c>
-      <c r="D23" s="56">
+      <c r="D23" s="59">
         <f>IF($J$41&lt;&gt;"参数有效",$J$41,IF(OR($D$8&lt;80%,$D$8&gt;=100%),"目标控筹率无效",IF(OR($J$7&lt;0,$J$7&gt;10%,$J$8&lt;0,$J$8&gt;10%),"税率无效",IF($J$22&gt;=$G$23,"目标+1%不可达","可达"))))</f>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="35" t="str">
         <v>当前控筹上限</v>
       </c>
-      <c r="G23" s="53">
+      <c r="G23" s="56">
         <f>$G$33+(1-$J$7)*$G$38/1000000000</f>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="35" t="str">
         <v>资金口径</v>
       </c>
-      <c r="J23" s="51" t="str">
+      <c r="J23" s="53" t="str">
         <v>Quote 预算 + 单独 Gas</v>
       </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" ht="40" customHeight="1">
+    <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="35" t="str">
         <v>使用价格 / USDT</v>
       </c>
-      <c r="D24" s="51">
+      <c r="D24" s="53">
         <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE),""))</f>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="35" t="str">
         <v>行情时间 / UTC</v>
       </c>
-      <c r="G24" s="55">
+      <c r="G24" s="58">
         <f>IF(VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE))</f>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="35" t="str">
         <v>价格状态</v>
       </c>
-      <c r="J24" s="51">
+      <c r="J24" s="53">
         <f>IF($D$9&lt;&gt;"",IF($D$24="","手动价格无效","手动价格"),IF($D$24="","缺少价格","每日行情"))</f>
       </c>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" ht="26" customHeight="1">
+    <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="35" t="str">
         <v>价格采用方式</v>
       </c>
-      <c r="D25" s="51">
+      <c r="D25" s="53">
         <f>IF($D$9&lt;&gt;"","手动覆盖","每日行情")</f>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="51"/>
+      <c r="G25" s="53"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2" t="str">
         <v>价格缺失时 USDT 结果留空</v>
       </c>
-      <c r="J25" s="51"/>
+      <c r="J25" s="53"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" ht="26" customHeight="1">
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="C26" s="35" t="str">
+        <v>内盘基础手续费</v>
+      </c>
+      <c r="D26" s="52">
+        <f>$G$31</f>
+      </c>
       <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="F26" s="35" t="str">
+        <v>外盘 LP 手续费</v>
+      </c>
+      <c r="G26" s="52">
+        <f>$G$32</f>
+      </c>
       <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="I26" s="35" t="str">
+        <v>洗筹双边总费率</v>
+      </c>
+      <c r="J26" s="52">
+        <f>SUM(G27,J27)</f>
+      </c>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" ht="26" customHeight="1">
+    <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="C27" s="35" t="str">
+        <v>内盘买入含税费率</v>
+      </c>
+      <c r="D27" s="52">
+        <f>$G$31+$J$7</f>
+      </c>
       <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="F27" s="35" t="str">
+        <v>外盘买入含税费率</v>
+      </c>
+      <c r="G27" s="52">
+        <f>$G$32+$J$7</f>
+      </c>
       <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+      <c r="I27" s="35" t="str">
+        <v>外盘卖出含税费率</v>
+      </c>
+      <c r="J27" s="52">
+        <f>$G$32+$J$8</f>
+      </c>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" ht="26" customHeight="1">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="C28" s="35" t="str">
+        <v>沉没成本 / Quote</v>
+      </c>
+      <c r="D28" s="53">
+        <f>E115</f>
+      </c>
       <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="F28" s="35" t="str">
+        <v>一套内盘打满 / Quote</v>
+      </c>
+      <c r="G28" s="53">
+        <f>$J$31</f>
+      </c>
       <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-    </row>
-    <row r="29" ht="27" customHeight="1">
+      <c r="I28" s="51" t="str">
+        <v>费率为预算加总口径；双边合计用于 FDV 洗筹预算。沉没成本与一套打满仅作参考，不重复计入总额。</v>
+      </c>
+      <c r="J28" s="51"/>
+      <c r="K28" s="51"/>
+      <c r="L28" s="51"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" collapsed="1">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="8" t="str">
-        <v>三、模型信息与计算口径</v>
+        <v>三、模型信息与计算口径（默认折叠，点左侧 + 展开）</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
@@ -1239,7 +1289,7 @@
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
     </row>
-    <row r="30" ht="26" customHeight="1">
+    <row r="30" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="42" t="str">
@@ -1259,313 +1309,313 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" ht="36" customHeight="1">
+    <row r="31" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="35" t="str">
         <v>Quote 名称</v>
       </c>
-      <c r="D31" s="56">
+      <c r="D31" s="59">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,2,FALSE)</f>
       </c>
       <c r="E31" s="35"/>
       <c r="F31" s="35" t="str">
         <v>内盘基础费</v>
       </c>
-      <c r="G31" s="53">
+      <c r="G31" s="56">
         <f>0.01</f>
       </c>
       <c r="H31" s="2"/>
       <c r="I31" s="35" t="str">
         <v>一套内盘打满 / Quote</v>
       </c>
-      <c r="J31" s="51">
+      <c r="J31" s="53">
         <f>$G$34*(1+$G$31+$J$7)</f>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" ht="36" customHeight="1">
+    <row r="32" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="35" t="str">
         <v>Quote 合约</v>
       </c>
-      <c r="D32" s="59">
+      <c r="D32" s="62">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,3,FALSE)</f>
       </c>
       <c r="E32" s="35"/>
       <c r="F32" s="35" t="str">
         <v>外盘 LP 费</v>
       </c>
-      <c r="G32" s="53">
+      <c r="G32" s="56">
         <f>0.0025</f>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="35" t="str">
         <v>目标+1% Pool TOKEN</v>
       </c>
-      <c r="J32" s="61">
+      <c r="J32" s="64">
         <f>IF($J$39="","",$G$38-$J$39)</f>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" ht="26" customHeight="1">
+    <row r="33" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
-      <c r="D33" s="56"/>
+      <c r="D33" s="59"/>
       <c r="E33" s="35"/>
       <c r="F33" s="35" t="str">
         <v>毕业控筹率</v>
       </c>
-      <c r="G33" s="53">
+      <c r="G33" s="56">
         <f>0.8</f>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="35" t="str">
         <v>目标+1% Pool Quote</v>
       </c>
-      <c r="J33" s="51">
+      <c r="J33" s="53">
         <f>IF($J$32="","",$G$40/$J$32)</f>
       </c>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" ht="26" customHeight="1">
+    <row r="34" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="35" t="str">
         <v>Decimals</v>
       </c>
-      <c r="D34" s="57">
+      <c r="D34" s="60">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,4,FALSE)</f>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="35" t="str">
         <v>毕业真实 Quote</v>
       </c>
-      <c r="G34" s="51">
+      <c r="G34" s="53">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,8,FALSE)</f>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="35" t="str">
         <v>外盘净增加 / Quote</v>
       </c>
-      <c r="J34" s="51">
+      <c r="J34" s="53">
         <f>IF($J$33="","",MAX(0,$J$33-$G$34))</f>
       </c>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" ht="26" customHeight="1">
+    <row r="35" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="35" t="str">
         <v>总供应量</v>
       </c>
-      <c r="D35" s="54" t="n">
+      <c r="D35" s="57" t="n">
         <v>1000000000</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="35" t="str">
         <v>内盘初始 TOKEN</v>
       </c>
-      <c r="G35" s="61">
+      <c r="G35" s="64">
         <f>$D$35+$G$42</f>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="35" t="str">
         <v>外盘含费投入 / Quote</v>
       </c>
-      <c r="J35" s="51">
+      <c r="J35" s="53">
         <f>IF($J$34="","",$J$34*(1+$G$32))</f>
       </c>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" ht="36" customHeight="1">
+    <row r="36" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="35" t="str">
         <v>协议参数时点</v>
       </c>
-      <c r="D36" s="60" t="str">
+      <c r="D36" s="63" t="str">
         <v>2026-09-10 / block 121074671</v>
       </c>
       <c r="E36" s="35"/>
       <c r="F36" s="35" t="str">
         <v>虚拟 Quote r</v>
       </c>
-      <c r="G36" s="51">
+      <c r="G36" s="53">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,5,FALSE)</f>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="35" t="str">
         <v>目标+1% FDV / Quote</v>
       </c>
-      <c r="J36" s="51">
+      <c r="J36" s="53">
         <f>IF($J$33="","",$J$33/$J$32*1000000000)</f>
       </c>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" ht="26" customHeight="1">
+    <row r="37" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="35" t="str">
         <v>外盘机制</v>
       </c>
-      <c r="D37" s="56" t="str">
+      <c r="D37" s="59" t="str">
         <v>Pancake V3</v>
       </c>
       <c r="E37" s="35"/>
       <c r="F37" s="35" t="str">
         <v>内盘 k</v>
       </c>
-      <c r="G37" s="58">
+      <c r="G37" s="61">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,7,FALSE)</f>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="35" t="str">
         <v>洗筹总费率</v>
       </c>
-      <c r="J37" s="53">
+      <c r="J37" s="56">
         <f>$G$32*2+$J$7+$J$8</f>
       </c>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" ht="36" customHeight="1">
+    <row r="38" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="35" t="str">
         <v>费用方向</v>
       </c>
-      <c r="D38" s="56" t="str">
+      <c r="D38" s="59" t="str">
         <v>内盘买税加收 Quote；DEX 买税扣 TOKEN 输出</v>
       </c>
       <c r="E38" s="35"/>
       <c r="F38" s="35" t="str">
         <v>外盘初始 TOKEN</v>
       </c>
-      <c r="G38" s="61">
+      <c r="G38" s="64">
         <f>1000000000*(1-0.8)</f>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="35" t="str">
         <v>外盘净控筹 TOKEN</v>
       </c>
-      <c r="J38" s="61">
+      <c r="J38" s="64">
         <f>IF($J$22&lt;$G$23,MAX(0,($J$22-$G$33)*1000000000),"")</f>
       </c>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" ht="36" customHeight="1">
+    <row r="39" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="35" t="str">
         <v>洗筹口径</v>
       </c>
-      <c r="D39" s="56" t="str">
+      <c r="D39" s="59" t="str">
         <v>目标+1% FDV ×（2×LP费 + 买税 + 卖税）</v>
       </c>
       <c r="E39" s="35"/>
       <c r="F39" s="35" t="str">
         <v>外盘初始 Quote</v>
       </c>
-      <c r="G39" s="51">
+      <c r="G39" s="53">
         <f>$G$34</f>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="35" t="str">
         <v>外盘需扫 TOKEN</v>
       </c>
-      <c r="J39" s="61">
+      <c r="J39" s="64">
         <f>IF($J$38="","",$J$38/(1-$J$7))</f>
       </c>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
     </row>
-    <row r="40" ht="26" customHeight="1">
+    <row r="40" ht="20" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
-      <c r="D40" s="56"/>
+      <c r="D40" s="59"/>
       <c r="E40" s="35"/>
       <c r="F40" s="35" t="str">
         <v>外盘 k</v>
       </c>
-      <c r="G40" s="58">
+      <c r="G40" s="61">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$N$36,10,FALSE)</f>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
-      <c r="J40" s="51"/>
+      <c r="J40" s="53"/>
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
     </row>
-    <row r="41" ht="36" customHeight="1">
+    <row r="41" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
-      <c r="D41" s="51"/>
+      <c r="D41" s="53"/>
       <c r="E41" s="2"/>
       <c r="F41" s="35" t="str">
         <v>协议来源</v>
       </c>
-      <c r="G41" s="62" t="str">
+      <c r="G41" s="65" t="str">
         <v>Quote参数页</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="35" t="str">
         <v>输入检查</v>
       </c>
-      <c r="J41" s="56">
-        <f>IF(COUNT($D$8,$D$10,$G$7:$G$11,$J$7:$J$8)&lt;&gt;9,"缺少或非数值参数",IF(OR($G$7&lt;1,$G$8&lt;0,$G$9&lt;0,$G$10&lt;0,$G$11&lt;0,$D$10&lt;0,$G$7&lt;&gt;INT($G$7),$G$8&lt;&gt;INT($G$8),$G$9&lt;&gt;INT($G$9),$G$10&lt;&gt;INT($G$10)),"地址/Gas/预留参数无效","参数有效"))</f>
+      <c r="J41" s="59">
+        <f>IF(COUNT($D$8,$G$7:$G$12,$J$7:$J$8)&lt;&gt;9,"缺少或非数值参数",IF(OR($G$7&lt;1,$G$8&lt;0,$G$9&lt;0,$G$10&lt;0,$G$11&lt;0,$G$12&lt;0,$G$7&lt;&gt;INT($G$7),$G$8&lt;&gt;INT($G$8),$G$9&lt;&gt;INT($G$9),$G$10&lt;&gt;INT($G$10)),"地址/Gas/预留参数无效","参数有效"))</f>
       </c>
       <c r="K41" s="35"/>
       <c r="L41" s="35"/>
     </row>
-    <row r="42" ht="36" customHeight="1">
+    <row r="42" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="51"/>
+      <c r="D42" s="53"/>
       <c r="E42" s="2"/>
       <c r="F42" s="35" t="str">
         <v>虚拟 TOKEN h</v>
       </c>
-      <c r="G42" s="62">
+      <c r="G42" s="65">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,6,FALSE)</f>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
-      <c r="J42" s="51"/>
+      <c r="J42" s="53"/>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
     </row>
-    <row r="43" ht="36" customHeight="1">
+    <row r="43" ht="36" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
-      <c r="D43" s="51"/>
+      <c r="D43" s="53"/>
       <c r="E43" s="2"/>
       <c r="F43" s="35" t="str">
         <v>买税方向</v>
       </c>
-      <c r="G43" s="63" t="str">
+      <c r="G43" s="66" t="str">
         <v>TOKEN 输出端</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
-      <c r="J43" s="51"/>
+      <c r="J43" s="53"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
     </row>
-    <row r="44" ht="26" customHeight="1">
+    <row r="44" ht="6" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1579,7 +1629,7 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
-    <row r="45" ht="26" customHeight="1">
+    <row r="45" ht="6" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1593,7 +1643,7 @@
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
     </row>
-    <row r="46" ht="26" customHeight="1">
+    <row r="46" ht="6" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1607,7 +1657,7 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
     </row>
-    <row r="47" ht="27" customHeight="1">
+    <row r="47" ht="24" customHeight="1">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="8" t="str">
@@ -1623,59 +1673,59 @@
       <c r="K47" s="8"/>
       <c r="L47" s="8"/>
     </row>
-    <row r="48" ht="38" customHeight="1">
+    <row r="48" ht="30" customHeight="1">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
-      <c r="C48" s="68" t="str">
+      <c r="C48" s="70" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D48" s="68" t="str">
+      <c r="D48" s="70" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E48" s="68" t="str">
+      <c r="E48" s="70" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F48" s="68" t="str">
+      <c r="F48" s="70" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G48" s="68" t="str">
+      <c r="G48" s="70" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H48" s="68" t="str">
+      <c r="H48" s="70" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I48" s="68" t="str">
+      <c r="I48" s="70" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J48" s="68" t="str">
+      <c r="J48" s="70" t="str">
         <v>区间净投入
 / Quote</v>
       </c>
-      <c r="K48" s="68" t="str">
+      <c r="K48" s="70" t="str">
         <v>区间含费
 / Quote</v>
       </c>
-      <c r="L48" s="68" t="str">
+      <c r="L48" s="70" t="str">
         <v>理论累计所需
 / Quote</v>
       </c>
     </row>
-    <row r="49" ht="26" customHeight="1">
+    <row r="49" ht="20" customHeight="1">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
-      <c r="C49" s="69" t="n">
+      <c r="C49" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="72">
+      <c r="D49" s="74">
         <f>$D$35+$G$42-$D$35*C49</f>
       </c>
       <c r="E49" s="26">
         <f>$G$37/D49</f>
       </c>
-      <c r="F49" s="75">
+      <c r="F49" s="77">
         <f>IF(OR(D49="",E49=""),"",E49/D49)</f>
       </c>
-      <c r="G49" s="75">
+      <c r="G49" s="77">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F49))),"",F49*$D$24)</f>
       </c>
       <c r="H49" s="26">
@@ -1690,26 +1740,26 @@
       <c r="K49" s="26">
         <f>J49*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L49" s="81">
+      <c r="L49" s="83">
         <f>(E49-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="50" ht="26" customHeight="1">
+    <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
-      <c r="C50" s="70" t="n">
+      <c r="C50" s="72" t="n">
         <v>0.1</v>
       </c>
-      <c r="D50" s="73">
+      <c r="D50" s="75">
         <f>$D$35+$G$42-$D$35*C50</f>
       </c>
       <c r="E50" s="27">
         <f>$G$37/D50</f>
       </c>
-      <c r="F50" s="76">
+      <c r="F50" s="78">
         <f>IF(OR(D50="",E50=""),"",E50/D50)</f>
       </c>
-      <c r="G50" s="76">
+      <c r="G50" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F50))),"",F50*$D$24)</f>
       </c>
       <c r="H50" s="27">
@@ -1724,26 +1774,26 @@
       <c r="K50" s="27">
         <f>J50*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L50" s="82">
+      <c r="L50" s="84">
         <f>(E50-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="51" ht="26" customHeight="1">
+    <row r="51" ht="20" customHeight="1">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
-      <c r="C51" s="70" t="n">
+      <c r="C51" s="72" t="n">
         <v>0.2</v>
       </c>
-      <c r="D51" s="73">
+      <c r="D51" s="75">
         <f>$D$35+$G$42-$D$35*C51</f>
       </c>
       <c r="E51" s="27">
         <f>$G$37/D51</f>
       </c>
-      <c r="F51" s="76">
+      <c r="F51" s="78">
         <f>IF(OR(D51="",E51=""),"",E51/D51)</f>
       </c>
-      <c r="G51" s="76">
+      <c r="G51" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F51))),"",F51*$D$24)</f>
       </c>
       <c r="H51" s="27">
@@ -1758,26 +1808,26 @@
       <c r="K51" s="27">
         <f>J51*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L51" s="82">
+      <c r="L51" s="84">
         <f>(E51-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="52" ht="26" customHeight="1">
+    <row r="52" ht="20" customHeight="1">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
-      <c r="C52" s="70" t="n">
+      <c r="C52" s="72" t="n">
         <v>0.3</v>
       </c>
-      <c r="D52" s="73">
+      <c r="D52" s="75">
         <f>$D$35+$G$42-$D$35*C52</f>
       </c>
       <c r="E52" s="27">
         <f>$G$37/D52</f>
       </c>
-      <c r="F52" s="76">
+      <c r="F52" s="78">
         <f>IF(OR(D52="",E52=""),"",E52/D52)</f>
       </c>
-      <c r="G52" s="76">
+      <c r="G52" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F52))),"",F52*$D$24)</f>
       </c>
       <c r="H52" s="27">
@@ -1792,26 +1842,26 @@
       <c r="K52" s="27">
         <f>J52*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L52" s="82">
+      <c r="L52" s="84">
         <f>(E52-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="53" ht="26" customHeight="1">
+    <row r="53" ht="20" customHeight="1">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
-      <c r="C53" s="70" t="n">
+      <c r="C53" s="72" t="n">
         <v>0.4</v>
       </c>
-      <c r="D53" s="73">
+      <c r="D53" s="75">
         <f>$D$35+$G$42-$D$35*C53</f>
       </c>
       <c r="E53" s="27">
         <f>$G$37/D53</f>
       </c>
-      <c r="F53" s="76">
+      <c r="F53" s="78">
         <f>IF(OR(D53="",E53=""),"",E53/D53)</f>
       </c>
-      <c r="G53" s="76">
+      <c r="G53" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F53))),"",F53*$D$24)</f>
       </c>
       <c r="H53" s="27">
@@ -1826,26 +1876,26 @@
       <c r="K53" s="27">
         <f>J53*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L53" s="82">
+      <c r="L53" s="84">
         <f>(E53-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="54" ht="26" customHeight="1">
+    <row r="54" ht="20" customHeight="1">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
-      <c r="C54" s="70" t="n">
+      <c r="C54" s="72" t="n">
         <v>0.5</v>
       </c>
-      <c r="D54" s="73">
+      <c r="D54" s="75">
         <f>$D$35+$G$42-$D$35*C54</f>
       </c>
       <c r="E54" s="27">
         <f>$G$37/D54</f>
       </c>
-      <c r="F54" s="76">
+      <c r="F54" s="78">
         <f>IF(OR(D54="",E54=""),"",E54/D54)</f>
       </c>
-      <c r="G54" s="76">
+      <c r="G54" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F54))),"",F54*$D$24)</f>
       </c>
       <c r="H54" s="27">
@@ -1860,26 +1910,26 @@
       <c r="K54" s="27">
         <f>J54*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L54" s="82">
+      <c r="L54" s="84">
         <f>(E54-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="55" ht="26" customHeight="1">
+    <row r="55" ht="20" customHeight="1">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
-      <c r="C55" s="70" t="n">
+      <c r="C55" s="72" t="n">
         <v>0.6</v>
       </c>
-      <c r="D55" s="73">
+      <c r="D55" s="75">
         <f>$D$35+$G$42-$D$35*C55</f>
       </c>
       <c r="E55" s="27">
         <f>$G$37/D55</f>
       </c>
-      <c r="F55" s="76">
+      <c r="F55" s="78">
         <f>IF(OR(D55="",E55=""),"",E55/D55)</f>
       </c>
-      <c r="G55" s="76">
+      <c r="G55" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F55))),"",F55*$D$24)</f>
       </c>
       <c r="H55" s="27">
@@ -1894,26 +1944,26 @@
       <c r="K55" s="27">
         <f>J55*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L55" s="82">
+      <c r="L55" s="84">
         <f>(E55-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="56" ht="26" customHeight="1">
+    <row r="56" ht="20" customHeight="1">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
-      <c r="C56" s="70" t="n">
+      <c r="C56" s="72" t="n">
         <v>0.7</v>
       </c>
-      <c r="D56" s="73">
+      <c r="D56" s="75">
         <f>$D$35+$G$42-$D$35*C56</f>
       </c>
       <c r="E56" s="27">
         <f>$G$37/D56</f>
       </c>
-      <c r="F56" s="76">
+      <c r="F56" s="78">
         <f>IF(OR(D56="",E56=""),"",E56/D56)</f>
       </c>
-      <c r="G56" s="76">
+      <c r="G56" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F56))),"",F56*$D$24)</f>
       </c>
       <c r="H56" s="27">
@@ -1928,45 +1978,45 @@
       <c r="K56" s="27">
         <f>J56*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L56" s="82">
+      <c r="L56" s="84">
         <f>(E56-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="57" ht="26" customHeight="1">
+    <row r="57" ht="20" customHeight="1">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
-      <c r="C57" s="84">
+      <c r="C57" s="86">
         <f>$G$33</f>
       </c>
-      <c r="D57" s="85">
+      <c r="D57" s="87">
         <f>$D$35+$G$42-$D$35*C57</f>
       </c>
-      <c r="E57" s="86">
+      <c r="E57" s="88">
         <f>$G$37/D57</f>
       </c>
-      <c r="F57" s="87">
+      <c r="F57" s="89">
         <f>IF(OR(D57="",E57=""),"",E57/D57)</f>
       </c>
-      <c r="G57" s="87">
+      <c r="G57" s="89">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F57))),"",F57*$D$24)</f>
       </c>
-      <c r="H57" s="86">
+      <c r="H57" s="88">
         <f>IF(NOT(ISNUMBER(F57)),"",F57*$D$35)</f>
       </c>
-      <c r="I57" s="86">
+      <c r="I57" s="88">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H57))),"",H57*$D$24)</f>
       </c>
-      <c r="J57" s="86">
+      <c r="J57" s="88">
         <f>E57-E56</f>
       </c>
-      <c r="K57" s="86">
+      <c r="K57" s="88">
         <f>J57*(1+$G$31+$J$7)</f>
       </c>
-      <c r="L57" s="83">
+      <c r="L57" s="85">
         <f>(E57-$G$36)*(1+$G$31+$J$7)</f>
       </c>
     </row>
-    <row r="58" ht="26" customHeight="1">
+    <row r="58" ht="20" customHeight="1">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -1980,7 +2030,7 @@
       <c r="K58" s="2"/>
       <c r="L58" s="2"/>
     </row>
-    <row r="59" ht="26" customHeight="1">
+    <row r="59" ht="20" customHeight="1">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -1994,7 +2044,7 @@
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>
     </row>
-    <row r="60" ht="27" customHeight="1">
+    <row r="60" ht="24" customHeight="1">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="8" t="str">
@@ -2010,93 +2060,93 @@
       <c r="K60" s="8"/>
       <c r="L60" s="8"/>
     </row>
-    <row r="61" ht="38" customHeight="1">
+    <row r="61" ht="30" customHeight="1">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
-      <c r="C61" s="68" t="str">
+      <c r="C61" s="70" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D61" s="68" t="str">
+      <c r="D61" s="70" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E61" s="68" t="str">
+      <c r="E61" s="70" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F61" s="68" t="str">
+      <c r="F61" s="70" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G61" s="68" t="str">
+      <c r="G61" s="70" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H61" s="68" t="str">
+      <c r="H61" s="70" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I61" s="68" t="str">
+      <c r="I61" s="70" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J61" s="68" t="str">
+      <c r="J61" s="70" t="str">
         <v>外盘净投入
 / Quote</v>
       </c>
-      <c r="K61" s="68" t="str">
+      <c r="K61" s="70" t="str">
         <v>外盘含费
 / Quote</v>
       </c>
-      <c r="L61" s="68" t="str">
+      <c r="L61" s="70" t="str">
         <v>理论累计所需
 / Quote</v>
       </c>
     </row>
-    <row r="62" ht="26" customHeight="1">
+    <row r="62" ht="20" customHeight="1">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
-      <c r="C62" s="88">
+      <c r="C62" s="90">
         <f>$G$33</f>
       </c>
-      <c r="D62" s="89">
+      <c r="D62" s="91">
         <f>$G$38</f>
       </c>
-      <c r="E62" s="90">
+      <c r="E62" s="92">
         <f>$G$34</f>
       </c>
-      <c r="F62" s="91">
+      <c r="F62" s="93">
         <f>IF(OR(D62="",E62=""),"",E62/D62)</f>
       </c>
-      <c r="G62" s="91">
+      <c r="G62" s="93">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F62))),"",F62*$D$24)</f>
       </c>
-      <c r="H62" s="90">
+      <c r="H62" s="92">
         <f>IF(NOT(ISNUMBER(F62)),"",F62*$D$35)</f>
       </c>
-      <c r="I62" s="90">
+      <c r="I62" s="92">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H62))),"",H62*$D$24)</f>
       </c>
-      <c r="J62" s="90">
+      <c r="J62" s="92">
         <f>0</f>
       </c>
-      <c r="K62" s="90">
+      <c r="K62" s="92">
         <f>0</f>
       </c>
-      <c r="L62" s="81">
+      <c r="L62" s="83">
         <f>$J$31</f>
       </c>
     </row>
-    <row r="63" ht="26" customHeight="1">
+    <row r="63" ht="20" customHeight="1">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
-      <c r="C63" s="70" t="n">
+      <c r="C63" s="72" t="n">
         <v>0.805</v>
       </c>
-      <c r="D63" s="73">
+      <c r="D63" s="75">
         <f>IF(C63&lt;$G$23,$G$38-MAX(0,(C63-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E63" s="27">
         <f>IF(D63="","",$G$40/D63)</f>
       </c>
-      <c r="F63" s="76">
+      <c r="F63" s="78">
         <f>IF(OR(D63="",E63=""),"",E63/D63)</f>
       </c>
-      <c r="G63" s="76">
+      <c r="G63" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F63))),"",F63*$D$24)</f>
       </c>
       <c r="H63" s="27">
@@ -2111,26 +2161,26 @@
       <c r="K63" s="27">
         <f>IF(J63="","",J63*(1+$G$32))</f>
       </c>
-      <c r="L63" s="82">
+      <c r="L63" s="84">
         <f>IF(K63="","",$J$31+K63)</f>
       </c>
     </row>
-    <row r="64" ht="26" customHeight="1">
+    <row r="64" ht="20" customHeight="1">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
-      <c r="C64" s="70" t="n">
+      <c r="C64" s="72" t="n">
         <v>0.81</v>
       </c>
-      <c r="D64" s="73">
+      <c r="D64" s="75">
         <f>IF(C64&lt;$G$23,$G$38-MAX(0,(C64-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E64" s="27">
         <f>IF(D64="","",$G$40/D64)</f>
       </c>
-      <c r="F64" s="76">
+      <c r="F64" s="78">
         <f>IF(OR(D64="",E64=""),"",E64/D64)</f>
       </c>
-      <c r="G64" s="76">
+      <c r="G64" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F64))),"",F64*$D$24)</f>
       </c>
       <c r="H64" s="27">
@@ -2145,26 +2195,26 @@
       <c r="K64" s="27">
         <f>IF(J64="","",J64*(1+$G$32))</f>
       </c>
-      <c r="L64" s="82">
+      <c r="L64" s="84">
         <f>IF(K64="","",$J$31+K64)</f>
       </c>
     </row>
-    <row r="65" ht="26" customHeight="1">
+    <row r="65" ht="20" customHeight="1">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
-      <c r="C65" s="70" t="n">
+      <c r="C65" s="72" t="n">
         <v>0.8150000000000001</v>
       </c>
-      <c r="D65" s="73">
+      <c r="D65" s="75">
         <f>IF(C65&lt;$G$23,$G$38-MAX(0,(C65-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E65" s="27">
         <f>IF(D65="","",$G$40/D65)</f>
       </c>
-      <c r="F65" s="76">
+      <c r="F65" s="78">
         <f>IF(OR(D65="",E65=""),"",E65/D65)</f>
       </c>
-      <c r="G65" s="76">
+      <c r="G65" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F65))),"",F65*$D$24)</f>
       </c>
       <c r="H65" s="27">
@@ -2179,26 +2229,26 @@
       <c r="K65" s="27">
         <f>IF(J65="","",J65*(1+$G$32))</f>
       </c>
-      <c r="L65" s="82">
+      <c r="L65" s="84">
         <f>IF(K65="","",$J$31+K65)</f>
       </c>
     </row>
-    <row r="66" ht="26" customHeight="1">
+    <row r="66" ht="20" customHeight="1">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
-      <c r="C66" s="70" t="n">
+      <c r="C66" s="72" t="n">
         <v>0.8200000000000001</v>
       </c>
-      <c r="D66" s="73">
+      <c r="D66" s="75">
         <f>IF(C66&lt;$G$23,$G$38-MAX(0,(C66-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E66" s="27">
         <f>IF(D66="","",$G$40/D66)</f>
       </c>
-      <c r="F66" s="76">
+      <c r="F66" s="78">
         <f>IF(OR(D66="",E66=""),"",E66/D66)</f>
       </c>
-      <c r="G66" s="76">
+      <c r="G66" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F66))),"",F66*$D$24)</f>
       </c>
       <c r="H66" s="27">
@@ -2213,26 +2263,26 @@
       <c r="K66" s="27">
         <f>IF(J66="","",J66*(1+$G$32))</f>
       </c>
-      <c r="L66" s="82">
+      <c r="L66" s="84">
         <f>IF(K66="","",$J$31+K66)</f>
       </c>
     </row>
-    <row r="67" ht="26" customHeight="1">
+    <row r="67" ht="20" customHeight="1">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
-      <c r="C67" s="70" t="n">
+      <c r="C67" s="72" t="n">
         <v>0.8250000000000001</v>
       </c>
-      <c r="D67" s="73">
+      <c r="D67" s="75">
         <f>IF(C67&lt;$G$23,$G$38-MAX(0,(C67-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E67" s="27">
         <f>IF(D67="","",$G$40/D67)</f>
       </c>
-      <c r="F67" s="76">
+      <c r="F67" s="78">
         <f>IF(OR(D67="",E67=""),"",E67/D67)</f>
       </c>
-      <c r="G67" s="76">
+      <c r="G67" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F67))),"",F67*$D$24)</f>
       </c>
       <c r="H67" s="27">
@@ -2247,26 +2297,26 @@
       <c r="K67" s="27">
         <f>IF(J67="","",J67*(1+$G$32))</f>
       </c>
-      <c r="L67" s="82">
+      <c r="L67" s="84">
         <f>IF(K67="","",$J$31+K67)</f>
       </c>
     </row>
-    <row r="68" ht="26" customHeight="1">
+    <row r="68" ht="20" customHeight="1">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
-      <c r="C68" s="70" t="n">
+      <c r="C68" s="72" t="n">
         <v>0.8300000000000001</v>
       </c>
-      <c r="D68" s="73">
+      <c r="D68" s="75">
         <f>IF(C68&lt;$G$23,$G$38-MAX(0,(C68-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E68" s="27">
         <f>IF(D68="","",$G$40/D68)</f>
       </c>
-      <c r="F68" s="76">
+      <c r="F68" s="78">
         <f>IF(OR(D68="",E68=""),"",E68/D68)</f>
       </c>
-      <c r="G68" s="76">
+      <c r="G68" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F68))),"",F68*$D$24)</f>
       </c>
       <c r="H68" s="27">
@@ -2281,26 +2331,26 @@
       <c r="K68" s="27">
         <f>IF(J68="","",J68*(1+$G$32))</f>
       </c>
-      <c r="L68" s="82">
+      <c r="L68" s="84">
         <f>IF(K68="","",$J$31+K68)</f>
       </c>
     </row>
-    <row r="69" ht="26" customHeight="1">
+    <row r="69" ht="20" customHeight="1">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
-      <c r="C69" s="70" t="n">
+      <c r="C69" s="72" t="n">
         <v>0.8350000000000001</v>
       </c>
-      <c r="D69" s="73">
+      <c r="D69" s="75">
         <f>IF(C69&lt;$G$23,$G$38-MAX(0,(C69-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E69" s="27">
         <f>IF(D69="","",$G$40/D69)</f>
       </c>
-      <c r="F69" s="76">
+      <c r="F69" s="78">
         <f>IF(OR(D69="",E69=""),"",E69/D69)</f>
       </c>
-      <c r="G69" s="76">
+      <c r="G69" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F69))),"",F69*$D$24)</f>
       </c>
       <c r="H69" s="27">
@@ -2315,26 +2365,26 @@
       <c r="K69" s="27">
         <f>IF(J69="","",J69*(1+$G$32))</f>
       </c>
-      <c r="L69" s="82">
+      <c r="L69" s="84">
         <f>IF(K69="","",$J$31+K69)</f>
       </c>
     </row>
-    <row r="70" ht="26" customHeight="1">
+    <row r="70" ht="20" customHeight="1">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
-      <c r="C70" s="70" t="n">
+      <c r="C70" s="72" t="n">
         <v>0.8400000000000001</v>
       </c>
-      <c r="D70" s="73">
+      <c r="D70" s="75">
         <f>IF(C70&lt;$G$23,$G$38-MAX(0,(C70-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E70" s="27">
         <f>IF(D70="","",$G$40/D70)</f>
       </c>
-      <c r="F70" s="76">
+      <c r="F70" s="78">
         <f>IF(OR(D70="",E70=""),"",E70/D70)</f>
       </c>
-      <c r="G70" s="76">
+      <c r="G70" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F70))),"",F70*$D$24)</f>
       </c>
       <c r="H70" s="27">
@@ -2349,26 +2399,26 @@
       <c r="K70" s="27">
         <f>IF(J70="","",J70*(1+$G$32))</f>
       </c>
-      <c r="L70" s="82">
+      <c r="L70" s="84">
         <f>IF(K70="","",$J$31+K70)</f>
       </c>
     </row>
-    <row r="71" ht="26" customHeight="1">
+    <row r="71" ht="20" customHeight="1">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
-      <c r="C71" s="70" t="n">
+      <c r="C71" s="72" t="n">
         <v>0.8450000000000001</v>
       </c>
-      <c r="D71" s="73">
+      <c r="D71" s="75">
         <f>IF(C71&lt;$G$23,$G$38-MAX(0,(C71-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E71" s="27">
         <f>IF(D71="","",$G$40/D71)</f>
       </c>
-      <c r="F71" s="76">
+      <c r="F71" s="78">
         <f>IF(OR(D71="",E71=""),"",E71/D71)</f>
       </c>
-      <c r="G71" s="76">
+      <c r="G71" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F71))),"",F71*$D$24)</f>
       </c>
       <c r="H71" s="27">
@@ -2383,26 +2433,26 @@
       <c r="K71" s="27">
         <f>IF(J71="","",J71*(1+$G$32))</f>
       </c>
-      <c r="L71" s="82">
+      <c r="L71" s="84">
         <f>IF(K71="","",$J$31+K71)</f>
       </c>
     </row>
-    <row r="72" ht="26" customHeight="1">
+    <row r="72" ht="20" customHeight="1">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
-      <c r="C72" s="70" t="n">
+      <c r="C72" s="72" t="n">
         <v>0.8500000000000001</v>
       </c>
-      <c r="D72" s="73">
+      <c r="D72" s="75">
         <f>IF(C72&lt;$G$23,$G$38-MAX(0,(C72-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E72" s="27">
         <f>IF(D72="","",$G$40/D72)</f>
       </c>
-      <c r="F72" s="76">
+      <c r="F72" s="78">
         <f>IF(OR(D72="",E72=""),"",E72/D72)</f>
       </c>
-      <c r="G72" s="76">
+      <c r="G72" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F72))),"",F72*$D$24)</f>
       </c>
       <c r="H72" s="27">
@@ -2417,26 +2467,26 @@
       <c r="K72" s="27">
         <f>IF(J72="","",J72*(1+$G$32))</f>
       </c>
-      <c r="L72" s="82">
+      <c r="L72" s="84">
         <f>IF(K72="","",$J$31+K72)</f>
       </c>
     </row>
-    <row r="73" ht="26" customHeight="1">
+    <row r="73" ht="20" customHeight="1">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
-      <c r="C73" s="70" t="n">
+      <c r="C73" s="72" t="n">
         <v>0.8550000000000001</v>
       </c>
-      <c r="D73" s="73">
+      <c r="D73" s="75">
         <f>IF(C73&lt;$G$23,$G$38-MAX(0,(C73-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E73" s="27">
         <f>IF(D73="","",$G$40/D73)</f>
       </c>
-      <c r="F73" s="76">
+      <c r="F73" s="78">
         <f>IF(OR(D73="",E73=""),"",E73/D73)</f>
       </c>
-      <c r="G73" s="76">
+      <c r="G73" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F73))),"",F73*$D$24)</f>
       </c>
       <c r="H73" s="27">
@@ -2451,26 +2501,26 @@
       <c r="K73" s="27">
         <f>IF(J73="","",J73*(1+$G$32))</f>
       </c>
-      <c r="L73" s="82">
+      <c r="L73" s="84">
         <f>IF(K73="","",$J$31+K73)</f>
       </c>
     </row>
-    <row r="74" ht="26" customHeight="1">
+    <row r="74" ht="20" customHeight="1">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
-      <c r="C74" s="70" t="n">
+      <c r="C74" s="72" t="n">
         <v>0.8600000000000001</v>
       </c>
-      <c r="D74" s="73">
+      <c r="D74" s="75">
         <f>IF(C74&lt;$G$23,$G$38-MAX(0,(C74-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E74" s="27">
         <f>IF(D74="","",$G$40/D74)</f>
       </c>
-      <c r="F74" s="76">
+      <c r="F74" s="78">
         <f>IF(OR(D74="",E74=""),"",E74/D74)</f>
       </c>
-      <c r="G74" s="76">
+      <c r="G74" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F74))),"",F74*$D$24)</f>
       </c>
       <c r="H74" s="27">
@@ -2485,26 +2535,26 @@
       <c r="K74" s="27">
         <f>IF(J74="","",J74*(1+$G$32))</f>
       </c>
-      <c r="L74" s="82">
+      <c r="L74" s="84">
         <f>IF(K74="","",$J$31+K74)</f>
       </c>
     </row>
-    <row r="75" ht="26" customHeight="1">
+    <row r="75" ht="20" customHeight="1">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
-      <c r="C75" s="70" t="n">
+      <c r="C75" s="72" t="n">
         <v>0.865</v>
       </c>
-      <c r="D75" s="73">
+      <c r="D75" s="75">
         <f>IF(C75&lt;$G$23,$G$38-MAX(0,(C75-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E75" s="27">
         <f>IF(D75="","",$G$40/D75)</f>
       </c>
-      <c r="F75" s="76">
+      <c r="F75" s="78">
         <f>IF(OR(D75="",E75=""),"",E75/D75)</f>
       </c>
-      <c r="G75" s="76">
+      <c r="G75" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F75))),"",F75*$D$24)</f>
       </c>
       <c r="H75" s="27">
@@ -2519,26 +2569,26 @@
       <c r="K75" s="27">
         <f>IF(J75="","",J75*(1+$G$32))</f>
       </c>
-      <c r="L75" s="82">
+      <c r="L75" s="84">
         <f>IF(K75="","",$J$31+K75)</f>
       </c>
     </row>
-    <row r="76" ht="26" customHeight="1">
+    <row r="76" ht="20" customHeight="1">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
-      <c r="C76" s="70" t="n">
+      <c r="C76" s="72" t="n">
         <v>0.8700000000000001</v>
       </c>
-      <c r="D76" s="73">
+      <c r="D76" s="75">
         <f>IF(C76&lt;$G$23,$G$38-MAX(0,(C76-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E76" s="27">
         <f>IF(D76="","",$G$40/D76)</f>
       </c>
-      <c r="F76" s="76">
+      <c r="F76" s="78">
         <f>IF(OR(D76="",E76=""),"",E76/D76)</f>
       </c>
-      <c r="G76" s="76">
+      <c r="G76" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F76))),"",F76*$D$24)</f>
       </c>
       <c r="H76" s="27">
@@ -2553,26 +2603,26 @@
       <c r="K76" s="27">
         <f>IF(J76="","",J76*(1+$G$32))</f>
       </c>
-      <c r="L76" s="82">
+      <c r="L76" s="84">
         <f>IF(K76="","",$J$31+K76)</f>
       </c>
     </row>
-    <row r="77" ht="26" customHeight="1">
+    <row r="77" ht="20" customHeight="1">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
-      <c r="C77" s="70" t="n">
+      <c r="C77" s="72" t="n">
         <v>0.875</v>
       </c>
-      <c r="D77" s="73">
+      <c r="D77" s="75">
         <f>IF(C77&lt;$G$23,$G$38-MAX(0,(C77-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E77" s="27">
         <f>IF(D77="","",$G$40/D77)</f>
       </c>
-      <c r="F77" s="76">
+      <c r="F77" s="78">
         <f>IF(OR(D77="",E77=""),"",E77/D77)</f>
       </c>
-      <c r="G77" s="76">
+      <c r="G77" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F77))),"",F77*$D$24)</f>
       </c>
       <c r="H77" s="27">
@@ -2587,26 +2637,26 @@
       <c r="K77" s="27">
         <f>IF(J77="","",J77*(1+$G$32))</f>
       </c>
-      <c r="L77" s="82">
+      <c r="L77" s="84">
         <f>IF(K77="","",$J$31+K77)</f>
       </c>
     </row>
-    <row r="78" ht="26" customHeight="1">
+    <row r="78" ht="20" customHeight="1">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
-      <c r="C78" s="70" t="n">
+      <c r="C78" s="72" t="n">
         <v>0.88</v>
       </c>
-      <c r="D78" s="73">
+      <c r="D78" s="75">
         <f>IF(C78&lt;$G$23,$G$38-MAX(0,(C78-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E78" s="27">
         <f>IF(D78="","",$G$40/D78)</f>
       </c>
-      <c r="F78" s="76">
+      <c r="F78" s="78">
         <f>IF(OR(D78="",E78=""),"",E78/D78)</f>
       </c>
-      <c r="G78" s="76">
+      <c r="G78" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F78))),"",F78*$D$24)</f>
       </c>
       <c r="H78" s="27">
@@ -2621,26 +2671,26 @@
       <c r="K78" s="27">
         <f>IF(J78="","",J78*(1+$G$32))</f>
       </c>
-      <c r="L78" s="82">
+      <c r="L78" s="84">
         <f>IF(K78="","",$J$31+K78)</f>
       </c>
     </row>
-    <row r="79" ht="26" customHeight="1">
+    <row r="79" ht="20" customHeight="1">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
-      <c r="C79" s="70" t="n">
+      <c r="C79" s="72" t="n">
         <v>0.885</v>
       </c>
-      <c r="D79" s="73">
+      <c r="D79" s="75">
         <f>IF(C79&lt;$G$23,$G$38-MAX(0,(C79-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E79" s="27">
         <f>IF(D79="","",$G$40/D79)</f>
       </c>
-      <c r="F79" s="76">
+      <c r="F79" s="78">
         <f>IF(OR(D79="",E79=""),"",E79/D79)</f>
       </c>
-      <c r="G79" s="76">
+      <c r="G79" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F79))),"",F79*$D$24)</f>
       </c>
       <c r="H79" s="27">
@@ -2655,26 +2705,26 @@
       <c r="K79" s="27">
         <f>IF(J79="","",J79*(1+$G$32))</f>
       </c>
-      <c r="L79" s="82">
+      <c r="L79" s="84">
         <f>IF(K79="","",$J$31+K79)</f>
       </c>
     </row>
-    <row r="80" ht="26" customHeight="1">
+    <row r="80" ht="20" customHeight="1">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
-      <c r="C80" s="70" t="n">
+      <c r="C80" s="72" t="n">
         <v>0.89</v>
       </c>
-      <c r="D80" s="73">
+      <c r="D80" s="75">
         <f>IF(C80&lt;$G$23,$G$38-MAX(0,(C80-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E80" s="27">
         <f>IF(D80="","",$G$40/D80)</f>
       </c>
-      <c r="F80" s="76">
+      <c r="F80" s="78">
         <f>IF(OR(D80="",E80=""),"",E80/D80)</f>
       </c>
-      <c r="G80" s="76">
+      <c r="G80" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F80))),"",F80*$D$24)</f>
       </c>
       <c r="H80" s="27">
@@ -2689,26 +2739,26 @@
       <c r="K80" s="27">
         <f>IF(J80="","",J80*(1+$G$32))</f>
       </c>
-      <c r="L80" s="82">
+      <c r="L80" s="84">
         <f>IF(K80="","",$J$31+K80)</f>
       </c>
     </row>
-    <row r="81" ht="26" customHeight="1">
+    <row r="81" ht="20" customHeight="1">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
-      <c r="C81" s="70" t="n">
+      <c r="C81" s="72" t="n">
         <v>0.895</v>
       </c>
-      <c r="D81" s="73">
+      <c r="D81" s="75">
         <f>IF(C81&lt;$G$23,$G$38-MAX(0,(C81-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E81" s="27">
         <f>IF(D81="","",$G$40/D81)</f>
       </c>
-      <c r="F81" s="76">
+      <c r="F81" s="78">
         <f>IF(OR(D81="",E81=""),"",E81/D81)</f>
       </c>
-      <c r="G81" s="76">
+      <c r="G81" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F81))),"",F81*$D$24)</f>
       </c>
       <c r="H81" s="27">
@@ -2723,26 +2773,26 @@
       <c r="K81" s="27">
         <f>IF(J81="","",J81*(1+$G$32))</f>
       </c>
-      <c r="L81" s="82">
+      <c r="L81" s="84">
         <f>IF(K81="","",$J$31+K81)</f>
       </c>
     </row>
-    <row r="82" ht="26" customHeight="1">
+    <row r="82" ht="20" customHeight="1">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
-      <c r="C82" s="70" t="n">
+      <c r="C82" s="72" t="n">
         <v>0.9</v>
       </c>
-      <c r="D82" s="73">
+      <c r="D82" s="75">
         <f>IF(C82&lt;$G$23,$G$38-MAX(0,(C82-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E82" s="27">
         <f>IF(D82="","",$G$40/D82)</f>
       </c>
-      <c r="F82" s="76">
+      <c r="F82" s="78">
         <f>IF(OR(D82="",E82=""),"",E82/D82)</f>
       </c>
-      <c r="G82" s="76">
+      <c r="G82" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F82))),"",F82*$D$24)</f>
       </c>
       <c r="H82" s="27">
@@ -2757,26 +2807,26 @@
       <c r="K82" s="27">
         <f>IF(J82="","",J82*(1+$G$32))</f>
       </c>
-      <c r="L82" s="82">
+      <c r="L82" s="84">
         <f>IF(K82="","",$J$31+K82)</f>
       </c>
     </row>
-    <row r="83" ht="26" customHeight="1">
+    <row r="83" ht="20" customHeight="1">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
-      <c r="C83" s="70" t="n">
+      <c r="C83" s="72" t="n">
         <v>0.905</v>
       </c>
-      <c r="D83" s="73">
+      <c r="D83" s="75">
         <f>IF(C83&lt;$G$23,$G$38-MAX(0,(C83-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E83" s="27">
         <f>IF(D83="","",$G$40/D83)</f>
       </c>
-      <c r="F83" s="76">
+      <c r="F83" s="78">
         <f>IF(OR(D83="",E83=""),"",E83/D83)</f>
       </c>
-      <c r="G83" s="76">
+      <c r="G83" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F83))),"",F83*$D$24)</f>
       </c>
       <c r="H83" s="27">
@@ -2791,26 +2841,26 @@
       <c r="K83" s="27">
         <f>IF(J83="","",J83*(1+$G$32))</f>
       </c>
-      <c r="L83" s="82">
+      <c r="L83" s="84">
         <f>IF(K83="","",$J$31+K83)</f>
       </c>
     </row>
-    <row r="84" ht="26" customHeight="1">
+    <row r="84" ht="20" customHeight="1">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
-      <c r="C84" s="70" t="n">
+      <c r="C84" s="72" t="n">
         <v>0.91</v>
       </c>
-      <c r="D84" s="73">
+      <c r="D84" s="75">
         <f>IF(C84&lt;$G$23,$G$38-MAX(0,(C84-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E84" s="27">
         <f>IF(D84="","",$G$40/D84)</f>
       </c>
-      <c r="F84" s="76">
+      <c r="F84" s="78">
         <f>IF(OR(D84="",E84=""),"",E84/D84)</f>
       </c>
-      <c r="G84" s="76">
+      <c r="G84" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F84))),"",F84*$D$24)</f>
       </c>
       <c r="H84" s="27">
@@ -2825,26 +2875,26 @@
       <c r="K84" s="27">
         <f>IF(J84="","",J84*(1+$G$32))</f>
       </c>
-      <c r="L84" s="82">
+      <c r="L84" s="84">
         <f>IF(K84="","",$J$31+K84)</f>
       </c>
     </row>
-    <row r="85" ht="26" customHeight="1">
+    <row r="85" ht="20" customHeight="1">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
-      <c r="C85" s="70" t="n">
+      <c r="C85" s="72" t="n">
         <v>0.915</v>
       </c>
-      <c r="D85" s="73">
+      <c r="D85" s="75">
         <f>IF(C85&lt;$G$23,$G$38-MAX(0,(C85-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E85" s="27">
         <f>IF(D85="","",$G$40/D85)</f>
       </c>
-      <c r="F85" s="76">
+      <c r="F85" s="78">
         <f>IF(OR(D85="",E85=""),"",E85/D85)</f>
       </c>
-      <c r="G85" s="76">
+      <c r="G85" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F85))),"",F85*$D$24)</f>
       </c>
       <c r="H85" s="27">
@@ -2859,26 +2909,26 @@
       <c r="K85" s="27">
         <f>IF(J85="","",J85*(1+$G$32))</f>
       </c>
-      <c r="L85" s="82">
+      <c r="L85" s="84">
         <f>IF(K85="","",$J$31+K85)</f>
       </c>
     </row>
-    <row r="86" ht="26" customHeight="1">
+    <row r="86" ht="20" customHeight="1">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
-      <c r="C86" s="70" t="n">
+      <c r="C86" s="72" t="n">
         <v>0.92</v>
       </c>
-      <c r="D86" s="73">
+      <c r="D86" s="75">
         <f>IF(C86&lt;$G$23,$G$38-MAX(0,(C86-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E86" s="27">
         <f>IF(D86="","",$G$40/D86)</f>
       </c>
-      <c r="F86" s="76">
+      <c r="F86" s="78">
         <f>IF(OR(D86="",E86=""),"",E86/D86)</f>
       </c>
-      <c r="G86" s="76">
+      <c r="G86" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F86))),"",F86*$D$24)</f>
       </c>
       <c r="H86" s="27">
@@ -2893,26 +2943,26 @@
       <c r="K86" s="27">
         <f>IF(J86="","",J86*(1+$G$32))</f>
       </c>
-      <c r="L86" s="82">
+      <c r="L86" s="84">
         <f>IF(K86="","",$J$31+K86)</f>
       </c>
     </row>
-    <row r="87" ht="26" customHeight="1">
+    <row r="87" ht="20" customHeight="1">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
-      <c r="C87" s="70" t="n">
+      <c r="C87" s="72" t="n">
         <v>0.925</v>
       </c>
-      <c r="D87" s="73">
+      <c r="D87" s="75">
         <f>IF(C87&lt;$G$23,$G$38-MAX(0,(C87-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E87" s="27">
         <f>IF(D87="","",$G$40/D87)</f>
       </c>
-      <c r="F87" s="76">
+      <c r="F87" s="78">
         <f>IF(OR(D87="",E87=""),"",E87/D87)</f>
       </c>
-      <c r="G87" s="76">
+      <c r="G87" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F87))),"",F87*$D$24)</f>
       </c>
       <c r="H87" s="27">
@@ -2927,26 +2977,26 @@
       <c r="K87" s="27">
         <f>IF(J87="","",J87*(1+$G$32))</f>
       </c>
-      <c r="L87" s="82">
+      <c r="L87" s="84">
         <f>IF(K87="","",$J$31+K87)</f>
       </c>
     </row>
-    <row r="88" ht="26" customHeight="1">
+    <row r="88" ht="20" customHeight="1">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
-      <c r="C88" s="70" t="n">
+      <c r="C88" s="72" t="n">
         <v>0.93</v>
       </c>
-      <c r="D88" s="73">
+      <c r="D88" s="75">
         <f>IF(C88&lt;$G$23,$G$38-MAX(0,(C88-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E88" s="27">
         <f>IF(D88="","",$G$40/D88)</f>
       </c>
-      <c r="F88" s="76">
+      <c r="F88" s="78">
         <f>IF(OR(D88="",E88=""),"",E88/D88)</f>
       </c>
-      <c r="G88" s="76">
+      <c r="G88" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F88))),"",F88*$D$24)</f>
       </c>
       <c r="H88" s="27">
@@ -2961,26 +3011,26 @@
       <c r="K88" s="27">
         <f>IF(J88="","",J88*(1+$G$32))</f>
       </c>
-      <c r="L88" s="82">
+      <c r="L88" s="84">
         <f>IF(K88="","",$J$31+K88)</f>
       </c>
     </row>
-    <row r="89" ht="26" customHeight="1">
+    <row r="89" ht="20" customHeight="1">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
-      <c r="C89" s="70" t="n">
+      <c r="C89" s="72" t="n">
         <v>0.935</v>
       </c>
-      <c r="D89" s="73">
+      <c r="D89" s="75">
         <f>IF(C89&lt;$G$23,$G$38-MAX(0,(C89-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E89" s="27">
         <f>IF(D89="","",$G$40/D89)</f>
       </c>
-      <c r="F89" s="76">
+      <c r="F89" s="78">
         <f>IF(OR(D89="",E89=""),"",E89/D89)</f>
       </c>
-      <c r="G89" s="76">
+      <c r="G89" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F89))),"",F89*$D$24)</f>
       </c>
       <c r="H89" s="27">
@@ -2995,26 +3045,26 @@
       <c r="K89" s="27">
         <f>IF(J89="","",J89*(1+$G$32))</f>
       </c>
-      <c r="L89" s="82">
+      <c r="L89" s="84">
         <f>IF(K89="","",$J$31+K89)</f>
       </c>
     </row>
-    <row r="90" ht="26" customHeight="1">
+    <row r="90" ht="20" customHeight="1">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
-      <c r="C90" s="70" t="n">
+      <c r="C90" s="72" t="n">
         <v>0.9400000000000001</v>
       </c>
-      <c r="D90" s="73">
+      <c r="D90" s="75">
         <f>IF(C90&lt;$G$23,$G$38-MAX(0,(C90-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E90" s="27">
         <f>IF(D90="","",$G$40/D90)</f>
       </c>
-      <c r="F90" s="76">
+      <c r="F90" s="78">
         <f>IF(OR(D90="",E90=""),"",E90/D90)</f>
       </c>
-      <c r="G90" s="76">
+      <c r="G90" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F90))),"",F90*$D$24)</f>
       </c>
       <c r="H90" s="27">
@@ -3029,26 +3079,26 @@
       <c r="K90" s="27">
         <f>IF(J90="","",J90*(1+$G$32))</f>
       </c>
-      <c r="L90" s="82">
+      <c r="L90" s="84">
         <f>IF(K90="","",$J$31+K90)</f>
       </c>
     </row>
-    <row r="91" ht="26" customHeight="1">
+    <row r="91" ht="20" customHeight="1">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
-      <c r="C91" s="70" t="n">
+      <c r="C91" s="72" t="n">
         <v>0.9450000000000001</v>
       </c>
-      <c r="D91" s="73">
+      <c r="D91" s="75">
         <f>IF(C91&lt;$G$23,$G$38-MAX(0,(C91-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E91" s="27">
         <f>IF(D91="","",$G$40/D91)</f>
       </c>
-      <c r="F91" s="76">
+      <c r="F91" s="78">
         <f>IF(OR(D91="",E91=""),"",E91/D91)</f>
       </c>
-      <c r="G91" s="76">
+      <c r="G91" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F91))),"",F91*$D$24)</f>
       </c>
       <c r="H91" s="27">
@@ -3063,26 +3113,26 @@
       <c r="K91" s="27">
         <f>IF(J91="","",J91*(1+$G$32))</f>
       </c>
-      <c r="L91" s="82">
+      <c r="L91" s="84">
         <f>IF(K91="","",$J$31+K91)</f>
       </c>
     </row>
-    <row r="92" ht="26" customHeight="1">
+    <row r="92" ht="20" customHeight="1">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
-      <c r="C92" s="70" t="n">
+      <c r="C92" s="72" t="n">
         <v>0.9500000000000001</v>
       </c>
-      <c r="D92" s="73">
+      <c r="D92" s="75">
         <f>IF(C92&lt;$G$23,$G$38-MAX(0,(C92-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E92" s="27">
         <f>IF(D92="","",$G$40/D92)</f>
       </c>
-      <c r="F92" s="76">
+      <c r="F92" s="78">
         <f>IF(OR(D92="",E92=""),"",E92/D92)</f>
       </c>
-      <c r="G92" s="76">
+      <c r="G92" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F92))),"",F92*$D$24)</f>
       </c>
       <c r="H92" s="27">
@@ -3097,26 +3147,26 @@
       <c r="K92" s="27">
         <f>IF(J92="","",J92*(1+$G$32))</f>
       </c>
-      <c r="L92" s="82">
+      <c r="L92" s="84">
         <f>IF(K92="","",$J$31+K92)</f>
       </c>
     </row>
-    <row r="93" ht="26" customHeight="1">
+    <row r="93" ht="20" customHeight="1">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
-      <c r="C93" s="70" t="n">
+      <c r="C93" s="72" t="n">
         <v>0.9550000000000001</v>
       </c>
-      <c r="D93" s="73">
+      <c r="D93" s="75">
         <f>IF(C93&lt;$G$23,$G$38-MAX(0,(C93-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E93" s="27">
         <f>IF(D93="","",$G$40/D93)</f>
       </c>
-      <c r="F93" s="76">
+      <c r="F93" s="78">
         <f>IF(OR(D93="",E93=""),"",E93/D93)</f>
       </c>
-      <c r="G93" s="76">
+      <c r="G93" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F93))),"",F93*$D$24)</f>
       </c>
       <c r="H93" s="27">
@@ -3131,26 +3181,26 @@
       <c r="K93" s="27">
         <f>IF(J93="","",J93*(1+$G$32))</f>
       </c>
-      <c r="L93" s="82">
+      <c r="L93" s="84">
         <f>IF(K93="","",$J$31+K93)</f>
       </c>
     </row>
-    <row r="94" ht="26" customHeight="1">
+    <row r="94" ht="20" customHeight="1">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
-      <c r="C94" s="70" t="n">
+      <c r="C94" s="72" t="n">
         <v>0.9600000000000001</v>
       </c>
-      <c r="D94" s="73">
+      <c r="D94" s="75">
         <f>IF(C94&lt;$G$23,$G$38-MAX(0,(C94-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E94" s="27">
         <f>IF(D94="","",$G$40/D94)</f>
       </c>
-      <c r="F94" s="76">
+      <c r="F94" s="78">
         <f>IF(OR(D94="",E94=""),"",E94/D94)</f>
       </c>
-      <c r="G94" s="76">
+      <c r="G94" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F94))),"",F94*$D$24)</f>
       </c>
       <c r="H94" s="27">
@@ -3165,26 +3215,26 @@
       <c r="K94" s="27">
         <f>IF(J94="","",J94*(1+$G$32))</f>
       </c>
-      <c r="L94" s="82">
+      <c r="L94" s="84">
         <f>IF(K94="","",$J$31+K94)</f>
       </c>
     </row>
-    <row r="95" ht="26" customHeight="1">
+    <row r="95" ht="20" customHeight="1">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
-      <c r="C95" s="70" t="n">
+      <c r="C95" s="72" t="n">
         <v>0.9650000000000001</v>
       </c>
-      <c r="D95" s="73">
+      <c r="D95" s="75">
         <f>IF(C95&lt;$G$23,$G$38-MAX(0,(C95-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E95" s="27">
         <f>IF(D95="","",$G$40/D95)</f>
       </c>
-      <c r="F95" s="76">
+      <c r="F95" s="78">
         <f>IF(OR(D95="",E95=""),"",E95/D95)</f>
       </c>
-      <c r="G95" s="76">
+      <c r="G95" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F95))),"",F95*$D$24)</f>
       </c>
       <c r="H95" s="27">
@@ -3199,26 +3249,26 @@
       <c r="K95" s="27">
         <f>IF(J95="","",J95*(1+$G$32))</f>
       </c>
-      <c r="L95" s="82">
+      <c r="L95" s="84">
         <f>IF(K95="","",$J$31+K95)</f>
       </c>
     </row>
-    <row r="96" ht="26" customHeight="1">
+    <row r="96" ht="20" customHeight="1">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
-      <c r="C96" s="70" t="n">
+      <c r="C96" s="72" t="n">
         <v>0.9700000000000001</v>
       </c>
-      <c r="D96" s="73">
+      <c r="D96" s="75">
         <f>IF(C96&lt;$G$23,$G$38-MAX(0,(C96-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E96" s="27">
         <f>IF(D96="","",$G$40/D96)</f>
       </c>
-      <c r="F96" s="76">
+      <c r="F96" s="78">
         <f>IF(OR(D96="",E96=""),"",E96/D96)</f>
       </c>
-      <c r="G96" s="76">
+      <c r="G96" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F96))),"",F96*$D$24)</f>
       </c>
       <c r="H96" s="27">
@@ -3233,26 +3283,26 @@
       <c r="K96" s="27">
         <f>IF(J96="","",J96*(1+$G$32))</f>
       </c>
-      <c r="L96" s="82">
+      <c r="L96" s="84">
         <f>IF(K96="","",$J$31+K96)</f>
       </c>
     </row>
-    <row r="97" ht="26" customHeight="1">
+    <row r="97" ht="20" customHeight="1">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
-      <c r="C97" s="70" t="n">
+      <c r="C97" s="72" t="n">
         <v>0.9750000000000001</v>
       </c>
-      <c r="D97" s="73">
+      <c r="D97" s="75">
         <f>IF(C97&lt;$G$23,$G$38-MAX(0,(C97-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E97" s="27">
         <f>IF(D97="","",$G$40/D97)</f>
       </c>
-      <c r="F97" s="76">
+      <c r="F97" s="78">
         <f>IF(OR(D97="",E97=""),"",E97/D97)</f>
       </c>
-      <c r="G97" s="76">
+      <c r="G97" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F97))),"",F97*$D$24)</f>
       </c>
       <c r="H97" s="27">
@@ -3267,26 +3317,26 @@
       <c r="K97" s="27">
         <f>IF(J97="","",J97*(1+$G$32))</f>
       </c>
-      <c r="L97" s="82">
+      <c r="L97" s="84">
         <f>IF(K97="","",$J$31+K97)</f>
       </c>
     </row>
-    <row r="98" ht="26" customHeight="1">
+    <row r="98" ht="20" customHeight="1">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
-      <c r="C98" s="70" t="n">
+      <c r="C98" s="72" t="n">
         <v>0.98</v>
       </c>
-      <c r="D98" s="73">
+      <c r="D98" s="75">
         <f>IF(C98&lt;$G$23,$G$38-MAX(0,(C98-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E98" s="27">
         <f>IF(D98="","",$G$40/D98)</f>
       </c>
-      <c r="F98" s="76">
+      <c r="F98" s="78">
         <f>IF(OR(D98="",E98=""),"",E98/D98)</f>
       </c>
-      <c r="G98" s="76">
+      <c r="G98" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F98))),"",F98*$D$24)</f>
       </c>
       <c r="H98" s="27">
@@ -3301,26 +3351,26 @@
       <c r="K98" s="27">
         <f>IF(J98="","",J98*(1+$G$32))</f>
       </c>
-      <c r="L98" s="82">
+      <c r="L98" s="84">
         <f>IF(K98="","",$J$31+K98)</f>
       </c>
     </row>
-    <row r="99" ht="26" customHeight="1">
+    <row r="99" ht="20" customHeight="1">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
-      <c r="C99" s="70" t="n">
+      <c r="C99" s="72" t="n">
         <v>0.9850000000000001</v>
       </c>
-      <c r="D99" s="73">
+      <c r="D99" s="75">
         <f>IF(C99&lt;$G$23,$G$38-MAX(0,(C99-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E99" s="27">
         <f>IF(D99="","",$G$40/D99)</f>
       </c>
-      <c r="F99" s="76">
+      <c r="F99" s="78">
         <f>IF(OR(D99="",E99=""),"",E99/D99)</f>
       </c>
-      <c r="G99" s="76">
+      <c r="G99" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F99))),"",F99*$D$24)</f>
       </c>
       <c r="H99" s="27">
@@ -3335,26 +3385,26 @@
       <c r="K99" s="27">
         <f>IF(J99="","",J99*(1+$G$32))</f>
       </c>
-      <c r="L99" s="82">
+      <c r="L99" s="84">
         <f>IF(K99="","",$J$31+K99)</f>
       </c>
     </row>
-    <row r="100" ht="26" customHeight="1">
+    <row r="100" ht="20" customHeight="1">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
-      <c r="C100" s="70" t="n">
+      <c r="C100" s="72" t="n">
         <v>0.99</v>
       </c>
-      <c r="D100" s="73">
+      <c r="D100" s="75">
         <f>IF(C100&lt;$G$23,$G$38-MAX(0,(C100-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E100" s="27">
         <f>IF(D100="","",$G$40/D100)</f>
       </c>
-      <c r="F100" s="76">
+      <c r="F100" s="78">
         <f>IF(OR(D100="",E100=""),"",E100/D100)</f>
       </c>
-      <c r="G100" s="76">
+      <c r="G100" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F100))),"",F100*$D$24)</f>
       </c>
       <c r="H100" s="27">
@@ -3369,26 +3419,26 @@
       <c r="K100" s="27">
         <f>IF(J100="","",J100*(1+$G$32))</f>
       </c>
-      <c r="L100" s="82">
+      <c r="L100" s="84">
         <f>IF(K100="","",$J$31+K100)</f>
       </c>
     </row>
-    <row r="101" ht="26" customHeight="1">
+    <row r="101" ht="20" customHeight="1">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
-      <c r="C101" s="70" t="n">
+      <c r="C101" s="72" t="n">
         <v>0.9950000000000001</v>
       </c>
-      <c r="D101" s="73">
+      <c r="D101" s="75">
         <f>IF(C101&lt;$G$23,$G$38-MAX(0,(C101-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E101" s="27">
         <f>IF(D101="","",$G$40/D101)</f>
       </c>
-      <c r="F101" s="76">
+      <c r="F101" s="78">
         <f>IF(OR(D101="",E101=""),"",E101/D101)</f>
       </c>
-      <c r="G101" s="76">
+      <c r="G101" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F101))),"",F101*$D$24)</f>
       </c>
       <c r="H101" s="27">
@@ -3403,26 +3453,26 @@
       <c r="K101" s="27">
         <f>IF(J101="","",J101*(1+$G$32))</f>
       </c>
-      <c r="L101" s="82">
+      <c r="L101" s="84">
         <f>IF(K101="","",$J$31+K101)</f>
       </c>
     </row>
-    <row r="102" ht="26" customHeight="1">
+    <row r="102" ht="20" customHeight="1">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
-      <c r="C102" s="71" t="n">
+      <c r="C102" s="73" t="n">
         <v>1</v>
       </c>
-      <c r="D102" s="74">
+      <c r="D102" s="76">
         <f>IF(C102&lt;$G$23,$G$38-MAX(0,(C102-$G$33)*$D$35)/(1-$J$7),"")</f>
       </c>
       <c r="E102" s="28">
         <f>IF(D102="","",$G$40/D102)</f>
       </c>
-      <c r="F102" s="77">
+      <c r="F102" s="79">
         <f>IF(OR(D102="",E102=""),"",E102/D102)</f>
       </c>
-      <c r="G102" s="77">
+      <c r="G102" s="79">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F102))),"",F102*$D$24)</f>
       </c>
       <c r="H102" s="28">
@@ -3437,11 +3487,11 @@
       <c r="K102" s="28">
         <f>IF(J102="","",J102*(1+$G$32))</f>
       </c>
-      <c r="L102" s="83">
+      <c r="L102" s="85">
         <f>IF(K102="","",$J$31+K102)</f>
       </c>
     </row>
-    <row r="103" ht="26" customHeight="1">
+    <row r="103" ht="20" customHeight="1">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -3455,7 +3505,7 @@
       <c r="K103" s="2"/>
       <c r="L103" s="2"/>
     </row>
-    <row r="104" ht="26" customHeight="1">
+    <row r="104" ht="20" customHeight="1">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -3469,98 +3519,98 @@
       <c r="K104" s="2"/>
       <c r="L104" s="2"/>
     </row>
-    <row r="105" ht="27" customHeight="1">
+    <row r="105" ht="24" customHeight="1">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
-      <c r="C105" s="93" t="str">
+      <c r="C105" s="95" t="str">
         <v>外盘回落参考</v>
       </c>
-      <c r="D105" s="93"/>
-      <c r="E105" s="93"/>
-      <c r="F105" s="93"/>
-      <c r="G105" s="93"/>
-      <c r="H105" s="93"/>
-      <c r="I105" s="93"/>
-      <c r="J105" s="93"/>
-      <c r="K105" s="93"/>
-      <c r="L105" s="93"/>
-    </row>
-    <row r="106" ht="38" customHeight="1">
+      <c r="D105" s="95"/>
+      <c r="E105" s="95"/>
+      <c r="F105" s="95"/>
+      <c r="G105" s="95"/>
+      <c r="H105" s="95"/>
+      <c r="I105" s="95"/>
+      <c r="J105" s="95"/>
+      <c r="K105" s="95"/>
+      <c r="L105" s="95"/>
+    </row>
+    <row r="106" ht="30" customHeight="1">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
-      <c r="C106" s="68" t="str">
+      <c r="C106" s="70" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D106" s="68" t="str">
+      <c r="D106" s="70" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E106" s="68" t="str">
+      <c r="E106" s="70" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F106" s="68" t="str">
+      <c r="F106" s="70" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G106" s="68" t="str">
+      <c r="G106" s="70" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H106" s="68" t="str">
+      <c r="H106" s="70" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I106" s="68" t="str">
+      <c r="I106" s="70" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J106" s="68" t="str">
+      <c r="J106" s="70" t="str">
         <v>较毕业点回撤</v>
       </c>
-      <c r="K106" s="68" t="str"/>
-      <c r="L106" s="68" t="str"/>
-    </row>
-    <row r="107" ht="26" customHeight="1">
+      <c r="K106" s="70" t="str"/>
+      <c r="L106" s="70" t="str"/>
+    </row>
+    <row r="107" ht="20" customHeight="1">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
-      <c r="C107" s="88" t="n">
+      <c r="C107" s="90" t="n">
         <v>0.8</v>
       </c>
-      <c r="D107" s="89">
+      <c r="D107" s="91">
         <f>$D$35*(1-C107)</f>
       </c>
-      <c r="E107" s="90">
+      <c r="E107" s="92">
         <f>$G$40/D107</f>
       </c>
-      <c r="F107" s="91">
+      <c r="F107" s="93">
         <f>IF(OR(D107="",E107=""),"",E107/D107)</f>
       </c>
-      <c r="G107" s="91">
+      <c r="G107" s="93">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F107))),"",F107*$D$24)</f>
       </c>
-      <c r="H107" s="90">
+      <c r="H107" s="92">
         <f>IF(NOT(ISNUMBER(F107)),"",F107*$D$35)</f>
       </c>
-      <c r="I107" s="90">
+      <c r="I107" s="92">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H107))),"",H107*$D$24)</f>
       </c>
-      <c r="J107" s="88">
+      <c r="J107" s="90">
         <f>IF($H$107&gt;0,1-H107/$H$107,0)</f>
       </c>
-      <c r="K107" s="90"/>
-      <c r="L107" s="90"/>
-    </row>
-    <row r="108" ht="26" customHeight="1">
+      <c r="K107" s="92"/>
+      <c r="L107" s="92"/>
+    </row>
+    <row r="108" ht="20" customHeight="1">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
-      <c r="C108" s="70" t="n">
+      <c r="C108" s="72" t="n">
         <v>0.7</v>
       </c>
-      <c r="D108" s="73">
+      <c r="D108" s="75">
         <f>$D$35*(1-C108)</f>
       </c>
       <c r="E108" s="27">
         <f>$G$40/D108</f>
       </c>
-      <c r="F108" s="76">
+      <c r="F108" s="78">
         <f>IF(OR(D108="",E108=""),"",E108/D108)</f>
       </c>
-      <c r="G108" s="76">
+      <c r="G108" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F108))),"",F108*$D$24)</f>
       </c>
       <c r="H108" s="27">
@@ -3569,28 +3619,28 @@
       <c r="I108" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H108))),"",H108*$D$24)</f>
       </c>
-      <c r="J108" s="70">
+      <c r="J108" s="72">
         <f>IF($H$107&gt;0,1-H108/$H$107,0)</f>
       </c>
       <c r="K108" s="27"/>
       <c r="L108" s="27"/>
     </row>
-    <row r="109" ht="26" customHeight="1">
+    <row r="109" ht="20" customHeight="1">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
-      <c r="C109" s="70" t="n">
+      <c r="C109" s="72" t="n">
         <v>0.6</v>
       </c>
-      <c r="D109" s="73">
+      <c r="D109" s="75">
         <f>$D$35*(1-C109)</f>
       </c>
       <c r="E109" s="27">
         <f>$G$40/D109</f>
       </c>
-      <c r="F109" s="76">
+      <c r="F109" s="78">
         <f>IF(OR(D109="",E109=""),"",E109/D109)</f>
       </c>
-      <c r="G109" s="76">
+      <c r="G109" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F109))),"",F109*$D$24)</f>
       </c>
       <c r="H109" s="27">
@@ -3599,28 +3649,28 @@
       <c r="I109" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H109))),"",H109*$D$24)</f>
       </c>
-      <c r="J109" s="70">
+      <c r="J109" s="72">
         <f>IF($H$107&gt;0,1-H109/$H$107,0)</f>
       </c>
       <c r="K109" s="27"/>
       <c r="L109" s="27"/>
     </row>
-    <row r="110" ht="26" customHeight="1">
+    <row r="110" ht="20" customHeight="1">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
-      <c r="C110" s="70" t="n">
+      <c r="C110" s="72" t="n">
         <v>0.5</v>
       </c>
-      <c r="D110" s="73">
+      <c r="D110" s="75">
         <f>$D$35*(1-C110)</f>
       </c>
       <c r="E110" s="27">
         <f>$G$40/D110</f>
       </c>
-      <c r="F110" s="76">
+      <c r="F110" s="78">
         <f>IF(OR(D110="",E110=""),"",E110/D110)</f>
       </c>
-      <c r="G110" s="76">
+      <c r="G110" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F110))),"",F110*$D$24)</f>
       </c>
       <c r="H110" s="27">
@@ -3629,28 +3679,28 @@
       <c r="I110" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H110))),"",H110*$D$24)</f>
       </c>
-      <c r="J110" s="70">
+      <c r="J110" s="72">
         <f>IF($H$107&gt;0,1-H110/$H$107,0)</f>
       </c>
       <c r="K110" s="27"/>
       <c r="L110" s="27"/>
     </row>
-    <row r="111" ht="26" customHeight="1">
+    <row r="111" ht="20" customHeight="1">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
-      <c r="C111" s="70" t="n">
+      <c r="C111" s="72" t="n">
         <v>0.4</v>
       </c>
-      <c r="D111" s="73">
+      <c r="D111" s="75">
         <f>$D$35*(1-C111)</f>
       </c>
       <c r="E111" s="27">
         <f>$G$40/D111</f>
       </c>
-      <c r="F111" s="76">
+      <c r="F111" s="78">
         <f>IF(OR(D111="",E111=""),"",E111/D111)</f>
       </c>
-      <c r="G111" s="76">
+      <c r="G111" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F111))),"",F111*$D$24)</f>
       </c>
       <c r="H111" s="27">
@@ -3659,28 +3709,28 @@
       <c r="I111" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H111))),"",H111*$D$24)</f>
       </c>
-      <c r="J111" s="70">
+      <c r="J111" s="72">
         <f>IF($H$107&gt;0,1-H111/$H$107,0)</f>
       </c>
       <c r="K111" s="27"/>
       <c r="L111" s="27"/>
     </row>
-    <row r="112" ht="26" customHeight="1">
+    <row r="112" ht="20" customHeight="1">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
-      <c r="C112" s="70" t="n">
+      <c r="C112" s="72" t="n">
         <v>0.3</v>
       </c>
-      <c r="D112" s="73">
+      <c r="D112" s="75">
         <f>$D$35*(1-C112)</f>
       </c>
       <c r="E112" s="27">
         <f>$G$40/D112</f>
       </c>
-      <c r="F112" s="76">
+      <c r="F112" s="78">
         <f>IF(OR(D112="",E112=""),"",E112/D112)</f>
       </c>
-      <c r="G112" s="76">
+      <c r="G112" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F112))),"",F112*$D$24)</f>
       </c>
       <c r="H112" s="27">
@@ -3689,28 +3739,28 @@
       <c r="I112" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H112))),"",H112*$D$24)</f>
       </c>
-      <c r="J112" s="70">
+      <c r="J112" s="72">
         <f>IF($H$107&gt;0,1-H112/$H$107,0)</f>
       </c>
       <c r="K112" s="27"/>
       <c r="L112" s="27"/>
     </row>
-    <row r="113" ht="26" customHeight="1">
+    <row r="113" ht="20" customHeight="1">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
-      <c r="C113" s="70" t="n">
+      <c r="C113" s="72" t="n">
         <v>0.2</v>
       </c>
-      <c r="D113" s="73">
+      <c r="D113" s="75">
         <f>$D$35*(1-C113)</f>
       </c>
       <c r="E113" s="27">
         <f>$G$40/D113</f>
       </c>
-      <c r="F113" s="76">
+      <c r="F113" s="78">
         <f>IF(OR(D113="",E113=""),"",E113/D113)</f>
       </c>
-      <c r="G113" s="76">
+      <c r="G113" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F113))),"",F113*$D$24)</f>
       </c>
       <c r="H113" s="27">
@@ -3719,28 +3769,28 @@
       <c r="I113" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H113))),"",H113*$D$24)</f>
       </c>
-      <c r="J113" s="70">
+      <c r="J113" s="72">
         <f>IF($H$107&gt;0,1-H113/$H$107,0)</f>
       </c>
       <c r="K113" s="27"/>
       <c r="L113" s="27"/>
     </row>
-    <row r="114" ht="26" customHeight="1">
+    <row r="114" ht="20" customHeight="1">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
-      <c r="C114" s="70" t="n">
+      <c r="C114" s="72" t="n">
         <v>0.1</v>
       </c>
-      <c r="D114" s="73">
+      <c r="D114" s="75">
         <f>$D$35*(1-C114)</f>
       </c>
       <c r="E114" s="27">
         <f>$G$40/D114</f>
       </c>
-      <c r="F114" s="76">
+      <c r="F114" s="78">
         <f>IF(OR(D114="",E114=""),"",E114/D114)</f>
       </c>
-      <c r="G114" s="76">
+      <c r="G114" s="78">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F114))),"",F114*$D$24)</f>
       </c>
       <c r="H114" s="27">
@@ -3749,28 +3799,28 @@
       <c r="I114" s="27">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H114))),"",H114*$D$24)</f>
       </c>
-      <c r="J114" s="70">
+      <c r="J114" s="72">
         <f>IF($H$107&gt;0,1-H114/$H$107,0)</f>
       </c>
       <c r="K114" s="27"/>
       <c r="L114" s="27"/>
     </row>
-    <row r="115" ht="26" customHeight="1">
+    <row r="115" ht="20" customHeight="1">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
-      <c r="C115" s="71" t="n">
+      <c r="C115" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D115" s="74">
+      <c r="D115" s="76">
         <f>$D$35*(1-C115)</f>
       </c>
       <c r="E115" s="28">
         <f>$G$40/D115</f>
       </c>
-      <c r="F115" s="77">
+      <c r="F115" s="79">
         <f>IF(OR(D115="",E115=""),"",E115/D115)</f>
       </c>
-      <c r="G115" s="77">
+      <c r="G115" s="79">
         <f>IF(OR($D$24="",NOT(ISNUMBER(F115))),"",F115*$D$24)</f>
       </c>
       <c r="H115" s="28">
@@ -3779,17 +3829,17 @@
       <c r="I115" s="28">
         <f>IF(OR($D$24="",NOT(ISNUMBER(H115))),"",H115*$D$24)</f>
       </c>
-      <c r="J115" s="71">
+      <c r="J115" s="73">
         <f>IF($H$107&gt;0,1-H115/$H$107,0)</f>
       </c>
-      <c r="K115" s="94" t="str">
+      <c r="K115" s="96" t="str">
         <v>沉没成本 / Quote</v>
       </c>
       <c r="L115" s="28">
         <f>E115</f>
       </c>
     </row>
-    <row r="116" ht="26" customHeight="1">
+    <row r="116" ht="20" customHeight="1">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -3803,7 +3853,7 @@
       <c r="K116" s="2"/>
       <c r="L116" s="2"/>
     </row>
-    <row r="117" ht="26" customHeight="1">
+    <row r="117" ht="20" customHeight="1">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -3817,7 +3867,7 @@
       <c r="K117" s="2"/>
       <c r="L117" s="2"/>
     </row>
-    <row r="118" ht="26" customHeight="1">
+    <row r="118" ht="20" customHeight="1">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -3831,7 +3881,7 @@
       <c r="K118" s="2"/>
       <c r="L118" s="2"/>
     </row>
-    <row r="119" ht="26" customHeight="1">
+    <row r="119" ht="20" customHeight="1">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -3845,7 +3895,7 @@
       <c r="K119" s="2"/>
       <c r="L119" s="2"/>
     </row>
-    <row r="120" ht="26" customHeight="1">
+    <row r="120" ht="20" customHeight="1">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -3859,7 +3909,7 @@
       <c r="K120" s="2"/>
       <c r="L120" s="2"/>
     </row>
-    <row r="121" ht="26" customHeight="1">
+    <row r="121" ht="20" customHeight="1">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -3873,7 +3923,7 @@
       <c r="K121" s="2"/>
       <c r="L121" s="2"/>
     </row>
-    <row r="122" ht="26" customHeight="1">
+    <row r="122" ht="20" customHeight="1">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -3887,7 +3937,7 @@
       <c r="K122" s="2"/>
       <c r="L122" s="2"/>
     </row>
-    <row r="123" ht="26" customHeight="1">
+    <row r="123" ht="20" customHeight="1">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -3901,7 +3951,7 @@
       <c r="K123" s="2"/>
       <c r="L123" s="2"/>
     </row>
-    <row r="124" ht="26" customHeight="1">
+    <row r="124" ht="20" customHeight="1">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -3915,7 +3965,7 @@
       <c r="K124" s="2"/>
       <c r="L124" s="2"/>
     </row>
-    <row r="125" ht="26" customHeight="1">
+    <row r="125" ht="20" customHeight="1">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -3929,7 +3979,7 @@
       <c r="K125" s="2"/>
       <c r="L125" s="2"/>
     </row>
-    <row r="126" ht="26" customHeight="1">
+    <row r="126" ht="20" customHeight="1">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -3943,7 +3993,7 @@
       <c r="K126" s="2"/>
       <c r="L126" s="2"/>
     </row>
-    <row r="127" ht="26" customHeight="1">
+    <row r="127" ht="20" customHeight="1">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -3957,7 +4007,7 @@
       <c r="K127" s="2"/>
       <c r="L127" s="2"/>
     </row>
-    <row r="128" ht="26" customHeight="1">
+    <row r="128" ht="20" customHeight="1">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -3971,7 +4021,7 @@
       <c r="K128" s="2"/>
       <c r="L128" s="2"/>
     </row>
-    <row r="129" ht="26" customHeight="1">
+    <row r="129" ht="20" customHeight="1">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -3985,7 +4035,7 @@
       <c r="K129" s="2"/>
       <c r="L129" s="2"/>
     </row>
-    <row r="130" ht="26" customHeight="1">
+    <row r="130" ht="20" customHeight="1">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -3999,7 +4049,7 @@
       <c r="K130" s="2"/>
       <c r="L130" s="2"/>
     </row>
-    <row r="131" ht="26" customHeight="1">
+    <row r="131" ht="20" customHeight="1">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -4013,7 +4063,7 @@
       <c r="K131" s="2"/>
       <c r="L131" s="2"/>
     </row>
-    <row r="132" ht="26" customHeight="1">
+    <row r="132" ht="20" customHeight="1">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -4027,7 +4077,7 @@
       <c r="K132" s="2"/>
       <c r="L132" s="2"/>
     </row>
-    <row r="133" ht="26" customHeight="1">
+    <row r="133" ht="20" customHeight="1">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -4041,7 +4091,7 @@
       <c r="K133" s="2"/>
       <c r="L133" s="2"/>
     </row>
-    <row r="134" ht="26" customHeight="1">
+    <row r="134" ht="20" customHeight="1">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -4055,7 +4105,7 @@
       <c r="K134" s="2"/>
       <c r="L134" s="2"/>
     </row>
-    <row r="135" ht="26" customHeight="1">
+    <row r="135" ht="20" customHeight="1">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -4069,7 +4119,7 @@
       <c r="K135" s="2"/>
       <c r="L135" s="2"/>
     </row>
-    <row r="136" ht="26" customHeight="1">
+    <row r="136" ht="20" customHeight="1">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -4083,7 +4133,7 @@
       <c r="K136" s="2"/>
       <c r="L136" s="2"/>
     </row>
-    <row r="137" ht="26" customHeight="1">
+    <row r="137" ht="20" customHeight="1">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -4097,7 +4147,7 @@
       <c r="K137" s="2"/>
       <c r="L137" s="2"/>
     </row>
-    <row r="138" ht="26" customHeight="1">
+    <row r="138" ht="20" customHeight="1">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -4111,7 +4161,7 @@
       <c r="K138" s="2"/>
       <c r="L138" s="2"/>
     </row>
-    <row r="139" ht="26" customHeight="1">
+    <row r="139" ht="20" customHeight="1">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -4125,7 +4175,7 @@
       <c r="K139" s="2"/>
       <c r="L139" s="2"/>
     </row>
-    <row r="140" ht="26" customHeight="1">
+    <row r="140" ht="20" customHeight="1">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -4143,6 +4193,8 @@
   <mergeCells>
     <mergeCell ref="C3:L3"/>
     <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C19:L19"/>
+    <mergeCell ref="I28:L28"/>
     <mergeCell ref="I25:L25"/>
     <mergeCell ref="J23:L23"/>
     <mergeCell ref="G24:H24"/>
@@ -4191,7 +4243,7 @@
     <dataValidation type="whole" errorStyle="stop" operator="greaterThan" showErrorMessage="1" errorTitle="地址参数无效" error="输入非负整数；内盘套数至少为 1。" sqref="G10">
       <formula1>-1</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="between" showErrorMessage="1" errorTitle="参数无效" error="Gas 与资金预留不能为负数。" sqref="D10">
+    <dataValidation type="decimal" errorStyle="stop" operator="between" showErrorMessage="1" errorTitle="参数无效" error="Gas 与资金预留不能为负数。" sqref="G12">
       <formula1>0</formula1>
       <formula2>1e+307</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Preserve moved curve headers and percentage formatting
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R7875033a8ecc4db1"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R1cee2a598a844959"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rb68aa64bfa934638"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R639d5daa445c4a97"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="143">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -462,11 +462,24 @@
     <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -509,7 +522,69 @@
     <x:xf numFmtId="208" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="1" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="11" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="11" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="11" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1170,7 +1245,7 @@
       <c r="C18" s="101" t="str">
         <v>建议 Quote 资金</v>
       </c>
-      <c r="D18" s="111">
+      <c r="D18" s="114">
         <f>IF(ISNUMBER($D$26),(IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($D$22="","",SUM($D$22,$D$23,$D$24,$D$25))))+$D$26,"")</f>
       </c>
       <c r="E18" s="58">
@@ -1188,7 +1263,7 @@
       <c r="I18" s="101" t="str">
         <v>总折算 / USDT</v>
       </c>
-      <c r="J18" s="111">
+      <c r="J18" s="114">
         <f>IF(AND(ISNUMBER($D$19),ISNUMBER($G$19)),SUM(D19,G19),"")</f>
       </c>
       <c r="K18" s="58" t="str">
@@ -1202,7 +1277,7 @@
       <c r="C19" s="101" t="str">
         <v>Quote 折算 / USDT</v>
       </c>
-      <c r="D19" s="112">
+      <c r="D19" s="115">
         <f>IF(ISNUMBER($D$18),IF($D$18=0,0,IF($D$33&gt;0,$D$18*$D$33,"")),"")</f>
       </c>
       <c r="E19" s="100" t="str">
@@ -1211,7 +1286,7 @@
       <c r="F19" s="101" t="str">
         <v>Gas 折算 / USDT</v>
       </c>
-      <c r="G19" s="112">
+      <c r="G19" s="115">
         <f>IF($G$18=0,0,IF($J$19="","",$G$18*$J$19))</f>
       </c>
       <c r="H19" s="100" t="str">
@@ -1220,7 +1295,7 @@
       <c r="I19" s="101" t="str">
         <v>原生币价格 / USDT</v>
       </c>
-      <c r="J19" s="113">
+      <c r="J19" s="116">
         <f>IF($D$7="BNB",$D$33,IF('Quote参数'!$P$7&gt;0,'Quote参数'!$P$7,""))</f>
       </c>
       <c r="K19" s="100"/>
@@ -1264,7 +1339,7 @@
       <c r="C22" s="100">
         <f>"预算 "&amp;TEXT($D$31,"0%")&amp;" 理论资金"</f>
       </c>
-      <c r="D22" s="112">
+      <c r="D22" s="115">
         <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($J$45="","",$J$41+$J$45))</f>
       </c>
       <c r="E22" s="100">
@@ -1273,12 +1348,12 @@
       <c r="F22" s="100"/>
       <c r="G22" s="100"/>
       <c r="H22" s="100"/>
-      <c r="I22" s="109" t="str">
+      <c r="I22" s="112" t="str">
         <v>内盘</v>
       </c>
-      <c r="J22" s="110"/>
-      <c r="K22" s="110"/>
-      <c r="L22" s="110"/>
+      <c r="J22" s="113"/>
+      <c r="K22" s="113"/>
+      <c r="L22" s="113"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2"/>
@@ -1286,7 +1361,7 @@
       <c r="C23" s="101" t="str">
         <v>额外内盘资金</v>
       </c>
-      <c r="D23" s="112">
+      <c r="D23" s="115">
         <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",$J$41*MAX(0,$G$7-1))</f>
       </c>
       <c r="E23" s="100">
@@ -1298,7 +1373,7 @@
       <c r="I23" s="101" t="str">
         <v>基础手续费</v>
       </c>
-      <c r="J23" s="114">
+      <c r="J23" s="117">
         <f>$G$41</f>
       </c>
       <c r="K23" s="100"/>
@@ -1310,7 +1385,7 @@
       <c r="C24" s="101" t="str">
         <v>洗筹损耗</v>
       </c>
-      <c r="D24" s="112">
+      <c r="D24" s="115">
         <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($J$46="","",$J$46*$J$47))</f>
       </c>
       <c r="E24" s="100">
@@ -1322,7 +1397,7 @@
       <c r="I24" s="101" t="str">
         <v>买入含税费率</v>
       </c>
-      <c r="J24" s="114">
+      <c r="J24" s="117">
         <f>$G$41+$J$7</f>
       </c>
       <c r="K24" s="100"/>
@@ -1334,7 +1409,7 @@
       <c r="C25" s="101" t="str">
         <v>资金预留</v>
       </c>
-      <c r="D25" s="112">
+      <c r="D25" s="115">
         <f>MAX(0,$G$12)</f>
       </c>
       <c r="E25" s="100">
@@ -1346,7 +1421,7 @@
       <c r="I25" s="101" t="str">
         <v>卖出含税费率</v>
       </c>
-      <c r="J25" s="114">
+      <c r="J25" s="117">
         <f>$G$41+$J$8</f>
       </c>
       <c r="K25" s="100"/>
@@ -1358,7 +1433,7 @@
       <c r="C26" s="101" t="str">
         <v>恢复目标控筹资金</v>
       </c>
-      <c r="D26" s="112">
+      <c r="D26" s="115">
         <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)))</f>
       </c>
       <c r="E26" s="100">
@@ -1378,19 +1453,19 @@
       <c r="C27" s="101" t="str">
         <v>洗后控筹率（估算）</v>
       </c>
-      <c r="D27" s="115">
+      <c r="D27" s="118">
         <f>$D$8*$J$54</f>
       </c>
       <c r="E27" s="100"/>
       <c r="F27" s="100"/>
       <c r="G27" s="100"/>
       <c r="H27" s="100"/>
-      <c r="I27" s="109" t="str">
+      <c r="I27" s="112" t="str">
         <v>外盘 · LP</v>
       </c>
-      <c r="J27" s="110"/>
-      <c r="K27" s="110"/>
-      <c r="L27" s="110"/>
+      <c r="J27" s="113"/>
+      <c r="K27" s="113"/>
+      <c r="L27" s="113"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2"/>
@@ -1398,7 +1473,7 @@
       <c r="C28" s="101" t="str">
         <v>补回目标控筹率</v>
       </c>
-      <c r="D28" s="114">
+      <c r="D28" s="117">
         <f>$D$8</f>
       </c>
       <c r="E28" s="100"/>
@@ -1408,7 +1483,7 @@
       <c r="I28" s="101" t="str">
         <v>基础手续费</v>
       </c>
-      <c r="J28" s="114">
+      <c r="J28" s="117">
         <f>$G$42</f>
       </c>
       <c r="K28" s="100"/>
@@ -1420,7 +1495,7 @@
       <c r="C29" s="101" t="str">
         <v>洗筹双边总费率</v>
       </c>
-      <c r="D29" s="114">
+      <c r="D29" s="117">
         <f>$J$47</f>
       </c>
       <c r="E29" s="100"/>
@@ -1430,7 +1505,7 @@
       <c r="I29" s="101" t="str">
         <v>买入含税费率</v>
       </c>
-      <c r="J29" s="114">
+      <c r="J29" s="117">
         <f>$G$42+$J$7</f>
       </c>
       <c r="K29" s="100"/>
@@ -1452,7 +1527,7 @@
       <c r="I30" s="101" t="str">
         <v>卖出含税费率</v>
       </c>
-      <c r="J30" s="114">
+      <c r="J30" s="117">
         <f>$G$42+$J$8</f>
       </c>
       <c r="K30" s="100"/>
@@ -1464,7 +1539,7 @@
       <c r="C31" s="101" t="str">
         <v>预算使用控筹率</v>
       </c>
-      <c r="D31" s="114">
+      <c r="D31" s="117">
         <f>$D$8+1%</f>
       </c>
       <c r="E31" s="100"/>
@@ -1482,14 +1557,14 @@
       <c r="C32" s="101" t="str">
         <v>地址总数</v>
       </c>
-      <c r="D32" s="112">
+      <c r="D32" s="115">
         <f>MAX(0,$G$8)*MAX(0,$G$7)+MAX(0,$G$9)+MAX(0,$G$10)</f>
       </c>
       <c r="E32" s="100"/>
       <c r="F32" s="101" t="str">
         <v>当前控筹上限</v>
       </c>
-      <c r="G32" s="114">
+      <c r="G32" s="117">
         <f>$G$43+(1-$J$7)*$G$48/1000000000</f>
       </c>
       <c r="H32" s="100"/>
@@ -1504,7 +1579,7 @@
       <c r="C33" s="101" t="str">
         <v>Quote 价格 / USDT</v>
       </c>
-      <c r="D33" s="113">
+      <c r="D33" s="116">
         <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE),""))</f>
       </c>
       <c r="E33" s="100"/>
@@ -1522,7 +1597,7 @@
       <c r="C34" s="101" t="str">
         <v>行情时间 / UTC</v>
       </c>
-      <c r="D34" s="116">
+      <c r="D34" s="119">
         <f>IF(VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE))</f>
       </c>
       <c r="E34" s="100"/>
@@ -1557,32 +1632,32 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="105" t="str">
+      <c r="C36" s="108" t="str">
         <v>目标持仓直接 Quote 洗一轮，无额外路由费。控筹下降为小单固定价近似，补回资金为外盘曲线差额（含买税与 LP）。损耗仍按目标+1% FDV；补回是额外保守预留，非逐笔交易模拟。</v>
       </c>
-      <c r="D36" s="105"/>
-      <c r="E36" s="105"/>
-      <c r="F36" s="105"/>
-      <c r="G36" s="105"/>
-      <c r="H36" s="105"/>
-      <c r="I36" s="105"/>
-      <c r="J36" s="105"/>
-      <c r="K36" s="105"/>
-      <c r="L36" s="105"/>
+      <c r="D36" s="108"/>
+      <c r="E36" s="108"/>
+      <c r="F36" s="108"/>
+      <c r="G36" s="108"/>
+      <c r="H36" s="108"/>
+      <c r="I36" s="108"/>
+      <c r="J36" s="108"/>
+      <c r="K36" s="108"/>
+      <c r="L36" s="108"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="117" t="str">
+      <c r="C37" s="120" t="str">
         <v>沉没成本（模型参考，不重复计入预算）</v>
       </c>
-      <c r="D37" s="117"/>
-      <c r="E37" s="117"/>
-      <c r="F37" s="117"/>
-      <c r="G37" s="118">
+      <c r="D37" s="120"/>
+      <c r="E37" s="120"/>
+      <c r="F37" s="120"/>
+      <c r="G37" s="121">
         <f>E125</f>
       </c>
-      <c r="H37" s="117">
+      <c r="H37" s="120">
         <f>$D$7</f>
       </c>
       <c r="I37" s="100"/>
@@ -1607,448 +1682,448 @@
     <row r="39" ht="24" customHeight="1" collapsed="1">
       <c r="A39"/>
       <c r="B39"/>
-      <c r="C39" s="104" t="str">
+      <c r="C39" s="8" t="str">
         <v>三、模型信息与计算口径（默认折叠，点左侧 + 展开）</v>
       </c>
-      <c r="D39" s="104"/>
-      <c r="E39" s="104"/>
-      <c r="F39" s="104"/>
-      <c r="G39" s="104"/>
-      <c r="H39" s="104"/>
-      <c r="I39" s="104"/>
-      <c r="J39" s="104"/>
-      <c r="K39" s="104"/>
-      <c r="L39" s="104"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+    </row>
+    <row r="40" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A40"/>
       <c r="B40"/>
-      <c r="C40" t="str">
+      <c r="C40" s="101" t="str">
         <v>Quote 信息</v>
       </c>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40" t="str">
+      <c r="D40" s="101"/>
+      <c r="E40" s="101"/>
+      <c r="F40" s="101" t="str">
         <v>协议与曲线参数</v>
       </c>
-      <c r="G40"/>
-      <c r="H40"/>
-      <c r="I40" t="str">
+      <c r="G40" s="101"/>
+      <c r="H40" s="101"/>
+      <c r="I40" s="101" t="str">
         <v>预算中间计算</v>
       </c>
-      <c r="J40"/>
-      <c r="K40"/>
-      <c r="L40"/>
-    </row>
-    <row r="41" ht="36" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="J40" s="101"/>
+      <c r="K40" s="101"/>
+      <c r="L40" s="101"/>
+    </row>
+    <row r="41" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A41"/>
       <c r="B41"/>
-      <c r="C41" t="str">
+      <c r="C41" s="101" t="str">
         <v>Quote 名称</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="102">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,2,FALSE)</f>
       </c>
-      <c r="E41"/>
-      <c r="F41" t="str">
+      <c r="E41" s="101"/>
+      <c r="F41" s="101" t="str">
         <v>内盘基础费</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="106">
         <f>0.01</f>
       </c>
-      <c r="H41"/>
-      <c r="I41" t="str">
+      <c r="H41" s="101"/>
+      <c r="I41" s="101" t="str">
         <v>一套内盘打满 / Quote</v>
       </c>
-      <c r="J41">
+      <c r="J41" s="102">
         <f>$G$44*(1+$G$41+$J$7)</f>
       </c>
-      <c r="K41"/>
-      <c r="L41"/>
-    </row>
-    <row r="42" ht="36" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K41" s="101"/>
+      <c r="L41" s="101"/>
+    </row>
+    <row r="42" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A42"/>
       <c r="B42"/>
-      <c r="C42" t="str">
+      <c r="C42" s="101" t="str">
         <v>Quote 合约</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="103">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,3,FALSE)</f>
       </c>
-      <c r="E42"/>
-      <c r="F42" t="str">
+      <c r="E42" s="101"/>
+      <c r="F42" s="101" t="str">
         <v>外盘 LP 费</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="106">
         <f>0.0025</f>
       </c>
-      <c r="H42"/>
-      <c r="I42" t="str">
+      <c r="H42" s="101"/>
+      <c r="I42" s="101" t="str">
         <v>目标+1% Pool TOKEN</v>
       </c>
-      <c r="J42">
+      <c r="J42" s="102">
         <f>IF($J$49="","",$G$48-$J$49)</f>
       </c>
-      <c r="K42"/>
-      <c r="L42"/>
-    </row>
-    <row r="43" ht="36" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K42" s="101"/>
+      <c r="L42" s="101"/>
+    </row>
+    <row r="43" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A43"/>
       <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43" t="str">
+      <c r="C43" s="101"/>
+      <c r="D43" s="102"/>
+      <c r="E43" s="101"/>
+      <c r="F43" s="101" t="str">
         <v>毕业控筹率</v>
       </c>
-      <c r="G43">
+      <c r="G43" s="106">
         <f>0.8</f>
       </c>
-      <c r="H43"/>
-      <c r="I43" t="str">
+      <c r="H43" s="101"/>
+      <c r="I43" s="101" t="str">
         <v>目标+1% Pool Quote</v>
       </c>
-      <c r="J43">
+      <c r="J43" s="102">
         <f>IF($J$42="","",$G$50/$J$42)</f>
       </c>
-      <c r="K43"/>
-      <c r="L43"/>
-    </row>
-    <row r="44" ht="6" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K43" s="101"/>
+      <c r="L43" s="101"/>
+    </row>
+    <row r="44" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A44"/>
       <c r="B44"/>
-      <c r="C44" t="str">
+      <c r="C44" s="101" t="str">
         <v>Decimals</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="104">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,4,FALSE)</f>
       </c>
-      <c r="E44"/>
-      <c r="F44" t="str">
+      <c r="E44" s="101"/>
+      <c r="F44" s="101" t="str">
         <v>毕业真实 Quote</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="102">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,8,FALSE)</f>
       </c>
-      <c r="H44"/>
-      <c r="I44" t="str">
+      <c r="H44" s="101"/>
+      <c r="I44" s="101" t="str">
         <v>外盘净增加 / Quote</v>
       </c>
-      <c r="J44">
+      <c r="J44" s="102">
         <f>IF($J$43="","",MAX(0,$J$43-$G$44))</f>
       </c>
-      <c r="K44"/>
-      <c r="L44"/>
-    </row>
-    <row r="45" ht="6" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K44" s="101"/>
+      <c r="L44" s="101"/>
+    </row>
+    <row r="45" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A45"/>
       <c r="B45"/>
-      <c r="C45" t="str">
+      <c r="C45" s="101" t="str">
         <v>总供应量</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D45" s="105" t="n">
         <v>1000000000</v>
       </c>
-      <c r="E45"/>
-      <c r="F45" t="str">
+      <c r="E45" s="101"/>
+      <c r="F45" s="101" t="str">
         <v>内盘初始 TOKEN</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="102">
         <f>$D$45+$G$52</f>
       </c>
-      <c r="H45"/>
-      <c r="I45" t="str">
+      <c r="H45" s="101"/>
+      <c r="I45" s="101" t="str">
         <v>外盘含费投入 / Quote</v>
       </c>
-      <c r="J45">
+      <c r="J45" s="102">
         <f>IF($J$44="","",$J$44*(1+$G$42))</f>
       </c>
-      <c r="K45"/>
-      <c r="L45"/>
-    </row>
-    <row r="46" ht="6" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K45" s="101"/>
+      <c r="L45" s="101"/>
+    </row>
+    <row r="46" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A46"/>
       <c r="B46"/>
-      <c r="C46" t="str">
+      <c r="C46" s="101" t="str">
         <v>协议参数时点</v>
       </c>
-      <c r="D46" t="str">
+      <c r="D46" s="102" t="str">
         <v>2026-09-10 / block 121074671</v>
       </c>
-      <c r="E46"/>
-      <c r="F46" t="str">
+      <c r="E46" s="101"/>
+      <c r="F46" s="101" t="str">
         <v>虚拟 Quote r</v>
       </c>
-      <c r="G46">
+      <c r="G46" s="102">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,5,FALSE)</f>
       </c>
-      <c r="H46"/>
-      <c r="I46" t="str">
+      <c r="H46" s="101"/>
+      <c r="I46" s="101" t="str">
         <v>目标+1% FDV / Quote</v>
       </c>
-      <c r="J46">
+      <c r="J46" s="102">
         <f>IF($J$43="","",$J$43/$J$42*1000000000)</f>
       </c>
-      <c r="K46"/>
-      <c r="L46"/>
-    </row>
-    <row r="47" ht="24" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K46" s="101"/>
+      <c r="L46" s="101"/>
+    </row>
+    <row r="47" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A47"/>
       <c r="B47"/>
-      <c r="C47" t="str">
+      <c r="C47" s="101" t="str">
         <v>外盘机制</v>
       </c>
-      <c r="D47" t="str">
+      <c r="D47" s="102" t="str">
         <v>Pancake V3</v>
       </c>
-      <c r="E47"/>
-      <c r="F47" t="str">
+      <c r="E47" s="101"/>
+      <c r="F47" s="101" t="str">
         <v>内盘 k</v>
       </c>
-      <c r="G47">
+      <c r="G47" s="107">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,7,FALSE)</f>
       </c>
-      <c r="H47"/>
-      <c r="I47" t="str">
+      <c r="H47" s="101"/>
+      <c r="I47" s="101" t="str">
         <v>洗筹总费率</v>
       </c>
-      <c r="J47">
+      <c r="J47" s="106">
         <f>$G$42*2+$J$7+$J$8</f>
       </c>
-      <c r="K47"/>
-      <c r="L47"/>
+      <c r="K47" s="101"/>
+      <c r="L47" s="101"/>
     </row>
     <row r="48" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A48"/>
       <c r="B48"/>
-      <c r="C48" t="str">
+      <c r="C48" s="101" t="str">
         <v>费用方向</v>
       </c>
-      <c r="D48" t="str">
+      <c r="D48" s="102" t="str">
         <v>内盘买税加收 Quote；DEX 买税扣 TOKEN 输出</v>
       </c>
-      <c r="E48"/>
-      <c r="F48" t="str">
+      <c r="E48" s="101"/>
+      <c r="F48" s="101" t="str">
         <v>外盘初始 TOKEN</v>
       </c>
-      <c r="G48">
+      <c r="G48" s="102">
         <f>1000000000*(1-0.8)</f>
       </c>
-      <c r="H48"/>
-      <c r="I48" t="str">
+      <c r="H48" s="101"/>
+      <c r="I48" s="101" t="str">
         <v>外盘净控筹 TOKEN</v>
       </c>
-      <c r="J48">
+      <c r="J48" s="102">
         <f>IF($D$31&lt;$G$32,MAX(0,($D$31-$G$43)*1000000000),"")</f>
       </c>
-      <c r="K48"/>
-      <c r="L48"/>
-    </row>
-    <row r="49" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K48" s="101"/>
+      <c r="L48" s="101"/>
+    </row>
+    <row r="49" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A49"/>
       <c r="B49"/>
-      <c r="C49" t="str">
+      <c r="C49" s="101" t="str">
         <v>洗筹口径</v>
       </c>
-      <c r="D49" t="str">
+      <c r="D49" s="102" t="str">
         <v>目标+1% FDV ×（2×LP费 + 买税 + 卖税）</v>
       </c>
-      <c r="E49"/>
-      <c r="F49" t="str">
+      <c r="E49" s="101"/>
+      <c r="F49" s="101" t="str">
         <v>外盘初始 Quote</v>
       </c>
-      <c r="G49">
+      <c r="G49" s="102">
         <f>$G$44</f>
       </c>
-      <c r="H49"/>
-      <c r="I49" t="str">
+      <c r="H49" s="101"/>
+      <c r="I49" s="101" t="str">
         <v>外盘需扫 TOKEN</v>
       </c>
-      <c r="J49">
+      <c r="J49" s="102">
         <f>IF($J$48="","",$J$48/(1-$J$7))</f>
       </c>
-      <c r="K49"/>
-      <c r="L49"/>
-    </row>
-    <row r="50" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K49" s="101"/>
+      <c r="L49" s="101"/>
+    </row>
+    <row r="50" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A50"/>
       <c r="B50"/>
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50" t="str">
+      <c r="C50" s="101"/>
+      <c r="D50" s="102"/>
+      <c r="E50" s="101"/>
+      <c r="F50" s="101" t="str">
         <v>外盘 k</v>
       </c>
-      <c r="G50">
+      <c r="G50" s="107">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$N$36,10,FALSE)</f>
       </c>
-      <c r="H50"/>
-      <c r="I50"/>
-      <c r="J50"/>
-      <c r="K50"/>
-      <c r="L50"/>
-    </row>
-    <row r="51" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="H50" s="101"/>
+      <c r="I50" s="101"/>
+      <c r="J50" s="102"/>
+      <c r="K50" s="101"/>
+      <c r="L50" s="101"/>
+    </row>
+    <row r="51" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A51"/>
       <c r="B51"/>
-      <c r="C51"/>
-      <c r="D51"/>
-      <c r="E51"/>
-      <c r="F51" t="str">
+      <c r="C51" s="101"/>
+      <c r="D51" s="102"/>
+      <c r="E51" s="101"/>
+      <c r="F51" s="101" t="str">
         <v>协议来源</v>
       </c>
-      <c r="G51" t="str">
+      <c r="G51" s="102" t="str">
         <v>Quote参数页</v>
       </c>
-      <c r="H51"/>
-      <c r="I51" t="str">
+      <c r="H51" s="101"/>
+      <c r="I51" s="101" t="str">
         <v>输入检查</v>
       </c>
-      <c r="J51">
+      <c r="J51" s="102">
         <f>IF(COUNT($D$8,$G$7:$G$12,$J$7:$J$8)&lt;&gt;9,"缺少或非数值参数",IF(OR($G$7&lt;1,$G$8&lt;0,$G$9&lt;0,$G$10&lt;0,$G$11&lt;0,$G$12&lt;0,$G$7&lt;&gt;INT($G$7),$G$8&lt;&gt;INT($G$8),$G$9&lt;&gt;INT($G$9),$G$10&lt;&gt;INT($G$10)),"地址/Gas/预留参数无效","参数有效"))</f>
       </c>
-      <c r="K51"/>
-      <c r="L51"/>
-    </row>
-    <row r="52" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K51" s="101"/>
+      <c r="L51" s="101"/>
+    </row>
+    <row r="52" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A52"/>
       <c r="B52"/>
-      <c r="C52"/>
-      <c r="D52"/>
-      <c r="E52"/>
-      <c r="F52" t="str">
+      <c r="C52" s="101"/>
+      <c r="D52" s="102"/>
+      <c r="E52" s="101"/>
+      <c r="F52" s="101" t="str">
         <v>虚拟 TOKEN h</v>
       </c>
-      <c r="G52">
+      <c r="G52" s="102">
         <f>VLOOKUP($D$7,'Quote参数'!$E$14:$M$36,6,FALSE)</f>
       </c>
-      <c r="H52"/>
-      <c r="I52"/>
-      <c r="J52"/>
-      <c r="K52"/>
-      <c r="L52"/>
-    </row>
-    <row r="53" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="H52" s="101"/>
+      <c r="I52" s="101"/>
+      <c r="J52" s="102"/>
+      <c r="K52" s="101"/>
+      <c r="L52" s="101"/>
+    </row>
+    <row r="53" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A53"/>
       <c r="B53"/>
-      <c r="C53"/>
-      <c r="D53"/>
-      <c r="E53"/>
-      <c r="F53" t="str">
+      <c r="C53" s="101"/>
+      <c r="D53" s="102"/>
+      <c r="E53" s="101"/>
+      <c r="F53" s="101" t="str">
         <v>买税方向</v>
       </c>
-      <c r="G53" t="str">
+      <c r="G53" s="102" t="str">
         <v>TOKEN 输出端</v>
       </c>
-      <c r="H53"/>
-      <c r="I53"/>
-      <c r="J53"/>
-      <c r="K53"/>
-      <c r="L53"/>
-    </row>
-    <row r="54" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="H53" s="101"/>
+      <c r="I53" s="101"/>
+      <c r="J53" s="102"/>
+      <c r="K53" s="101"/>
+      <c r="L53" s="101"/>
+    </row>
+    <row r="54" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A54"/>
       <c r="B54"/>
-      <c r="C54"/>
-      <c r="D54"/>
-      <c r="E54"/>
-      <c r="F54"/>
-      <c r="G54"/>
-      <c r="H54"/>
-      <c r="I54" s="102" t="str">
+      <c r="C54" s="101"/>
+      <c r="D54" s="102"/>
+      <c r="E54" s="101"/>
+      <c r="F54" s="101"/>
+      <c r="G54" s="102"/>
+      <c r="H54" s="101"/>
+      <c r="I54" s="101" t="str">
         <v>洗后持仓保留比例</v>
       </c>
-      <c r="J54">
+      <c r="J54" s="106">
         <f>(1-$J$7)*(1-$J$8)*(1-$G$42)^2</f>
       </c>
-      <c r="K54"/>
-      <c r="L54"/>
-    </row>
-    <row r="55" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K54" s="101"/>
+      <c r="L54" s="101"/>
+    </row>
+    <row r="55" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A55"/>
       <c r="B55"/>
-      <c r="C55"/>
-      <c r="D55"/>
-      <c r="E55"/>
-      <c r="F55"/>
-      <c r="G55"/>
-      <c r="H55"/>
-      <c r="I55" s="102" t="str">
+      <c r="C55" s="101"/>
+      <c r="D55" s="102"/>
+      <c r="E55" s="101"/>
+      <c r="F55" s="101"/>
+      <c r="G55" s="102"/>
+      <c r="H55" s="101"/>
+      <c r="I55" s="101" t="str">
         <v>目标外盘 Pool TOKEN</v>
       </c>
-      <c r="J55">
+      <c r="J55" s="102">
         <f>$G$48-($D$8-$G$43)*$D$45/(1-$J$7)</f>
       </c>
-      <c r="K55"/>
-      <c r="L55"/>
-    </row>
-    <row r="56" ht="20" customHeight="1" outlineLevel="1" hidden="1">
+      <c r="K55" s="101"/>
+      <c r="L55" s="101"/>
+    </row>
+    <row r="56" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A56"/>
       <c r="B56"/>
-      <c r="C56"/>
-      <c r="D56"/>
-      <c r="E56"/>
-      <c r="F56"/>
-      <c r="G56"/>
-      <c r="H56"/>
-      <c r="I56" s="102" t="str">
+      <c r="C56" s="101"/>
+      <c r="D56" s="102"/>
+      <c r="E56" s="101"/>
+      <c r="F56" s="101"/>
+      <c r="G56" s="102"/>
+      <c r="H56" s="101"/>
+      <c r="I56" s="101" t="str">
         <v>洗后外盘 Pool TOKEN</v>
       </c>
-      <c r="J56">
+      <c r="J56" s="102">
         <f>$G$48-($D$27-$G$43)*$D$45/(1-$J$7)</f>
       </c>
-      <c r="K56"/>
-      <c r="L56"/>
-    </row>
-    <row r="57" ht="20" customHeight="1">
+      <c r="K56" s="101"/>
+      <c r="L56" s="101"/>
+    </row>
+    <row r="57" ht="24" customHeight="1">
       <c r="A57"/>
       <c r="B57"/>
-      <c r="C57" t="str">
+      <c r="C57" s="8" t="str">
         <v>内盘曲线</v>
       </c>
-      <c r="D57"/>
-      <c r="E57"/>
-      <c r="F57"/>
-      <c r="G57"/>
-      <c r="H57"/>
-      <c r="I57"/>
-      <c r="J57"/>
-      <c r="K57"/>
-      <c r="L57"/>
-    </row>
-    <row r="58" ht="20" customHeight="1">
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8"/>
+      <c r="L57" s="8"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
       <c r="A58"/>
       <c r="B58"/>
-      <c r="C58" t="str">
+      <c r="C58" s="71" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D58" t="str">
+      <c r="D58" s="71" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E58" t="str">
+      <c r="E58" s="71" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F58" t="str">
+      <c r="F58" s="71" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G58" t="str">
+      <c r="G58" s="71" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H58" t="str">
+      <c r="H58" s="71" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I58" t="str">
+      <c r="I58" s="71" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J58" t="str">
+      <c r="J58" s="71" t="str">
         <v>区间净投入
 / Quote</v>
       </c>
-      <c r="K58" t="str">
+      <c r="K58" s="71" t="str">
         <v>区间含费
 / Quote</v>
       </c>
-      <c r="L58" t="str">
+      <c r="L58" s="71" t="str">
         <v>理论累计所需
 / Quote</v>
       </c>
@@ -2056,386 +2131,386 @@
     <row r="59" ht="20" customHeight="1">
       <c r="A59"/>
       <c r="B59"/>
-      <c r="C59" t="n">
+      <c r="C59" s="125" t="n">
         <v>0</v>
       </c>
-      <c r="D59" s="119">
+      <c r="D59" s="137">
         <f>$D$45+$G$52-$D$45*C59</f>
       </c>
-      <c r="E59" s="119">
+      <c r="E59" s="137">
         <f>$G$47/D59</f>
       </c>
-      <c r="F59">
+      <c r="F59" s="128">
         <f>IF(OR(D59="",E59=""),"",E59/D59)</f>
       </c>
-      <c r="G59">
+      <c r="G59" s="128">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F59))),"",F59*$D$33)</f>
       </c>
-      <c r="H59" s="119">
+      <c r="H59" s="137">
         <f>IF(NOT(ISNUMBER(F59)),"",F59*$D$45)</f>
       </c>
-      <c r="I59" s="119">
+      <c r="I59" s="137">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H59))),"",H59*$D$33)</f>
       </c>
-      <c r="J59" s="119">
+      <c r="J59" s="137">
         <f>0</f>
       </c>
-      <c r="K59" s="119">
+      <c r="K59" s="137">
         <f>J59*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L59" s="119">
+      <c r="L59" s="140">
         <f>(E59-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
-    <row r="60" ht="24" customHeight="1">
+    <row r="60" ht="20" customHeight="1">
       <c r="A60"/>
       <c r="B60"/>
-      <c r="C60" t="n">
+      <c r="C60" s="126" t="n">
         <v>0.1</v>
       </c>
-      <c r="D60" s="119">
+      <c r="D60" s="138">
         <f>$D$45+$G$52-$D$45*C60</f>
       </c>
-      <c r="E60" s="119">
+      <c r="E60" s="138">
         <f>$G$47/D60</f>
       </c>
-      <c r="F60">
+      <c r="F60" s="129">
         <f>IF(OR(D60="",E60=""),"",E60/D60)</f>
       </c>
-      <c r="G60">
+      <c r="G60" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F60))),"",F60*$D$33)</f>
       </c>
-      <c r="H60" s="119">
+      <c r="H60" s="138">
         <f>IF(NOT(ISNUMBER(F60)),"",F60*$D$45)</f>
       </c>
-      <c r="I60" s="119">
+      <c r="I60" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H60))),"",H60*$D$33)</f>
       </c>
-      <c r="J60" s="119">
+      <c r="J60" s="138">
         <f>E60-E59</f>
       </c>
-      <c r="K60" s="119">
+      <c r="K60" s="138">
         <f>J60*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L60" s="119">
+      <c r="L60" s="141">
         <f>(E60-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
-    <row r="61" ht="30" customHeight="1">
+    <row r="61" ht="20" customHeight="1">
       <c r="A61"/>
       <c r="B61"/>
-      <c r="C61" t="n">
+      <c r="C61" s="126" t="n">
         <v>0.2</v>
       </c>
-      <c r="D61" s="119">
+      <c r="D61" s="138">
         <f>$D$45+$G$52-$D$45*C61</f>
       </c>
-      <c r="E61" s="119">
+      <c r="E61" s="138">
         <f>$G$47/D61</f>
       </c>
-      <c r="F61">
+      <c r="F61" s="129">
         <f>IF(OR(D61="",E61=""),"",E61/D61)</f>
       </c>
-      <c r="G61">
+      <c r="G61" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F61))),"",F61*$D$33)</f>
       </c>
-      <c r="H61" s="119">
+      <c r="H61" s="138">
         <f>IF(NOT(ISNUMBER(F61)),"",F61*$D$45)</f>
       </c>
-      <c r="I61" s="119">
+      <c r="I61" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H61))),"",H61*$D$33)</f>
       </c>
-      <c r="J61" s="119">
+      <c r="J61" s="138">
         <f>E61-E60</f>
       </c>
-      <c r="K61" s="119">
+      <c r="K61" s="138">
         <f>J61*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L61" s="119">
+      <c r="L61" s="141">
         <f>(E61-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62"/>
       <c r="B62"/>
-      <c r="C62" t="n">
+      <c r="C62" s="126" t="n">
         <v>0.3</v>
       </c>
-      <c r="D62" s="119">
+      <c r="D62" s="138">
         <f>$D$45+$G$52-$D$45*C62</f>
       </c>
-      <c r="E62" s="119">
+      <c r="E62" s="138">
         <f>$G$47/D62</f>
       </c>
-      <c r="F62">
+      <c r="F62" s="129">
         <f>IF(OR(D62="",E62=""),"",E62/D62)</f>
       </c>
-      <c r="G62">
+      <c r="G62" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F62))),"",F62*$D$33)</f>
       </c>
-      <c r="H62" s="119">
+      <c r="H62" s="138">
         <f>IF(NOT(ISNUMBER(F62)),"",F62*$D$45)</f>
       </c>
-      <c r="I62" s="119">
+      <c r="I62" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H62))),"",H62*$D$33)</f>
       </c>
-      <c r="J62" s="119">
+      <c r="J62" s="138">
         <f>E62-E61</f>
       </c>
-      <c r="K62" s="119">
+      <c r="K62" s="138">
         <f>J62*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L62" s="119">
+      <c r="L62" s="141">
         <f>(E62-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63"/>
       <c r="B63"/>
-      <c r="C63" t="n">
+      <c r="C63" s="126" t="n">
         <v>0.4</v>
       </c>
-      <c r="D63" s="119">
+      <c r="D63" s="138">
         <f>$D$45+$G$52-$D$45*C63</f>
       </c>
-      <c r="E63" s="119">
+      <c r="E63" s="138">
         <f>$G$47/D63</f>
       </c>
-      <c r="F63">
+      <c r="F63" s="129">
         <f>IF(OR(D63="",E63=""),"",E63/D63)</f>
       </c>
-      <c r="G63">
+      <c r="G63" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F63))),"",F63*$D$33)</f>
       </c>
-      <c r="H63" s="119">
+      <c r="H63" s="138">
         <f>IF(NOT(ISNUMBER(F63)),"",F63*$D$45)</f>
       </c>
-      <c r="I63" s="119">
+      <c r="I63" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H63))),"",H63*$D$33)</f>
       </c>
-      <c r="J63" s="119">
+      <c r="J63" s="138">
         <f>E63-E62</f>
       </c>
-      <c r="K63" s="119">
+      <c r="K63" s="138">
         <f>J63*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L63" s="119">
+      <c r="L63" s="141">
         <f>(E63-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64"/>
       <c r="B64"/>
-      <c r="C64" t="n">
+      <c r="C64" s="126" t="n">
         <v>0.5</v>
       </c>
-      <c r="D64" s="119">
+      <c r="D64" s="138">
         <f>$D$45+$G$52-$D$45*C64</f>
       </c>
-      <c r="E64" s="119">
+      <c r="E64" s="138">
         <f>$G$47/D64</f>
       </c>
-      <c r="F64">
+      <c r="F64" s="129">
         <f>IF(OR(D64="",E64=""),"",E64/D64)</f>
       </c>
-      <c r="G64">
+      <c r="G64" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F64))),"",F64*$D$33)</f>
       </c>
-      <c r="H64" s="119">
+      <c r="H64" s="138">
         <f>IF(NOT(ISNUMBER(F64)),"",F64*$D$45)</f>
       </c>
-      <c r="I64" s="119">
+      <c r="I64" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H64))),"",H64*$D$33)</f>
       </c>
-      <c r="J64" s="119">
+      <c r="J64" s="138">
         <f>E64-E63</f>
       </c>
-      <c r="K64" s="119">
+      <c r="K64" s="138">
         <f>J64*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L64" s="119">
+      <c r="L64" s="141">
         <f>(E64-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65"/>
       <c r="B65"/>
-      <c r="C65" t="n">
+      <c r="C65" s="126" t="n">
         <v>0.6</v>
       </c>
-      <c r="D65" s="119">
+      <c r="D65" s="138">
         <f>$D$45+$G$52-$D$45*C65</f>
       </c>
-      <c r="E65" s="119">
+      <c r="E65" s="138">
         <f>$G$47/D65</f>
       </c>
-      <c r="F65">
+      <c r="F65" s="129">
         <f>IF(OR(D65="",E65=""),"",E65/D65)</f>
       </c>
-      <c r="G65">
+      <c r="G65" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F65))),"",F65*$D$33)</f>
       </c>
-      <c r="H65" s="119">
+      <c r="H65" s="138">
         <f>IF(NOT(ISNUMBER(F65)),"",F65*$D$45)</f>
       </c>
-      <c r="I65" s="119">
+      <c r="I65" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H65))),"",H65*$D$33)</f>
       </c>
-      <c r="J65" s="119">
+      <c r="J65" s="138">
         <f>E65-E64</f>
       </c>
-      <c r="K65" s="119">
+      <c r="K65" s="138">
         <f>J65*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L65" s="119">
+      <c r="L65" s="141">
         <f>(E65-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66"/>
       <c r="B66"/>
-      <c r="C66" t="n">
+      <c r="C66" s="126" t="n">
         <v>0.7</v>
       </c>
-      <c r="D66" s="119">
+      <c r="D66" s="138">
         <f>$D$45+$G$52-$D$45*C66</f>
       </c>
-      <c r="E66" s="119">
+      <c r="E66" s="138">
         <f>$G$47/D66</f>
       </c>
-      <c r="F66">
+      <c r="F66" s="129">
         <f>IF(OR(D66="",E66=""),"",E66/D66)</f>
       </c>
-      <c r="G66">
+      <c r="G66" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F66))),"",F66*$D$33)</f>
       </c>
-      <c r="H66" s="119">
+      <c r="H66" s="138">
         <f>IF(NOT(ISNUMBER(F66)),"",F66*$D$45)</f>
       </c>
-      <c r="I66" s="119">
+      <c r="I66" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H66))),"",H66*$D$33)</f>
       </c>
-      <c r="J66" s="119">
+      <c r="J66" s="138">
         <f>E66-E65</f>
       </c>
-      <c r="K66" s="119">
+      <c r="K66" s="138">
         <f>J66*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L66" s="119">
+      <c r="L66" s="141">
         <f>(E66-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67"/>
       <c r="B67"/>
-      <c r="C67">
+      <c r="C67" s="127">
         <f>$G$43</f>
       </c>
-      <c r="D67" s="119">
+      <c r="D67" s="139">
         <f>$D$45+$G$52-$D$45*C67</f>
       </c>
-      <c r="E67" s="119">
+      <c r="E67" s="139">
         <f>$G$47/D67</f>
       </c>
-      <c r="F67">
+      <c r="F67" s="130">
         <f>IF(OR(D67="",E67=""),"",E67/D67)</f>
       </c>
-      <c r="G67">
+      <c r="G67" s="130">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F67))),"",F67*$D$33)</f>
       </c>
-      <c r="H67" s="119">
+      <c r="H67" s="139">
         <f>IF(NOT(ISNUMBER(F67)),"",F67*$D$45)</f>
       </c>
-      <c r="I67" s="119">
+      <c r="I67" s="139">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H67))),"",H67*$D$33)</f>
       </c>
-      <c r="J67" s="119">
+      <c r="J67" s="139">
         <f>E67-E66</f>
       </c>
-      <c r="K67" s="119">
+      <c r="K67" s="139">
         <f>J67*(1+$G$41+$J$7)</f>
       </c>
-      <c r="L67" s="119">
+      <c r="L67" s="142">
         <f>(E67-$G$46)*(1+$G$41+$J$7)</f>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68"/>
       <c r="B68"/>
-      <c r="C68"/>
-      <c r="D68"/>
-      <c r="E68"/>
-      <c r="F68"/>
-      <c r="G68"/>
-      <c r="H68"/>
-      <c r="I68"/>
-      <c r="J68"/>
-      <c r="K68"/>
-      <c r="L68"/>
+      <c r="C68" s="100"/>
+      <c r="D68" s="100"/>
+      <c r="E68" s="100"/>
+      <c r="F68" s="100"/>
+      <c r="G68" s="100"/>
+      <c r="H68" s="100"/>
+      <c r="I68" s="100"/>
+      <c r="J68" s="100"/>
+      <c r="K68" s="100"/>
+      <c r="L68" s="100"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69"/>
       <c r="B69"/>
-      <c r="C69"/>
-      <c r="D69"/>
-      <c r="E69"/>
-      <c r="F69"/>
-      <c r="G69"/>
-      <c r="H69"/>
-      <c r="I69"/>
-      <c r="J69"/>
-      <c r="K69"/>
-      <c r="L69"/>
-    </row>
-    <row r="70" ht="20" customHeight="1">
+      <c r="C69" s="100"/>
+      <c r="D69" s="100"/>
+      <c r="E69" s="100"/>
+      <c r="F69" s="100"/>
+      <c r="G69" s="100"/>
+      <c r="H69" s="100"/>
+      <c r="I69" s="100"/>
+      <c r="J69" s="100"/>
+      <c r="K69" s="100"/>
+      <c r="L69" s="100"/>
+    </row>
+    <row r="70" ht="24" customHeight="1">
       <c r="A70"/>
       <c r="B70"/>
-      <c r="C70" t="str">
+      <c r="C70" s="8" t="str">
         <v>外盘曲线</v>
       </c>
-      <c r="D70"/>
-      <c r="E70"/>
-      <c r="F70"/>
-      <c r="G70"/>
-      <c r="H70"/>
-      <c r="I70"/>
-      <c r="J70"/>
-      <c r="K70"/>
-      <c r="L70"/>
-    </row>
-    <row r="71" ht="20" customHeight="1">
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="8"/>
+      <c r="I70" s="8"/>
+      <c r="J70" s="8"/>
+      <c r="K70" s="8"/>
+      <c r="L70" s="8"/>
+    </row>
+    <row r="71" ht="32" customHeight="1">
       <c r="A71"/>
       <c r="B71"/>
-      <c r="C71" t="str">
+      <c r="C71" s="71" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D71" t="str">
+      <c r="D71" s="71" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E71" t="str">
+      <c r="E71" s="71" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F71" t="str">
+      <c r="F71" s="71" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G71" t="str">
+      <c r="G71" s="71" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H71" t="str">
+      <c r="H71" s="71" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I71" t="str">
+      <c r="I71" s="71" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J71" t="str">
+      <c r="J71" s="71" t="str">
         <v>外盘净投入
 / Quote</v>
       </c>
-      <c r="K71" t="str">
+      <c r="K71" s="71" t="str">
         <v>外盘含费
 / Quote</v>
       </c>
-      <c r="L71" t="str">
+      <c r="L71" s="71" t="str">
         <v>理论累计所需
 / Quote</v>
       </c>
@@ -2443,2094 +2518,2094 @@
     <row r="72" ht="20" customHeight="1">
       <c r="A72"/>
       <c r="B72"/>
-      <c r="C72">
+      <c r="C72" s="125">
         <f>$G$43</f>
       </c>
-      <c r="D72" s="119">
+      <c r="D72" s="137">
         <f>$G$48</f>
       </c>
-      <c r="E72" s="119">
+      <c r="E72" s="137">
         <f>$G$44</f>
       </c>
-      <c r="F72">
+      <c r="F72" s="128">
         <f>IF(OR(D72="",E72=""),"",E72/D72)</f>
       </c>
-      <c r="G72">
+      <c r="G72" s="128">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F72))),"",F72*$D$33)</f>
       </c>
-      <c r="H72" s="119">
+      <c r="H72" s="137">
         <f>IF(NOT(ISNUMBER(F72)),"",F72*$D$45)</f>
       </c>
-      <c r="I72" s="119">
+      <c r="I72" s="137">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H72))),"",H72*$D$33)</f>
       </c>
-      <c r="J72" s="119">
+      <c r="J72" s="137">
         <f>0</f>
       </c>
-      <c r="K72" s="119">
+      <c r="K72" s="137">
         <f>0</f>
       </c>
-      <c r="L72" s="119">
+      <c r="L72" s="140">
         <f>$J$41</f>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73"/>
       <c r="B73"/>
-      <c r="C73" t="n">
+      <c r="C73" s="126" t="n">
         <v>0.805</v>
       </c>
-      <c r="D73" s="119">
+      <c r="D73" s="138">
         <f>IF(C73&lt;$G$32,$G$48-MAX(0,(C73-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E73" s="119">
+      <c r="E73" s="138">
         <f>IF(D73="","",$G$50/D73)</f>
       </c>
-      <c r="F73">
+      <c r="F73" s="129">
         <f>IF(OR(D73="",E73=""),"",E73/D73)</f>
       </c>
-      <c r="G73">
+      <c r="G73" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F73))),"",F73*$D$33)</f>
       </c>
-      <c r="H73" s="119">
+      <c r="H73" s="138">
         <f>IF(NOT(ISNUMBER(F73)),"",F73*$D$45)</f>
       </c>
-      <c r="I73" s="119">
+      <c r="I73" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H73))),"",H73*$D$33)</f>
       </c>
-      <c r="J73" s="119">
+      <c r="J73" s="138">
         <f>IF(E73="","",MAX(0,E73-$G$44))</f>
       </c>
-      <c r="K73" s="119">
+      <c r="K73" s="138">
         <f>IF(J73="","",J73*(1+$G$42))</f>
       </c>
-      <c r="L73" s="119">
+      <c r="L73" s="141">
         <f>IF(K73="","",$J$41+K73)</f>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74"/>
       <c r="B74"/>
-      <c r="C74" t="n">
+      <c r="C74" s="126" t="n">
         <v>0.81</v>
       </c>
-      <c r="D74" s="119">
+      <c r="D74" s="138">
         <f>IF(C74&lt;$G$32,$G$48-MAX(0,(C74-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E74" s="119">
+      <c r="E74" s="138">
         <f>IF(D74="","",$G$50/D74)</f>
       </c>
-      <c r="F74">
+      <c r="F74" s="129">
         <f>IF(OR(D74="",E74=""),"",E74/D74)</f>
       </c>
-      <c r="G74">
+      <c r="G74" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F74))),"",F74*$D$33)</f>
       </c>
-      <c r="H74" s="119">
+      <c r="H74" s="138">
         <f>IF(NOT(ISNUMBER(F74)),"",F74*$D$45)</f>
       </c>
-      <c r="I74" s="119">
+      <c r="I74" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H74))),"",H74*$D$33)</f>
       </c>
-      <c r="J74" s="119">
+      <c r="J74" s="138">
         <f>IF(E74="","",MAX(0,E74-$G$44))</f>
       </c>
-      <c r="K74" s="119">
+      <c r="K74" s="138">
         <f>IF(J74="","",J74*(1+$G$42))</f>
       </c>
-      <c r="L74" s="119">
+      <c r="L74" s="141">
         <f>IF(K74="","",$J$41+K74)</f>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75"/>
       <c r="B75"/>
-      <c r="C75" t="n">
+      <c r="C75" s="126" t="n">
         <v>0.8150000000000001</v>
       </c>
-      <c r="D75" s="119">
+      <c r="D75" s="138">
         <f>IF(C75&lt;$G$32,$G$48-MAX(0,(C75-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E75" s="119">
+      <c r="E75" s="138">
         <f>IF(D75="","",$G$50/D75)</f>
       </c>
-      <c r="F75">
+      <c r="F75" s="129">
         <f>IF(OR(D75="",E75=""),"",E75/D75)</f>
       </c>
-      <c r="G75">
+      <c r="G75" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F75))),"",F75*$D$33)</f>
       </c>
-      <c r="H75" s="119">
+      <c r="H75" s="138">
         <f>IF(NOT(ISNUMBER(F75)),"",F75*$D$45)</f>
       </c>
-      <c r="I75" s="119">
+      <c r="I75" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H75))),"",H75*$D$33)</f>
       </c>
-      <c r="J75" s="119">
+      <c r="J75" s="138">
         <f>IF(E75="","",MAX(0,E75-$G$44))</f>
       </c>
-      <c r="K75" s="119">
+      <c r="K75" s="138">
         <f>IF(J75="","",J75*(1+$G$42))</f>
       </c>
-      <c r="L75" s="119">
+      <c r="L75" s="141">
         <f>IF(K75="","",$J$41+K75)</f>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76"/>
       <c r="B76"/>
-      <c r="C76" t="n">
+      <c r="C76" s="126" t="n">
         <v>0.8200000000000001</v>
       </c>
-      <c r="D76" s="119">
+      <c r="D76" s="138">
         <f>IF(C76&lt;$G$32,$G$48-MAX(0,(C76-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E76" s="119">
+      <c r="E76" s="138">
         <f>IF(D76="","",$G$50/D76)</f>
       </c>
-      <c r="F76">
+      <c r="F76" s="129">
         <f>IF(OR(D76="",E76=""),"",E76/D76)</f>
       </c>
-      <c r="G76">
+      <c r="G76" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F76))),"",F76*$D$33)</f>
       </c>
-      <c r="H76" s="119">
+      <c r="H76" s="138">
         <f>IF(NOT(ISNUMBER(F76)),"",F76*$D$45)</f>
       </c>
-      <c r="I76" s="119">
+      <c r="I76" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H76))),"",H76*$D$33)</f>
       </c>
-      <c r="J76" s="119">
+      <c r="J76" s="138">
         <f>IF(E76="","",MAX(0,E76-$G$44))</f>
       </c>
-      <c r="K76" s="119">
+      <c r="K76" s="138">
         <f>IF(J76="","",J76*(1+$G$42))</f>
       </c>
-      <c r="L76" s="119">
+      <c r="L76" s="141">
         <f>IF(K76="","",$J$41+K76)</f>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77"/>
       <c r="B77"/>
-      <c r="C77" t="n">
+      <c r="C77" s="126" t="n">
         <v>0.8250000000000001</v>
       </c>
-      <c r="D77" s="119">
+      <c r="D77" s="138">
         <f>IF(C77&lt;$G$32,$G$48-MAX(0,(C77-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E77" s="119">
+      <c r="E77" s="138">
         <f>IF(D77="","",$G$50/D77)</f>
       </c>
-      <c r="F77">
+      <c r="F77" s="129">
         <f>IF(OR(D77="",E77=""),"",E77/D77)</f>
       </c>
-      <c r="G77">
+      <c r="G77" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F77))),"",F77*$D$33)</f>
       </c>
-      <c r="H77" s="119">
+      <c r="H77" s="138">
         <f>IF(NOT(ISNUMBER(F77)),"",F77*$D$45)</f>
       </c>
-      <c r="I77" s="119">
+      <c r="I77" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H77))),"",H77*$D$33)</f>
       </c>
-      <c r="J77" s="119">
+      <c r="J77" s="138">
         <f>IF(E77="","",MAX(0,E77-$G$44))</f>
       </c>
-      <c r="K77" s="119">
+      <c r="K77" s="138">
         <f>IF(J77="","",J77*(1+$G$42))</f>
       </c>
-      <c r="L77" s="119">
+      <c r="L77" s="141">
         <f>IF(K77="","",$J$41+K77)</f>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78"/>
       <c r="B78"/>
-      <c r="C78" t="n">
+      <c r="C78" s="126" t="n">
         <v>0.8300000000000001</v>
       </c>
-      <c r="D78" s="119">
+      <c r="D78" s="138">
         <f>IF(C78&lt;$G$32,$G$48-MAX(0,(C78-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E78" s="119">
+      <c r="E78" s="138">
         <f>IF(D78="","",$G$50/D78)</f>
       </c>
-      <c r="F78">
+      <c r="F78" s="129">
         <f>IF(OR(D78="",E78=""),"",E78/D78)</f>
       </c>
-      <c r="G78">
+      <c r="G78" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F78))),"",F78*$D$33)</f>
       </c>
-      <c r="H78" s="119">
+      <c r="H78" s="138">
         <f>IF(NOT(ISNUMBER(F78)),"",F78*$D$45)</f>
       </c>
-      <c r="I78" s="119">
+      <c r="I78" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H78))),"",H78*$D$33)</f>
       </c>
-      <c r="J78" s="119">
+      <c r="J78" s="138">
         <f>IF(E78="","",MAX(0,E78-$G$44))</f>
       </c>
-      <c r="K78" s="119">
+      <c r="K78" s="138">
         <f>IF(J78="","",J78*(1+$G$42))</f>
       </c>
-      <c r="L78" s="119">
+      <c r="L78" s="141">
         <f>IF(K78="","",$J$41+K78)</f>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79"/>
       <c r="B79"/>
-      <c r="C79" t="n">
+      <c r="C79" s="126" t="n">
         <v>0.8350000000000001</v>
       </c>
-      <c r="D79" s="119">
+      <c r="D79" s="138">
         <f>IF(C79&lt;$G$32,$G$48-MAX(0,(C79-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E79" s="119">
+      <c r="E79" s="138">
         <f>IF(D79="","",$G$50/D79)</f>
       </c>
-      <c r="F79">
+      <c r="F79" s="129">
         <f>IF(OR(D79="",E79=""),"",E79/D79)</f>
       </c>
-      <c r="G79">
+      <c r="G79" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F79))),"",F79*$D$33)</f>
       </c>
-      <c r="H79" s="119">
+      <c r="H79" s="138">
         <f>IF(NOT(ISNUMBER(F79)),"",F79*$D$45)</f>
       </c>
-      <c r="I79" s="119">
+      <c r="I79" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H79))),"",H79*$D$33)</f>
       </c>
-      <c r="J79" s="119">
+      <c r="J79" s="138">
         <f>IF(E79="","",MAX(0,E79-$G$44))</f>
       </c>
-      <c r="K79" s="119">
+      <c r="K79" s="138">
         <f>IF(J79="","",J79*(1+$G$42))</f>
       </c>
-      <c r="L79" s="119">
+      <c r="L79" s="141">
         <f>IF(K79="","",$J$41+K79)</f>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80"/>
       <c r="B80"/>
-      <c r="C80" t="n">
+      <c r="C80" s="126" t="n">
         <v>0.8400000000000001</v>
       </c>
-      <c r="D80" s="119">
+      <c r="D80" s="138">
         <f>IF(C80&lt;$G$32,$G$48-MAX(0,(C80-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E80" s="119">
+      <c r="E80" s="138">
         <f>IF(D80="","",$G$50/D80)</f>
       </c>
-      <c r="F80">
+      <c r="F80" s="129">
         <f>IF(OR(D80="",E80=""),"",E80/D80)</f>
       </c>
-      <c r="G80">
+      <c r="G80" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F80))),"",F80*$D$33)</f>
       </c>
-      <c r="H80" s="119">
+      <c r="H80" s="138">
         <f>IF(NOT(ISNUMBER(F80)),"",F80*$D$45)</f>
       </c>
-      <c r="I80" s="119">
+      <c r="I80" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H80))),"",H80*$D$33)</f>
       </c>
-      <c r="J80" s="119">
+      <c r="J80" s="138">
         <f>IF(E80="","",MAX(0,E80-$G$44))</f>
       </c>
-      <c r="K80" s="119">
+      <c r="K80" s="138">
         <f>IF(J80="","",J80*(1+$G$42))</f>
       </c>
-      <c r="L80" s="119">
+      <c r="L80" s="141">
         <f>IF(K80="","",$J$41+K80)</f>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81"/>
       <c r="B81"/>
-      <c r="C81" t="n">
+      <c r="C81" s="126" t="n">
         <v>0.8450000000000001</v>
       </c>
-      <c r="D81" s="119">
+      <c r="D81" s="138">
         <f>IF(C81&lt;$G$32,$G$48-MAX(0,(C81-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E81" s="119">
+      <c r="E81" s="138">
         <f>IF(D81="","",$G$50/D81)</f>
       </c>
-      <c r="F81">
+      <c r="F81" s="129">
         <f>IF(OR(D81="",E81=""),"",E81/D81)</f>
       </c>
-      <c r="G81">
+      <c r="G81" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F81))),"",F81*$D$33)</f>
       </c>
-      <c r="H81" s="119">
+      <c r="H81" s="138">
         <f>IF(NOT(ISNUMBER(F81)),"",F81*$D$45)</f>
       </c>
-      <c r="I81" s="119">
+      <c r="I81" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H81))),"",H81*$D$33)</f>
       </c>
-      <c r="J81" s="119">
+      <c r="J81" s="138">
         <f>IF(E81="","",MAX(0,E81-$G$44))</f>
       </c>
-      <c r="K81" s="119">
+      <c r="K81" s="138">
         <f>IF(J81="","",J81*(1+$G$42))</f>
       </c>
-      <c r="L81" s="119">
+      <c r="L81" s="141">
         <f>IF(K81="","",$J$41+K81)</f>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82"/>
       <c r="B82"/>
-      <c r="C82" t="n">
+      <c r="C82" s="126" t="n">
         <v>0.8500000000000001</v>
       </c>
-      <c r="D82" s="119">
+      <c r="D82" s="138">
         <f>IF(C82&lt;$G$32,$G$48-MAX(0,(C82-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E82" s="119">
+      <c r="E82" s="138">
         <f>IF(D82="","",$G$50/D82)</f>
       </c>
-      <c r="F82">
+      <c r="F82" s="129">
         <f>IF(OR(D82="",E82=""),"",E82/D82)</f>
       </c>
-      <c r="G82">
+      <c r="G82" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F82))),"",F82*$D$33)</f>
       </c>
-      <c r="H82" s="119">
+      <c r="H82" s="138">
         <f>IF(NOT(ISNUMBER(F82)),"",F82*$D$45)</f>
       </c>
-      <c r="I82" s="119">
+      <c r="I82" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H82))),"",H82*$D$33)</f>
       </c>
-      <c r="J82" s="119">
+      <c r="J82" s="138">
         <f>IF(E82="","",MAX(0,E82-$G$44))</f>
       </c>
-      <c r="K82" s="119">
+      <c r="K82" s="138">
         <f>IF(J82="","",J82*(1+$G$42))</f>
       </c>
-      <c r="L82" s="119">
+      <c r="L82" s="141">
         <f>IF(K82="","",$J$41+K82)</f>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83"/>
       <c r="B83"/>
-      <c r="C83" t="n">
+      <c r="C83" s="126" t="n">
         <v>0.8550000000000001</v>
       </c>
-      <c r="D83" s="119">
+      <c r="D83" s="138">
         <f>IF(C83&lt;$G$32,$G$48-MAX(0,(C83-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E83" s="119">
+      <c r="E83" s="138">
         <f>IF(D83="","",$G$50/D83)</f>
       </c>
-      <c r="F83">
+      <c r="F83" s="129">
         <f>IF(OR(D83="",E83=""),"",E83/D83)</f>
       </c>
-      <c r="G83">
+      <c r="G83" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F83))),"",F83*$D$33)</f>
       </c>
-      <c r="H83" s="119">
+      <c r="H83" s="138">
         <f>IF(NOT(ISNUMBER(F83)),"",F83*$D$45)</f>
       </c>
-      <c r="I83" s="119">
+      <c r="I83" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H83))),"",H83*$D$33)</f>
       </c>
-      <c r="J83" s="119">
+      <c r="J83" s="138">
         <f>IF(E83="","",MAX(0,E83-$G$44))</f>
       </c>
-      <c r="K83" s="119">
+      <c r="K83" s="138">
         <f>IF(J83="","",J83*(1+$G$42))</f>
       </c>
-      <c r="L83" s="119">
+      <c r="L83" s="141">
         <f>IF(K83="","",$J$41+K83)</f>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84"/>
       <c r="B84"/>
-      <c r="C84" t="n">
+      <c r="C84" s="126" t="n">
         <v>0.8600000000000001</v>
       </c>
-      <c r="D84" s="119">
+      <c r="D84" s="138">
         <f>IF(C84&lt;$G$32,$G$48-MAX(0,(C84-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E84" s="119">
+      <c r="E84" s="138">
         <f>IF(D84="","",$G$50/D84)</f>
       </c>
-      <c r="F84">
+      <c r="F84" s="129">
         <f>IF(OR(D84="",E84=""),"",E84/D84)</f>
       </c>
-      <c r="G84">
+      <c r="G84" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F84))),"",F84*$D$33)</f>
       </c>
-      <c r="H84" s="119">
+      <c r="H84" s="138">
         <f>IF(NOT(ISNUMBER(F84)),"",F84*$D$45)</f>
       </c>
-      <c r="I84" s="119">
+      <c r="I84" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H84))),"",H84*$D$33)</f>
       </c>
-      <c r="J84" s="119">
+      <c r="J84" s="138">
         <f>IF(E84="","",MAX(0,E84-$G$44))</f>
       </c>
-      <c r="K84" s="119">
+      <c r="K84" s="138">
         <f>IF(J84="","",J84*(1+$G$42))</f>
       </c>
-      <c r="L84" s="119">
+      <c r="L84" s="141">
         <f>IF(K84="","",$J$41+K84)</f>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85"/>
       <c r="B85"/>
-      <c r="C85" t="n">
+      <c r="C85" s="126" t="n">
         <v>0.865</v>
       </c>
-      <c r="D85" s="119">
+      <c r="D85" s="138">
         <f>IF(C85&lt;$G$32,$G$48-MAX(0,(C85-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E85" s="119">
+      <c r="E85" s="138">
         <f>IF(D85="","",$G$50/D85)</f>
       </c>
-      <c r="F85">
+      <c r="F85" s="129">
         <f>IF(OR(D85="",E85=""),"",E85/D85)</f>
       </c>
-      <c r="G85">
+      <c r="G85" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F85))),"",F85*$D$33)</f>
       </c>
-      <c r="H85" s="119">
+      <c r="H85" s="138">
         <f>IF(NOT(ISNUMBER(F85)),"",F85*$D$45)</f>
       </c>
-      <c r="I85" s="119">
+      <c r="I85" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H85))),"",H85*$D$33)</f>
       </c>
-      <c r="J85" s="119">
+      <c r="J85" s="138">
         <f>IF(E85="","",MAX(0,E85-$G$44))</f>
       </c>
-      <c r="K85" s="119">
+      <c r="K85" s="138">
         <f>IF(J85="","",J85*(1+$G$42))</f>
       </c>
-      <c r="L85" s="119">
+      <c r="L85" s="141">
         <f>IF(K85="","",$J$41+K85)</f>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86"/>
       <c r="B86"/>
-      <c r="C86" t="n">
+      <c r="C86" s="126" t="n">
         <v>0.8700000000000001</v>
       </c>
-      <c r="D86" s="119">
+      <c r="D86" s="138">
         <f>IF(C86&lt;$G$32,$G$48-MAX(0,(C86-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E86" s="119">
+      <c r="E86" s="138">
         <f>IF(D86="","",$G$50/D86)</f>
       </c>
-      <c r="F86">
+      <c r="F86" s="129">
         <f>IF(OR(D86="",E86=""),"",E86/D86)</f>
       </c>
-      <c r="G86">
+      <c r="G86" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F86))),"",F86*$D$33)</f>
       </c>
-      <c r="H86" s="119">
+      <c r="H86" s="138">
         <f>IF(NOT(ISNUMBER(F86)),"",F86*$D$45)</f>
       </c>
-      <c r="I86" s="119">
+      <c r="I86" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H86))),"",H86*$D$33)</f>
       </c>
-      <c r="J86" s="119">
+      <c r="J86" s="138">
         <f>IF(E86="","",MAX(0,E86-$G$44))</f>
       </c>
-      <c r="K86" s="119">
+      <c r="K86" s="138">
         <f>IF(J86="","",J86*(1+$G$42))</f>
       </c>
-      <c r="L86" s="119">
+      <c r="L86" s="141">
         <f>IF(K86="","",$J$41+K86)</f>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87"/>
       <c r="B87"/>
-      <c r="C87" t="n">
+      <c r="C87" s="126" t="n">
         <v>0.875</v>
       </c>
-      <c r="D87" s="119">
+      <c r="D87" s="138">
         <f>IF(C87&lt;$G$32,$G$48-MAX(0,(C87-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E87" s="119">
+      <c r="E87" s="138">
         <f>IF(D87="","",$G$50/D87)</f>
       </c>
-      <c r="F87">
+      <c r="F87" s="129">
         <f>IF(OR(D87="",E87=""),"",E87/D87)</f>
       </c>
-      <c r="G87">
+      <c r="G87" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F87))),"",F87*$D$33)</f>
       </c>
-      <c r="H87" s="119">
+      <c r="H87" s="138">
         <f>IF(NOT(ISNUMBER(F87)),"",F87*$D$45)</f>
       </c>
-      <c r="I87" s="119">
+      <c r="I87" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H87))),"",H87*$D$33)</f>
       </c>
-      <c r="J87" s="119">
+      <c r="J87" s="138">
         <f>IF(E87="","",MAX(0,E87-$G$44))</f>
       </c>
-      <c r="K87" s="119">
+      <c r="K87" s="138">
         <f>IF(J87="","",J87*(1+$G$42))</f>
       </c>
-      <c r="L87" s="119">
+      <c r="L87" s="141">
         <f>IF(K87="","",$J$41+K87)</f>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88"/>
       <c r="B88"/>
-      <c r="C88" t="n">
+      <c r="C88" s="126" t="n">
         <v>0.88</v>
       </c>
-      <c r="D88" s="119">
+      <c r="D88" s="138">
         <f>IF(C88&lt;$G$32,$G$48-MAX(0,(C88-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E88" s="119">
+      <c r="E88" s="138">
         <f>IF(D88="","",$G$50/D88)</f>
       </c>
-      <c r="F88">
+      <c r="F88" s="129">
         <f>IF(OR(D88="",E88=""),"",E88/D88)</f>
       </c>
-      <c r="G88">
+      <c r="G88" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F88))),"",F88*$D$33)</f>
       </c>
-      <c r="H88" s="119">
+      <c r="H88" s="138">
         <f>IF(NOT(ISNUMBER(F88)),"",F88*$D$45)</f>
       </c>
-      <c r="I88" s="119">
+      <c r="I88" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H88))),"",H88*$D$33)</f>
       </c>
-      <c r="J88" s="119">
+      <c r="J88" s="138">
         <f>IF(E88="","",MAX(0,E88-$G$44))</f>
       </c>
-      <c r="K88" s="119">
+      <c r="K88" s="138">
         <f>IF(J88="","",J88*(1+$G$42))</f>
       </c>
-      <c r="L88" s="119">
+      <c r="L88" s="141">
         <f>IF(K88="","",$J$41+K88)</f>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89"/>
       <c r="B89"/>
-      <c r="C89" t="n">
+      <c r="C89" s="126" t="n">
         <v>0.885</v>
       </c>
-      <c r="D89" s="119">
+      <c r="D89" s="138">
         <f>IF(C89&lt;$G$32,$G$48-MAX(0,(C89-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E89" s="119">
+      <c r="E89" s="138">
         <f>IF(D89="","",$G$50/D89)</f>
       </c>
-      <c r="F89">
+      <c r="F89" s="129">
         <f>IF(OR(D89="",E89=""),"",E89/D89)</f>
       </c>
-      <c r="G89">
+      <c r="G89" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F89))),"",F89*$D$33)</f>
       </c>
-      <c r="H89" s="119">
+      <c r="H89" s="138">
         <f>IF(NOT(ISNUMBER(F89)),"",F89*$D$45)</f>
       </c>
-      <c r="I89" s="119">
+      <c r="I89" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H89))),"",H89*$D$33)</f>
       </c>
-      <c r="J89" s="119">
+      <c r="J89" s="138">
         <f>IF(E89="","",MAX(0,E89-$G$44))</f>
       </c>
-      <c r="K89" s="119">
+      <c r="K89" s="138">
         <f>IF(J89="","",J89*(1+$G$42))</f>
       </c>
-      <c r="L89" s="119">
+      <c r="L89" s="141">
         <f>IF(K89="","",$J$41+K89)</f>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90"/>
       <c r="B90"/>
-      <c r="C90" t="n">
+      <c r="C90" s="126" t="n">
         <v>0.89</v>
       </c>
-      <c r="D90" s="119">
+      <c r="D90" s="138">
         <f>IF(C90&lt;$G$32,$G$48-MAX(0,(C90-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E90" s="119">
+      <c r="E90" s="138">
         <f>IF(D90="","",$G$50/D90)</f>
       </c>
-      <c r="F90">
+      <c r="F90" s="129">
         <f>IF(OR(D90="",E90=""),"",E90/D90)</f>
       </c>
-      <c r="G90">
+      <c r="G90" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F90))),"",F90*$D$33)</f>
       </c>
-      <c r="H90" s="119">
+      <c r="H90" s="138">
         <f>IF(NOT(ISNUMBER(F90)),"",F90*$D$45)</f>
       </c>
-      <c r="I90" s="119">
+      <c r="I90" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H90))),"",H90*$D$33)</f>
       </c>
-      <c r="J90" s="119">
+      <c r="J90" s="138">
         <f>IF(E90="","",MAX(0,E90-$G$44))</f>
       </c>
-      <c r="K90" s="119">
+      <c r="K90" s="138">
         <f>IF(J90="","",J90*(1+$G$42))</f>
       </c>
-      <c r="L90" s="119">
+      <c r="L90" s="141">
         <f>IF(K90="","",$J$41+K90)</f>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91"/>
       <c r="B91"/>
-      <c r="C91" t="n">
+      <c r="C91" s="126" t="n">
         <v>0.895</v>
       </c>
-      <c r="D91" s="119">
+      <c r="D91" s="138">
         <f>IF(C91&lt;$G$32,$G$48-MAX(0,(C91-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E91" s="119">
+      <c r="E91" s="138">
         <f>IF(D91="","",$G$50/D91)</f>
       </c>
-      <c r="F91">
+      <c r="F91" s="129">
         <f>IF(OR(D91="",E91=""),"",E91/D91)</f>
       </c>
-      <c r="G91">
+      <c r="G91" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F91))),"",F91*$D$33)</f>
       </c>
-      <c r="H91" s="119">
+      <c r="H91" s="138">
         <f>IF(NOT(ISNUMBER(F91)),"",F91*$D$45)</f>
       </c>
-      <c r="I91" s="119">
+      <c r="I91" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H91))),"",H91*$D$33)</f>
       </c>
-      <c r="J91" s="119">
+      <c r="J91" s="138">
         <f>IF(E91="","",MAX(0,E91-$G$44))</f>
       </c>
-      <c r="K91" s="119">
+      <c r="K91" s="138">
         <f>IF(J91="","",J91*(1+$G$42))</f>
       </c>
-      <c r="L91" s="119">
+      <c r="L91" s="141">
         <f>IF(K91="","",$J$41+K91)</f>
       </c>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92"/>
       <c r="B92"/>
-      <c r="C92" t="n">
+      <c r="C92" s="126" t="n">
         <v>0.9</v>
       </c>
-      <c r="D92" s="119">
+      <c r="D92" s="138">
         <f>IF(C92&lt;$G$32,$G$48-MAX(0,(C92-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E92" s="119">
+      <c r="E92" s="138">
         <f>IF(D92="","",$G$50/D92)</f>
       </c>
-      <c r="F92">
+      <c r="F92" s="129">
         <f>IF(OR(D92="",E92=""),"",E92/D92)</f>
       </c>
-      <c r="G92">
+      <c r="G92" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F92))),"",F92*$D$33)</f>
       </c>
-      <c r="H92" s="119">
+      <c r="H92" s="138">
         <f>IF(NOT(ISNUMBER(F92)),"",F92*$D$45)</f>
       </c>
-      <c r="I92" s="119">
+      <c r="I92" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H92))),"",H92*$D$33)</f>
       </c>
-      <c r="J92" s="119">
+      <c r="J92" s="138">
         <f>IF(E92="","",MAX(0,E92-$G$44))</f>
       </c>
-      <c r="K92" s="119">
+      <c r="K92" s="138">
         <f>IF(J92="","",J92*(1+$G$42))</f>
       </c>
-      <c r="L92" s="119">
+      <c r="L92" s="141">
         <f>IF(K92="","",$J$41+K92)</f>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93"/>
       <c r="B93"/>
-      <c r="C93" t="n">
+      <c r="C93" s="126" t="n">
         <v>0.905</v>
       </c>
-      <c r="D93" s="119">
+      <c r="D93" s="138">
         <f>IF(C93&lt;$G$32,$G$48-MAX(0,(C93-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E93" s="119">
+      <c r="E93" s="138">
         <f>IF(D93="","",$G$50/D93)</f>
       </c>
-      <c r="F93">
+      <c r="F93" s="129">
         <f>IF(OR(D93="",E93=""),"",E93/D93)</f>
       </c>
-      <c r="G93">
+      <c r="G93" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F93))),"",F93*$D$33)</f>
       </c>
-      <c r="H93" s="119">
+      <c r="H93" s="138">
         <f>IF(NOT(ISNUMBER(F93)),"",F93*$D$45)</f>
       </c>
-      <c r="I93" s="119">
+      <c r="I93" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H93))),"",H93*$D$33)</f>
       </c>
-      <c r="J93" s="119">
+      <c r="J93" s="138">
         <f>IF(E93="","",MAX(0,E93-$G$44))</f>
       </c>
-      <c r="K93" s="119">
+      <c r="K93" s="138">
         <f>IF(J93="","",J93*(1+$G$42))</f>
       </c>
-      <c r="L93" s="119">
+      <c r="L93" s="141">
         <f>IF(K93="","",$J$41+K93)</f>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94"/>
       <c r="B94"/>
-      <c r="C94" t="n">
+      <c r="C94" s="126" t="n">
         <v>0.91</v>
       </c>
-      <c r="D94" s="119">
+      <c r="D94" s="138">
         <f>IF(C94&lt;$G$32,$G$48-MAX(0,(C94-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E94" s="119">
+      <c r="E94" s="138">
         <f>IF(D94="","",$G$50/D94)</f>
       </c>
-      <c r="F94">
+      <c r="F94" s="129">
         <f>IF(OR(D94="",E94=""),"",E94/D94)</f>
       </c>
-      <c r="G94">
+      <c r="G94" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F94))),"",F94*$D$33)</f>
       </c>
-      <c r="H94" s="119">
+      <c r="H94" s="138">
         <f>IF(NOT(ISNUMBER(F94)),"",F94*$D$45)</f>
       </c>
-      <c r="I94" s="119">
+      <c r="I94" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H94))),"",H94*$D$33)</f>
       </c>
-      <c r="J94" s="119">
+      <c r="J94" s="138">
         <f>IF(E94="","",MAX(0,E94-$G$44))</f>
       </c>
-      <c r="K94" s="119">
+      <c r="K94" s="138">
         <f>IF(J94="","",J94*(1+$G$42))</f>
       </c>
-      <c r="L94" s="119">
+      <c r="L94" s="141">
         <f>IF(K94="","",$J$41+K94)</f>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95"/>
       <c r="B95"/>
-      <c r="C95" t="n">
+      <c r="C95" s="126" t="n">
         <v>0.915</v>
       </c>
-      <c r="D95" s="119">
+      <c r="D95" s="138">
         <f>IF(C95&lt;$G$32,$G$48-MAX(0,(C95-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E95" s="119">
+      <c r="E95" s="138">
         <f>IF(D95="","",$G$50/D95)</f>
       </c>
-      <c r="F95">
+      <c r="F95" s="129">
         <f>IF(OR(D95="",E95=""),"",E95/D95)</f>
       </c>
-      <c r="G95">
+      <c r="G95" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F95))),"",F95*$D$33)</f>
       </c>
-      <c r="H95" s="119">
+      <c r="H95" s="138">
         <f>IF(NOT(ISNUMBER(F95)),"",F95*$D$45)</f>
       </c>
-      <c r="I95" s="119">
+      <c r="I95" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H95))),"",H95*$D$33)</f>
       </c>
-      <c r="J95" s="119">
+      <c r="J95" s="138">
         <f>IF(E95="","",MAX(0,E95-$G$44))</f>
       </c>
-      <c r="K95" s="119">
+      <c r="K95" s="138">
         <f>IF(J95="","",J95*(1+$G$42))</f>
       </c>
-      <c r="L95" s="119">
+      <c r="L95" s="141">
         <f>IF(K95="","",$J$41+K95)</f>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96"/>
       <c r="B96"/>
-      <c r="C96" t="n">
+      <c r="C96" s="126" t="n">
         <v>0.92</v>
       </c>
-      <c r="D96" s="119">
+      <c r="D96" s="138">
         <f>IF(C96&lt;$G$32,$G$48-MAX(0,(C96-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E96" s="119">
+      <c r="E96" s="138">
         <f>IF(D96="","",$G$50/D96)</f>
       </c>
-      <c r="F96">
+      <c r="F96" s="129">
         <f>IF(OR(D96="",E96=""),"",E96/D96)</f>
       </c>
-      <c r="G96">
+      <c r="G96" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F96))),"",F96*$D$33)</f>
       </c>
-      <c r="H96" s="119">
+      <c r="H96" s="138">
         <f>IF(NOT(ISNUMBER(F96)),"",F96*$D$45)</f>
       </c>
-      <c r="I96" s="119">
+      <c r="I96" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H96))),"",H96*$D$33)</f>
       </c>
-      <c r="J96" s="119">
+      <c r="J96" s="138">
         <f>IF(E96="","",MAX(0,E96-$G$44))</f>
       </c>
-      <c r="K96" s="119">
+      <c r="K96" s="138">
         <f>IF(J96="","",J96*(1+$G$42))</f>
       </c>
-      <c r="L96" s="119">
+      <c r="L96" s="141">
         <f>IF(K96="","",$J$41+K96)</f>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97"/>
       <c r="B97"/>
-      <c r="C97" t="n">
+      <c r="C97" s="126" t="n">
         <v>0.925</v>
       </c>
-      <c r="D97" s="119">
+      <c r="D97" s="138">
         <f>IF(C97&lt;$G$32,$G$48-MAX(0,(C97-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E97" s="119">
+      <c r="E97" s="138">
         <f>IF(D97="","",$G$50/D97)</f>
       </c>
-      <c r="F97">
+      <c r="F97" s="129">
         <f>IF(OR(D97="",E97=""),"",E97/D97)</f>
       </c>
-      <c r="G97">
+      <c r="G97" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F97))),"",F97*$D$33)</f>
       </c>
-      <c r="H97" s="119">
+      <c r="H97" s="138">
         <f>IF(NOT(ISNUMBER(F97)),"",F97*$D$45)</f>
       </c>
-      <c r="I97" s="119">
+      <c r="I97" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H97))),"",H97*$D$33)</f>
       </c>
-      <c r="J97" s="119">
+      <c r="J97" s="138">
         <f>IF(E97="","",MAX(0,E97-$G$44))</f>
       </c>
-      <c r="K97" s="119">
+      <c r="K97" s="138">
         <f>IF(J97="","",J97*(1+$G$42))</f>
       </c>
-      <c r="L97" s="119">
+      <c r="L97" s="141">
         <f>IF(K97="","",$J$41+K97)</f>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98"/>
       <c r="B98"/>
-      <c r="C98" t="n">
+      <c r="C98" s="126" t="n">
         <v>0.93</v>
       </c>
-      <c r="D98" s="119">
+      <c r="D98" s="138">
         <f>IF(C98&lt;$G$32,$G$48-MAX(0,(C98-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E98" s="119">
+      <c r="E98" s="138">
         <f>IF(D98="","",$G$50/D98)</f>
       </c>
-      <c r="F98">
+      <c r="F98" s="129">
         <f>IF(OR(D98="",E98=""),"",E98/D98)</f>
       </c>
-      <c r="G98">
+      <c r="G98" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F98))),"",F98*$D$33)</f>
       </c>
-      <c r="H98" s="119">
+      <c r="H98" s="138">
         <f>IF(NOT(ISNUMBER(F98)),"",F98*$D$45)</f>
       </c>
-      <c r="I98" s="119">
+      <c r="I98" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H98))),"",H98*$D$33)</f>
       </c>
-      <c r="J98" s="119">
+      <c r="J98" s="138">
         <f>IF(E98="","",MAX(0,E98-$G$44))</f>
       </c>
-      <c r="K98" s="119">
+      <c r="K98" s="138">
         <f>IF(J98="","",J98*(1+$G$42))</f>
       </c>
-      <c r="L98" s="119">
+      <c r="L98" s="141">
         <f>IF(K98="","",$J$41+K98)</f>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99"/>
       <c r="B99"/>
-      <c r="C99" t="n">
+      <c r="C99" s="126" t="n">
         <v>0.935</v>
       </c>
-      <c r="D99" s="119">
+      <c r="D99" s="138">
         <f>IF(C99&lt;$G$32,$G$48-MAX(0,(C99-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E99" s="119">
+      <c r="E99" s="138">
         <f>IF(D99="","",$G$50/D99)</f>
       </c>
-      <c r="F99">
+      <c r="F99" s="129">
         <f>IF(OR(D99="",E99=""),"",E99/D99)</f>
       </c>
-      <c r="G99">
+      <c r="G99" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F99))),"",F99*$D$33)</f>
       </c>
-      <c r="H99" s="119">
+      <c r="H99" s="138">
         <f>IF(NOT(ISNUMBER(F99)),"",F99*$D$45)</f>
       </c>
-      <c r="I99" s="119">
+      <c r="I99" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H99))),"",H99*$D$33)</f>
       </c>
-      <c r="J99" s="119">
+      <c r="J99" s="138">
         <f>IF(E99="","",MAX(0,E99-$G$44))</f>
       </c>
-      <c r="K99" s="119">
+      <c r="K99" s="138">
         <f>IF(J99="","",J99*(1+$G$42))</f>
       </c>
-      <c r="L99" s="119">
+      <c r="L99" s="141">
         <f>IF(K99="","",$J$41+K99)</f>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100"/>
       <c r="B100"/>
-      <c r="C100" t="n">
+      <c r="C100" s="126" t="n">
         <v>0.9400000000000001</v>
       </c>
-      <c r="D100" s="119">
+      <c r="D100" s="138">
         <f>IF(C100&lt;$G$32,$G$48-MAX(0,(C100-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E100" s="119">
+      <c r="E100" s="138">
         <f>IF(D100="","",$G$50/D100)</f>
       </c>
-      <c r="F100">
+      <c r="F100" s="129">
         <f>IF(OR(D100="",E100=""),"",E100/D100)</f>
       </c>
-      <c r="G100">
+      <c r="G100" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F100))),"",F100*$D$33)</f>
       </c>
-      <c r="H100" s="119">
+      <c r="H100" s="138">
         <f>IF(NOT(ISNUMBER(F100)),"",F100*$D$45)</f>
       </c>
-      <c r="I100" s="119">
+      <c r="I100" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H100))),"",H100*$D$33)</f>
       </c>
-      <c r="J100" s="119">
+      <c r="J100" s="138">
         <f>IF(E100="","",MAX(0,E100-$G$44))</f>
       </c>
-      <c r="K100" s="119">
+      <c r="K100" s="138">
         <f>IF(J100="","",J100*(1+$G$42))</f>
       </c>
-      <c r="L100" s="119">
+      <c r="L100" s="141">
         <f>IF(K100="","",$J$41+K100)</f>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101"/>
       <c r="B101"/>
-      <c r="C101" t="n">
+      <c r="C101" s="126" t="n">
         <v>0.9450000000000001</v>
       </c>
-      <c r="D101" s="119">
+      <c r="D101" s="138">
         <f>IF(C101&lt;$G$32,$G$48-MAX(0,(C101-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E101" s="119">
+      <c r="E101" s="138">
         <f>IF(D101="","",$G$50/D101)</f>
       </c>
-      <c r="F101">
+      <c r="F101" s="129">
         <f>IF(OR(D101="",E101=""),"",E101/D101)</f>
       </c>
-      <c r="G101">
+      <c r="G101" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F101))),"",F101*$D$33)</f>
       </c>
-      <c r="H101" s="119">
+      <c r="H101" s="138">
         <f>IF(NOT(ISNUMBER(F101)),"",F101*$D$45)</f>
       </c>
-      <c r="I101" s="119">
+      <c r="I101" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H101))),"",H101*$D$33)</f>
       </c>
-      <c r="J101" s="119">
+      <c r="J101" s="138">
         <f>IF(E101="","",MAX(0,E101-$G$44))</f>
       </c>
-      <c r="K101" s="119">
+      <c r="K101" s="138">
         <f>IF(J101="","",J101*(1+$G$42))</f>
       </c>
-      <c r="L101" s="119">
+      <c r="L101" s="141">
         <f>IF(K101="","",$J$41+K101)</f>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102"/>
       <c r="B102"/>
-      <c r="C102" t="n">
+      <c r="C102" s="126" t="n">
         <v>0.9500000000000001</v>
       </c>
-      <c r="D102" s="119">
+      <c r="D102" s="138">
         <f>IF(C102&lt;$G$32,$G$48-MAX(0,(C102-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E102" s="119">
+      <c r="E102" s="138">
         <f>IF(D102="","",$G$50/D102)</f>
       </c>
-      <c r="F102">
+      <c r="F102" s="129">
         <f>IF(OR(D102="",E102=""),"",E102/D102)</f>
       </c>
-      <c r="G102">
+      <c r="G102" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F102))),"",F102*$D$33)</f>
       </c>
-      <c r="H102" s="119">
+      <c r="H102" s="138">
         <f>IF(NOT(ISNUMBER(F102)),"",F102*$D$45)</f>
       </c>
-      <c r="I102" s="119">
+      <c r="I102" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H102))),"",H102*$D$33)</f>
       </c>
-      <c r="J102" s="119">
+      <c r="J102" s="138">
         <f>IF(E102="","",MAX(0,E102-$G$44))</f>
       </c>
-      <c r="K102" s="119">
+      <c r="K102" s="138">
         <f>IF(J102="","",J102*(1+$G$42))</f>
       </c>
-      <c r="L102" s="119">
+      <c r="L102" s="141">
         <f>IF(K102="","",$J$41+K102)</f>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103"/>
       <c r="B103"/>
-      <c r="C103" t="n">
+      <c r="C103" s="126" t="n">
         <v>0.9550000000000001</v>
       </c>
-      <c r="D103" s="119">
+      <c r="D103" s="138">
         <f>IF(C103&lt;$G$32,$G$48-MAX(0,(C103-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E103" s="119">
+      <c r="E103" s="138">
         <f>IF(D103="","",$G$50/D103)</f>
       </c>
-      <c r="F103">
+      <c r="F103" s="129">
         <f>IF(OR(D103="",E103=""),"",E103/D103)</f>
       </c>
-      <c r="G103">
+      <c r="G103" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F103))),"",F103*$D$33)</f>
       </c>
-      <c r="H103" s="119">
+      <c r="H103" s="138">
         <f>IF(NOT(ISNUMBER(F103)),"",F103*$D$45)</f>
       </c>
-      <c r="I103" s="119">
+      <c r="I103" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H103))),"",H103*$D$33)</f>
       </c>
-      <c r="J103" s="119">
+      <c r="J103" s="138">
         <f>IF(E103="","",MAX(0,E103-$G$44))</f>
       </c>
-      <c r="K103" s="119">
+      <c r="K103" s="138">
         <f>IF(J103="","",J103*(1+$G$42))</f>
       </c>
-      <c r="L103" s="119">
+      <c r="L103" s="141">
         <f>IF(K103="","",$J$41+K103)</f>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104"/>
       <c r="B104"/>
-      <c r="C104" t="n">
+      <c r="C104" s="126" t="n">
         <v>0.9600000000000001</v>
       </c>
-      <c r="D104" s="119">
+      <c r="D104" s="138">
         <f>IF(C104&lt;$G$32,$G$48-MAX(0,(C104-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E104" s="119">
+      <c r="E104" s="138">
         <f>IF(D104="","",$G$50/D104)</f>
       </c>
-      <c r="F104">
+      <c r="F104" s="129">
         <f>IF(OR(D104="",E104=""),"",E104/D104)</f>
       </c>
-      <c r="G104">
+      <c r="G104" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F104))),"",F104*$D$33)</f>
       </c>
-      <c r="H104" s="119">
+      <c r="H104" s="138">
         <f>IF(NOT(ISNUMBER(F104)),"",F104*$D$45)</f>
       </c>
-      <c r="I104" s="119">
+      <c r="I104" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H104))),"",H104*$D$33)</f>
       </c>
-      <c r="J104" s="119">
+      <c r="J104" s="138">
         <f>IF(E104="","",MAX(0,E104-$G$44))</f>
       </c>
-      <c r="K104" s="119">
+      <c r="K104" s="138">
         <f>IF(J104="","",J104*(1+$G$42))</f>
       </c>
-      <c r="L104" s="119">
+      <c r="L104" s="141">
         <f>IF(K104="","",$J$41+K104)</f>
       </c>
     </row>
-    <row r="105" ht="24" customHeight="1">
+    <row r="105" ht="20" customHeight="1">
       <c r="A105"/>
       <c r="B105"/>
-      <c r="C105" t="n">
+      <c r="C105" s="126" t="n">
         <v>0.9650000000000001</v>
       </c>
-      <c r="D105" s="119">
+      <c r="D105" s="138">
         <f>IF(C105&lt;$G$32,$G$48-MAX(0,(C105-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E105" s="119">
+      <c r="E105" s="138">
         <f>IF(D105="","",$G$50/D105)</f>
       </c>
-      <c r="F105">
+      <c r="F105" s="129">
         <f>IF(OR(D105="",E105=""),"",E105/D105)</f>
       </c>
-      <c r="G105">
+      <c r="G105" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F105))),"",F105*$D$33)</f>
       </c>
-      <c r="H105" s="119">
+      <c r="H105" s="138">
         <f>IF(NOT(ISNUMBER(F105)),"",F105*$D$45)</f>
       </c>
-      <c r="I105" s="119">
+      <c r="I105" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H105))),"",H105*$D$33)</f>
       </c>
-      <c r="J105" s="119">
+      <c r="J105" s="138">
         <f>IF(E105="","",MAX(0,E105-$G$44))</f>
       </c>
-      <c r="K105" s="119">
+      <c r="K105" s="138">
         <f>IF(J105="","",J105*(1+$G$42))</f>
       </c>
-      <c r="L105" s="119">
+      <c r="L105" s="141">
         <f>IF(K105="","",$J$41+K105)</f>
       </c>
     </row>
-    <row r="106" ht="30" customHeight="1">
+    <row r="106" ht="20" customHeight="1">
       <c r="A106"/>
       <c r="B106"/>
-      <c r="C106" t="n">
+      <c r="C106" s="126" t="n">
         <v>0.9700000000000001</v>
       </c>
-      <c r="D106" s="119">
+      <c r="D106" s="138">
         <f>IF(C106&lt;$G$32,$G$48-MAX(0,(C106-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E106" s="119">
+      <c r="E106" s="138">
         <f>IF(D106="","",$G$50/D106)</f>
       </c>
-      <c r="F106">
+      <c r="F106" s="129">
         <f>IF(OR(D106="",E106=""),"",E106/D106)</f>
       </c>
-      <c r="G106">
+      <c r="G106" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F106))),"",F106*$D$33)</f>
       </c>
-      <c r="H106" s="119">
+      <c r="H106" s="138">
         <f>IF(NOT(ISNUMBER(F106)),"",F106*$D$45)</f>
       </c>
-      <c r="I106" s="119">
+      <c r="I106" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H106))),"",H106*$D$33)</f>
       </c>
-      <c r="J106" s="119">
+      <c r="J106" s="138">
         <f>IF(E106="","",MAX(0,E106-$G$44))</f>
       </c>
-      <c r="K106" s="119">
+      <c r="K106" s="138">
         <f>IF(J106="","",J106*(1+$G$42))</f>
       </c>
-      <c r="L106" s="119">
+      <c r="L106" s="141">
         <f>IF(K106="","",$J$41+K106)</f>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107"/>
       <c r="B107"/>
-      <c r="C107" t="n">
+      <c r="C107" s="126" t="n">
         <v>0.9750000000000001</v>
       </c>
-      <c r="D107" s="119">
+      <c r="D107" s="138">
         <f>IF(C107&lt;$G$32,$G$48-MAX(0,(C107-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E107" s="119">
+      <c r="E107" s="138">
         <f>IF(D107="","",$G$50/D107)</f>
       </c>
-      <c r="F107">
+      <c r="F107" s="129">
         <f>IF(OR(D107="",E107=""),"",E107/D107)</f>
       </c>
-      <c r="G107">
+      <c r="G107" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F107))),"",F107*$D$33)</f>
       </c>
-      <c r="H107" s="119">
+      <c r="H107" s="138">
         <f>IF(NOT(ISNUMBER(F107)),"",F107*$D$45)</f>
       </c>
-      <c r="I107" s="119">
+      <c r="I107" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H107))),"",H107*$D$33)</f>
       </c>
-      <c r="J107" s="119">
+      <c r="J107" s="138">
         <f>IF(E107="","",MAX(0,E107-$G$44))</f>
       </c>
-      <c r="K107" s="119">
+      <c r="K107" s="138">
         <f>IF(J107="","",J107*(1+$G$42))</f>
       </c>
-      <c r="L107" s="119">
+      <c r="L107" s="141">
         <f>IF(K107="","",$J$41+K107)</f>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108"/>
       <c r="B108"/>
-      <c r="C108" t="n">
+      <c r="C108" s="126" t="n">
         <v>0.98</v>
       </c>
-      <c r="D108" s="119">
+      <c r="D108" s="138">
         <f>IF(C108&lt;$G$32,$G$48-MAX(0,(C108-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E108" s="119">
+      <c r="E108" s="138">
         <f>IF(D108="","",$G$50/D108)</f>
       </c>
-      <c r="F108">
+      <c r="F108" s="129">
         <f>IF(OR(D108="",E108=""),"",E108/D108)</f>
       </c>
-      <c r="G108">
+      <c r="G108" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F108))),"",F108*$D$33)</f>
       </c>
-      <c r="H108" s="119">
+      <c r="H108" s="138">
         <f>IF(NOT(ISNUMBER(F108)),"",F108*$D$45)</f>
       </c>
-      <c r="I108" s="119">
+      <c r="I108" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H108))),"",H108*$D$33)</f>
       </c>
-      <c r="J108" s="119">
+      <c r="J108" s="138">
         <f>IF(E108="","",MAX(0,E108-$G$44))</f>
       </c>
-      <c r="K108" s="119">
+      <c r="K108" s="138">
         <f>IF(J108="","",J108*(1+$G$42))</f>
       </c>
-      <c r="L108" s="119">
+      <c r="L108" s="141">
         <f>IF(K108="","",$J$41+K108)</f>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109"/>
       <c r="B109"/>
-      <c r="C109" t="n">
+      <c r="C109" s="126" t="n">
         <v>0.9850000000000001</v>
       </c>
-      <c r="D109" s="119">
+      <c r="D109" s="138">
         <f>IF(C109&lt;$G$32,$G$48-MAX(0,(C109-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E109" s="119">
+      <c r="E109" s="138">
         <f>IF(D109="","",$G$50/D109)</f>
       </c>
-      <c r="F109">
+      <c r="F109" s="129">
         <f>IF(OR(D109="",E109=""),"",E109/D109)</f>
       </c>
-      <c r="G109">
+      <c r="G109" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F109))),"",F109*$D$33)</f>
       </c>
-      <c r="H109" s="119">
+      <c r="H109" s="138">
         <f>IF(NOT(ISNUMBER(F109)),"",F109*$D$45)</f>
       </c>
-      <c r="I109" s="119">
+      <c r="I109" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H109))),"",H109*$D$33)</f>
       </c>
-      <c r="J109" s="119">
+      <c r="J109" s="138">
         <f>IF(E109="","",MAX(0,E109-$G$44))</f>
       </c>
-      <c r="K109" s="119">
+      <c r="K109" s="138">
         <f>IF(J109="","",J109*(1+$G$42))</f>
       </c>
-      <c r="L109" s="119">
+      <c r="L109" s="141">
         <f>IF(K109="","",$J$41+K109)</f>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110"/>
       <c r="B110"/>
-      <c r="C110" t="n">
+      <c r="C110" s="126" t="n">
         <v>0.99</v>
       </c>
-      <c r="D110" s="119">
+      <c r="D110" s="138">
         <f>IF(C110&lt;$G$32,$G$48-MAX(0,(C110-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E110" s="119">
+      <c r="E110" s="138">
         <f>IF(D110="","",$G$50/D110)</f>
       </c>
-      <c r="F110">
+      <c r="F110" s="129">
         <f>IF(OR(D110="",E110=""),"",E110/D110)</f>
       </c>
-      <c r="G110">
+      <c r="G110" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F110))),"",F110*$D$33)</f>
       </c>
-      <c r="H110" s="119">
+      <c r="H110" s="138">
         <f>IF(NOT(ISNUMBER(F110)),"",F110*$D$45)</f>
       </c>
-      <c r="I110" s="119">
+      <c r="I110" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H110))),"",H110*$D$33)</f>
       </c>
-      <c r="J110" s="119">
+      <c r="J110" s="138">
         <f>IF(E110="","",MAX(0,E110-$G$44))</f>
       </c>
-      <c r="K110" s="119">
+      <c r="K110" s="138">
         <f>IF(J110="","",J110*(1+$G$42))</f>
       </c>
-      <c r="L110" s="119">
+      <c r="L110" s="141">
         <f>IF(K110="","",$J$41+K110)</f>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111"/>
       <c r="B111"/>
-      <c r="C111" t="n">
+      <c r="C111" s="126" t="n">
         <v>0.9950000000000001</v>
       </c>
-      <c r="D111" s="119">
+      <c r="D111" s="138">
         <f>IF(C111&lt;$G$32,$G$48-MAX(0,(C111-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E111" s="119">
+      <c r="E111" s="138">
         <f>IF(D111="","",$G$50/D111)</f>
       </c>
-      <c r="F111">
+      <c r="F111" s="129">
         <f>IF(OR(D111="",E111=""),"",E111/D111)</f>
       </c>
-      <c r="G111">
+      <c r="G111" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F111))),"",F111*$D$33)</f>
       </c>
-      <c r="H111" s="119">
+      <c r="H111" s="138">
         <f>IF(NOT(ISNUMBER(F111)),"",F111*$D$45)</f>
       </c>
-      <c r="I111" s="119">
+      <c r="I111" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H111))),"",H111*$D$33)</f>
       </c>
-      <c r="J111" s="119">
+      <c r="J111" s="138">
         <f>IF(E111="","",MAX(0,E111-$G$44))</f>
       </c>
-      <c r="K111" s="119">
+      <c r="K111" s="138">
         <f>IF(J111="","",J111*(1+$G$42))</f>
       </c>
-      <c r="L111" s="119">
+      <c r="L111" s="141">
         <f>IF(K111="","",$J$41+K111)</f>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112"/>
       <c r="B112"/>
-      <c r="C112" t="n">
+      <c r="C112" s="127" t="n">
         <v>1</v>
       </c>
-      <c r="D112" s="119">
+      <c r="D112" s="139">
         <f>IF(C112&lt;$G$32,$G$48-MAX(0,(C112-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
-      <c r="E112" s="119">
+      <c r="E112" s="139">
         <f>IF(D112="","",$G$50/D112)</f>
       </c>
-      <c r="F112">
+      <c r="F112" s="130">
         <f>IF(OR(D112="",E112=""),"",E112/D112)</f>
       </c>
-      <c r="G112">
+      <c r="G112" s="130">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F112))),"",F112*$D$33)</f>
       </c>
-      <c r="H112" s="119">
+      <c r="H112" s="139">
         <f>IF(NOT(ISNUMBER(F112)),"",F112*$D$45)</f>
       </c>
-      <c r="I112" s="119">
+      <c r="I112" s="139">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H112))),"",H112*$D$33)</f>
       </c>
-      <c r="J112" s="119">
+      <c r="J112" s="139">
         <f>IF(E112="","",MAX(0,E112-$G$44))</f>
       </c>
-      <c r="K112" s="119">
+      <c r="K112" s="139">
         <f>IF(J112="","",J112*(1+$G$42))</f>
       </c>
-      <c r="L112" s="119">
+      <c r="L112" s="142">
         <f>IF(K112="","",$J$41+K112)</f>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113"/>
       <c r="B113"/>
-      <c r="C113"/>
-      <c r="D113"/>
-      <c r="E113"/>
-      <c r="F113"/>
-      <c r="G113"/>
-      <c r="H113"/>
-      <c r="I113"/>
-      <c r="J113"/>
-      <c r="K113"/>
-      <c r="L113"/>
+      <c r="C113" s="100"/>
+      <c r="D113" s="100"/>
+      <c r="E113" s="100"/>
+      <c r="F113" s="100"/>
+      <c r="G113" s="100"/>
+      <c r="H113" s="100"/>
+      <c r="I113" s="100"/>
+      <c r="J113" s="100"/>
+      <c r="K113" s="100"/>
+      <c r="L113" s="100"/>
     </row>
     <row r="114" ht="20" customHeight="1">
       <c r="A114"/>
       <c r="B114"/>
-      <c r="C114"/>
-      <c r="D114"/>
-      <c r="E114"/>
-      <c r="F114"/>
-      <c r="G114"/>
-      <c r="H114"/>
-      <c r="I114"/>
-      <c r="J114"/>
-      <c r="K114"/>
-      <c r="L114"/>
-    </row>
-    <row r="115" ht="20" customHeight="1">
+      <c r="C114" s="100"/>
+      <c r="D114" s="100"/>
+      <c r="E114" s="100"/>
+      <c r="F114" s="100"/>
+      <c r="G114" s="100"/>
+      <c r="H114" s="100"/>
+      <c r="I114" s="100"/>
+      <c r="J114" s="100"/>
+      <c r="K114" s="100"/>
+      <c r="L114" s="100"/>
+    </row>
+    <row r="115" ht="24" customHeight="1">
       <c r="A115"/>
       <c r="B115"/>
-      <c r="C115" t="str">
+      <c r="C115" s="96" t="str">
         <v>外盘回落参考</v>
       </c>
-      <c r="D115"/>
-      <c r="E115"/>
-      <c r="F115"/>
-      <c r="G115"/>
-      <c r="H115"/>
-      <c r="I115"/>
-      <c r="J115"/>
-      <c r="K115"/>
-      <c r="L115"/>
-    </row>
-    <row r="116" ht="20" customHeight="1">
+      <c r="D115" s="96"/>
+      <c r="E115" s="96"/>
+      <c r="F115" s="96"/>
+      <c r="G115" s="96"/>
+      <c r="H115" s="96"/>
+      <c r="I115" s="96"/>
+      <c r="J115" s="96"/>
+      <c r="K115" s="96"/>
+      <c r="L115" s="96"/>
+    </row>
+    <row r="116" ht="32" customHeight="1">
       <c r="A116"/>
       <c r="B116"/>
-      <c r="C116" t="str">
+      <c r="C116" s="71" t="str">
         <v>控筹率</v>
       </c>
-      <c r="D116" t="str">
+      <c r="D116" s="71" t="str">
         <v>pooled TOKEN</v>
       </c>
-      <c r="E116" t="str">
+      <c r="E116" s="71" t="str">
         <v>pooled Quote</v>
       </c>
-      <c r="F116" t="str">
+      <c r="F116" s="71" t="str">
         <v>价格 / Quote</v>
       </c>
-      <c r="G116" t="str">
+      <c r="G116" s="71" t="str">
         <v>价格 / USDT</v>
       </c>
-      <c r="H116" t="str">
+      <c r="H116" s="71" t="str">
         <v>市值 / Quote</v>
       </c>
-      <c r="I116" t="str">
+      <c r="I116" s="71" t="str">
         <v>市值 / USDT</v>
       </c>
-      <c r="J116" t="str">
+      <c r="J116" s="71" t="str">
         <v>较毕业点回撤</v>
       </c>
-      <c r="K116" t="str"/>
-      <c r="L116" t="str"/>
+      <c r="K116" s="71" t="str"/>
+      <c r="L116" s="71" t="str"/>
     </row>
     <row r="117" ht="20" customHeight="1">
       <c r="A117"/>
       <c r="B117"/>
-      <c r="C117" t="n">
+      <c r="C117" s="125" t="n">
         <v>0.8</v>
       </c>
-      <c r="D117" s="119">
+      <c r="D117" s="137">
         <f>$D$45*(1-C117)</f>
       </c>
-      <c r="E117" s="119">
+      <c r="E117" s="137">
         <f>$G$50/D117</f>
       </c>
-      <c r="F117">
+      <c r="F117" s="128">
         <f>IF(OR(D117="",E117=""),"",E117/D117)</f>
       </c>
-      <c r="G117">
+      <c r="G117" s="128">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F117))),"",F117*$D$33)</f>
       </c>
-      <c r="H117" s="119">
+      <c r="H117" s="137">
         <f>IF(NOT(ISNUMBER(F117)),"",F117*$D$45)</f>
       </c>
-      <c r="I117" s="119">
+      <c r="I117" s="137">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H117))),"",H117*$D$33)</f>
       </c>
-      <c r="J117">
+      <c r="J117" s="125">
         <f>IF($H$117&gt;0,1-H117/$H$117,0)</f>
       </c>
-      <c r="K117"/>
-      <c r="L117"/>
+      <c r="K117" s="122"/>
+      <c r="L117" s="122"/>
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118"/>
       <c r="B118"/>
-      <c r="C118" t="n">
+      <c r="C118" s="126" t="n">
         <v>0.7</v>
       </c>
-      <c r="D118" s="119">
+      <c r="D118" s="138">
         <f>$D$45*(1-C118)</f>
       </c>
-      <c r="E118" s="119">
+      <c r="E118" s="138">
         <f>$G$50/D118</f>
       </c>
-      <c r="F118">
+      <c r="F118" s="129">
         <f>IF(OR(D118="",E118=""),"",E118/D118)</f>
       </c>
-      <c r="G118">
+      <c r="G118" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F118))),"",F118*$D$33)</f>
       </c>
-      <c r="H118" s="119">
+      <c r="H118" s="138">
         <f>IF(NOT(ISNUMBER(F118)),"",F118*$D$45)</f>
       </c>
-      <c r="I118" s="119">
+      <c r="I118" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H118))),"",H118*$D$33)</f>
       </c>
-      <c r="J118">
+      <c r="J118" s="126">
         <f>IF($H$117&gt;0,1-H118/$H$117,0)</f>
       </c>
-      <c r="K118"/>
-      <c r="L118"/>
+      <c r="K118" s="123"/>
+      <c r="L118" s="123"/>
     </row>
     <row r="119" ht="20" customHeight="1">
       <c r="A119"/>
       <c r="B119"/>
-      <c r="C119" t="n">
+      <c r="C119" s="126" t="n">
         <v>0.6</v>
       </c>
-      <c r="D119" s="119">
+      <c r="D119" s="138">
         <f>$D$45*(1-C119)</f>
       </c>
-      <c r="E119" s="119">
+      <c r="E119" s="138">
         <f>$G$50/D119</f>
       </c>
-      <c r="F119">
+      <c r="F119" s="129">
         <f>IF(OR(D119="",E119=""),"",E119/D119)</f>
       </c>
-      <c r="G119">
+      <c r="G119" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F119))),"",F119*$D$33)</f>
       </c>
-      <c r="H119" s="119">
+      <c r="H119" s="138">
         <f>IF(NOT(ISNUMBER(F119)),"",F119*$D$45)</f>
       </c>
-      <c r="I119" s="119">
+      <c r="I119" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H119))),"",H119*$D$33)</f>
       </c>
-      <c r="J119">
+      <c r="J119" s="126">
         <f>IF($H$117&gt;0,1-H119/$H$117,0)</f>
       </c>
-      <c r="K119"/>
-      <c r="L119"/>
+      <c r="K119" s="123"/>
+      <c r="L119" s="123"/>
     </row>
     <row r="120" ht="20" customHeight="1">
       <c r="A120"/>
       <c r="B120"/>
-      <c r="C120" t="n">
+      <c r="C120" s="126" t="n">
         <v>0.5</v>
       </c>
-      <c r="D120" s="119">
+      <c r="D120" s="138">
         <f>$D$45*(1-C120)</f>
       </c>
-      <c r="E120" s="119">
+      <c r="E120" s="138">
         <f>$G$50/D120</f>
       </c>
-      <c r="F120">
+      <c r="F120" s="129">
         <f>IF(OR(D120="",E120=""),"",E120/D120)</f>
       </c>
-      <c r="G120">
+      <c r="G120" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F120))),"",F120*$D$33)</f>
       </c>
-      <c r="H120" s="119">
+      <c r="H120" s="138">
         <f>IF(NOT(ISNUMBER(F120)),"",F120*$D$45)</f>
       </c>
-      <c r="I120" s="119">
+      <c r="I120" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H120))),"",H120*$D$33)</f>
       </c>
-      <c r="J120">
+      <c r="J120" s="126">
         <f>IF($H$117&gt;0,1-H120/$H$117,0)</f>
       </c>
-      <c r="K120"/>
-      <c r="L120"/>
+      <c r="K120" s="123"/>
+      <c r="L120" s="123"/>
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121"/>
       <c r="B121"/>
-      <c r="C121" t="n">
+      <c r="C121" s="126" t="n">
         <v>0.4</v>
       </c>
-      <c r="D121" s="119">
+      <c r="D121" s="138">
         <f>$D$45*(1-C121)</f>
       </c>
-      <c r="E121" s="119">
+      <c r="E121" s="138">
         <f>$G$50/D121</f>
       </c>
-      <c r="F121">
+      <c r="F121" s="129">
         <f>IF(OR(D121="",E121=""),"",E121/D121)</f>
       </c>
-      <c r="G121">
+      <c r="G121" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F121))),"",F121*$D$33)</f>
       </c>
-      <c r="H121" s="119">
+      <c r="H121" s="138">
         <f>IF(NOT(ISNUMBER(F121)),"",F121*$D$45)</f>
       </c>
-      <c r="I121" s="119">
+      <c r="I121" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H121))),"",H121*$D$33)</f>
       </c>
-      <c r="J121">
+      <c r="J121" s="126">
         <f>IF($H$117&gt;0,1-H121/$H$117,0)</f>
       </c>
-      <c r="K121"/>
-      <c r="L121"/>
+      <c r="K121" s="123"/>
+      <c r="L121" s="123"/>
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122"/>
       <c r="B122"/>
-      <c r="C122" t="n">
+      <c r="C122" s="126" t="n">
         <v>0.3</v>
       </c>
-      <c r="D122" s="119">
+      <c r="D122" s="138">
         <f>$D$45*(1-C122)</f>
       </c>
-      <c r="E122" s="119">
+      <c r="E122" s="138">
         <f>$G$50/D122</f>
       </c>
-      <c r="F122">
+      <c r="F122" s="129">
         <f>IF(OR(D122="",E122=""),"",E122/D122)</f>
       </c>
-      <c r="G122">
+      <c r="G122" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F122))),"",F122*$D$33)</f>
       </c>
-      <c r="H122" s="119">
+      <c r="H122" s="138">
         <f>IF(NOT(ISNUMBER(F122)),"",F122*$D$45)</f>
       </c>
-      <c r="I122" s="119">
+      <c r="I122" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H122))),"",H122*$D$33)</f>
       </c>
-      <c r="J122">
+      <c r="J122" s="126">
         <f>IF($H$117&gt;0,1-H122/$H$117,0)</f>
       </c>
-      <c r="K122"/>
-      <c r="L122"/>
+      <c r="K122" s="123"/>
+      <c r="L122" s="123"/>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123"/>
       <c r="B123"/>
-      <c r="C123" t="n">
+      <c r="C123" s="126" t="n">
         <v>0.2</v>
       </c>
-      <c r="D123" s="119">
+      <c r="D123" s="138">
         <f>$D$45*(1-C123)</f>
       </c>
-      <c r="E123" s="119">
+      <c r="E123" s="138">
         <f>$G$50/D123</f>
       </c>
-      <c r="F123">
+      <c r="F123" s="129">
         <f>IF(OR(D123="",E123=""),"",E123/D123)</f>
       </c>
-      <c r="G123">
+      <c r="G123" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F123))),"",F123*$D$33)</f>
       </c>
-      <c r="H123" s="119">
+      <c r="H123" s="138">
         <f>IF(NOT(ISNUMBER(F123)),"",F123*$D$45)</f>
       </c>
-      <c r="I123" s="119">
+      <c r="I123" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H123))),"",H123*$D$33)</f>
       </c>
-      <c r="J123">
+      <c r="J123" s="126">
         <f>IF($H$117&gt;0,1-H123/$H$117,0)</f>
       </c>
-      <c r="K123"/>
-      <c r="L123"/>
+      <c r="K123" s="123"/>
+      <c r="L123" s="123"/>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124"/>
       <c r="B124"/>
-      <c r="C124" t="n">
+      <c r="C124" s="126" t="n">
         <v>0.1</v>
       </c>
-      <c r="D124" s="119">
+      <c r="D124" s="138">
         <f>$D$45*(1-C124)</f>
       </c>
-      <c r="E124" s="119">
+      <c r="E124" s="138">
         <f>$G$50/D124</f>
       </c>
-      <c r="F124">
+      <c r="F124" s="129">
         <f>IF(OR(D124="",E124=""),"",E124/D124)</f>
       </c>
-      <c r="G124">
+      <c r="G124" s="129">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F124))),"",F124*$D$33)</f>
       </c>
-      <c r="H124" s="119">
+      <c r="H124" s="138">
         <f>IF(NOT(ISNUMBER(F124)),"",F124*$D$45)</f>
       </c>
-      <c r="I124" s="119">
+      <c r="I124" s="138">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H124))),"",H124*$D$33)</f>
       </c>
-      <c r="J124">
+      <c r="J124" s="126">
         <f>IF($H$117&gt;0,1-H124/$H$117,0)</f>
       </c>
-      <c r="K124"/>
-      <c r="L124"/>
+      <c r="K124" s="123"/>
+      <c r="L124" s="123"/>
     </row>
     <row r="125" ht="20" customHeight="1">
       <c r="A125"/>
       <c r="B125"/>
-      <c r="C125" t="n">
+      <c r="C125" s="127" t="n">
         <v>0</v>
       </c>
-      <c r="D125" s="119">
+      <c r="D125" s="139">
         <f>$D$45*(1-C125)</f>
       </c>
-      <c r="E125" s="119">
+      <c r="E125" s="139">
         <f>$G$50/D125</f>
       </c>
-      <c r="F125">
+      <c r="F125" s="130">
         <f>IF(OR(D125="",E125=""),"",E125/D125)</f>
       </c>
-      <c r="G125">
+      <c r="G125" s="130">
         <f>IF(OR($D$33="",NOT(ISNUMBER(F125))),"",F125*$D$33)</f>
       </c>
-      <c r="H125" s="119">
+      <c r="H125" s="139">
         <f>IF(NOT(ISNUMBER(F125)),"",F125*$D$45)</f>
       </c>
-      <c r="I125" s="119">
+      <c r="I125" s="139">
         <f>IF(OR($D$33="",NOT(ISNUMBER(H125))),"",H125*$D$33)</f>
       </c>
-      <c r="J125">
+      <c r="J125" s="127">
         <f>IF($H$117&gt;0,1-H125/$H$117,0)</f>
       </c>
-      <c r="K125" t="str">
+      <c r="K125" s="124" t="str">
         <v>沉没成本 / Quote</v>
       </c>
-      <c r="L125">
+      <c r="L125" s="124">
         <f>E125</f>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126"/>
       <c r="B126"/>
-      <c r="C126"/>
-      <c r="D126"/>
-      <c r="E126"/>
-      <c r="F126"/>
-      <c r="G126"/>
-      <c r="H126"/>
-      <c r="I126"/>
-      <c r="J126"/>
-      <c r="K126"/>
-      <c r="L126"/>
+      <c r="C126" s="100"/>
+      <c r="D126" s="100"/>
+      <c r="E126" s="100"/>
+      <c r="F126" s="100"/>
+      <c r="G126" s="100"/>
+      <c r="H126" s="100"/>
+      <c r="I126" s="100"/>
+      <c r="J126" s="100"/>
+      <c r="K126" s="100"/>
+      <c r="L126" s="100"/>
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127"/>
       <c r="B127"/>
-      <c r="C127"/>
-      <c r="D127"/>
-      <c r="E127"/>
-      <c r="F127"/>
-      <c r="G127"/>
-      <c r="H127"/>
-      <c r="I127"/>
-      <c r="J127"/>
-      <c r="K127"/>
-      <c r="L127"/>
+      <c r="C127" s="100"/>
+      <c r="D127" s="100"/>
+      <c r="E127" s="100"/>
+      <c r="F127" s="100"/>
+      <c r="G127" s="100"/>
+      <c r="H127" s="100"/>
+      <c r="I127" s="100"/>
+      <c r="J127" s="100"/>
+      <c r="K127" s="100"/>
+      <c r="L127" s="100"/>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128"/>
       <c r="B128"/>
-      <c r="C128"/>
-      <c r="D128"/>
-      <c r="E128"/>
-      <c r="F128"/>
-      <c r="G128"/>
-      <c r="H128"/>
-      <c r="I128"/>
-      <c r="J128"/>
-      <c r="K128"/>
-      <c r="L128"/>
+      <c r="C128" s="100"/>
+      <c r="D128" s="100"/>
+      <c r="E128" s="100"/>
+      <c r="F128" s="100"/>
+      <c r="G128" s="100"/>
+      <c r="H128" s="100"/>
+      <c r="I128" s="100"/>
+      <c r="J128" s="100"/>
+      <c r="K128" s="100"/>
+      <c r="L128" s="100"/>
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129"/>
       <c r="B129"/>
-      <c r="C129"/>
-      <c r="D129"/>
-      <c r="E129"/>
-      <c r="F129"/>
-      <c r="G129"/>
-      <c r="H129"/>
-      <c r="I129"/>
-      <c r="J129"/>
-      <c r="K129"/>
-      <c r="L129"/>
+      <c r="C129" s="100"/>
+      <c r="D129" s="100"/>
+      <c r="E129" s="100"/>
+      <c r="F129" s="100"/>
+      <c r="G129" s="100"/>
+      <c r="H129" s="100"/>
+      <c r="I129" s="100"/>
+      <c r="J129" s="100"/>
+      <c r="K129" s="100"/>
+      <c r="L129" s="100"/>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130"/>
       <c r="B130"/>
-      <c r="C130"/>
-      <c r="D130"/>
-      <c r="E130"/>
-      <c r="F130"/>
-      <c r="G130"/>
-      <c r="H130"/>
-      <c r="I130"/>
-      <c r="J130"/>
-      <c r="K130"/>
-      <c r="L130"/>
+      <c r="C130" s="100"/>
+      <c r="D130" s="100"/>
+      <c r="E130" s="100"/>
+      <c r="F130" s="100"/>
+      <c r="G130" s="100"/>
+      <c r="H130" s="100"/>
+      <c r="I130" s="100"/>
+      <c r="J130" s="100"/>
+      <c r="K130" s="100"/>
+      <c r="L130" s="100"/>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131"/>
       <c r="B131"/>
-      <c r="C131"/>
-      <c r="D131"/>
-      <c r="E131"/>
-      <c r="F131"/>
-      <c r="G131"/>
-      <c r="H131"/>
-      <c r="I131"/>
-      <c r="J131"/>
-      <c r="K131"/>
-      <c r="L131"/>
+      <c r="C131" s="100"/>
+      <c r="D131" s="100"/>
+      <c r="E131" s="100"/>
+      <c r="F131" s="100"/>
+      <c r="G131" s="100"/>
+      <c r="H131" s="100"/>
+      <c r="I131" s="100"/>
+      <c r="J131" s="100"/>
+      <c r="K131" s="100"/>
+      <c r="L131" s="100"/>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132"/>
       <c r="B132"/>
-      <c r="C132"/>
-      <c r="D132"/>
-      <c r="E132"/>
-      <c r="F132"/>
-      <c r="G132"/>
-      <c r="H132"/>
-      <c r="I132"/>
-      <c r="J132"/>
-      <c r="K132"/>
-      <c r="L132"/>
+      <c r="C132" s="100"/>
+      <c r="D132" s="100"/>
+      <c r="E132" s="100"/>
+      <c r="F132" s="100"/>
+      <c r="G132" s="100"/>
+      <c r="H132" s="100"/>
+      <c r="I132" s="100"/>
+      <c r="J132" s="100"/>
+      <c r="K132" s="100"/>
+      <c r="L132" s="100"/>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133"/>
       <c r="B133"/>
-      <c r="C133"/>
-      <c r="D133"/>
-      <c r="E133"/>
-      <c r="F133"/>
-      <c r="G133"/>
-      <c r="H133"/>
-      <c r="I133"/>
-      <c r="J133"/>
-      <c r="K133"/>
-      <c r="L133"/>
+      <c r="C133" s="100"/>
+      <c r="D133" s="100"/>
+      <c r="E133" s="100"/>
+      <c r="F133" s="100"/>
+      <c r="G133" s="100"/>
+      <c r="H133" s="100"/>
+      <c r="I133" s="100"/>
+      <c r="J133" s="100"/>
+      <c r="K133" s="100"/>
+      <c r="L133" s="100"/>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134"/>
       <c r="B134"/>
-      <c r="C134"/>
-      <c r="D134"/>
-      <c r="E134"/>
-      <c r="F134"/>
-      <c r="G134"/>
-      <c r="H134"/>
-      <c r="I134"/>
-      <c r="J134"/>
-      <c r="K134"/>
-      <c r="L134"/>
+      <c r="C134" s="100"/>
+      <c r="D134" s="100"/>
+      <c r="E134" s="100"/>
+      <c r="F134" s="100"/>
+      <c r="G134" s="100"/>
+      <c r="H134" s="100"/>
+      <c r="I134" s="100"/>
+      <c r="J134" s="100"/>
+      <c r="K134" s="100"/>
+      <c r="L134" s="100"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135"/>
       <c r="B135"/>
-      <c r="C135"/>
-      <c r="D135"/>
-      <c r="E135"/>
-      <c r="F135"/>
-      <c r="G135"/>
-      <c r="H135"/>
-      <c r="I135"/>
-      <c r="J135"/>
-      <c r="K135"/>
-      <c r="L135"/>
+      <c r="C135" s="100"/>
+      <c r="D135" s="100"/>
+      <c r="E135" s="100"/>
+      <c r="F135" s="100"/>
+      <c r="G135" s="100"/>
+      <c r="H135" s="100"/>
+      <c r="I135" s="100"/>
+      <c r="J135" s="100"/>
+      <c r="K135" s="100"/>
+      <c r="L135" s="100"/>
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136"/>
       <c r="B136"/>
-      <c r="C136"/>
-      <c r="D136"/>
-      <c r="E136"/>
-      <c r="F136"/>
-      <c r="G136"/>
-      <c r="H136"/>
-      <c r="I136"/>
-      <c r="J136"/>
-      <c r="K136"/>
-      <c r="L136"/>
+      <c r="C136" s="100"/>
+      <c r="D136" s="100"/>
+      <c r="E136" s="100"/>
+      <c r="F136" s="100"/>
+      <c r="G136" s="100"/>
+      <c r="H136" s="100"/>
+      <c r="I136" s="100"/>
+      <c r="J136" s="100"/>
+      <c r="K136" s="100"/>
+      <c r="L136" s="100"/>
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137"/>
       <c r="B137"/>
-      <c r="C137"/>
-      <c r="D137"/>
-      <c r="E137"/>
-      <c r="F137"/>
-      <c r="G137"/>
-      <c r="H137"/>
-      <c r="I137"/>
-      <c r="J137"/>
-      <c r="K137"/>
-      <c r="L137"/>
+      <c r="C137" s="100"/>
+      <c r="D137" s="100"/>
+      <c r="E137" s="100"/>
+      <c r="F137" s="100"/>
+      <c r="G137" s="100"/>
+      <c r="H137" s="100"/>
+      <c r="I137" s="100"/>
+      <c r="J137" s="100"/>
+      <c r="K137" s="100"/>
+      <c r="L137" s="100"/>
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138"/>
       <c r="B138"/>
-      <c r="C138"/>
-      <c r="D138"/>
-      <c r="E138"/>
-      <c r="F138"/>
-      <c r="G138"/>
-      <c r="H138"/>
-      <c r="I138"/>
-      <c r="J138"/>
-      <c r="K138"/>
-      <c r="L138"/>
+      <c r="C138" s="100"/>
+      <c r="D138" s="100"/>
+      <c r="E138" s="100"/>
+      <c r="F138" s="100"/>
+      <c r="G138" s="100"/>
+      <c r="H138" s="100"/>
+      <c r="I138" s="100"/>
+      <c r="J138" s="100"/>
+      <c r="K138" s="100"/>
+      <c r="L138" s="100"/>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139"/>
       <c r="B139"/>
-      <c r="C139"/>
-      <c r="D139"/>
-      <c r="E139"/>
-      <c r="F139"/>
-      <c r="G139"/>
-      <c r="H139"/>
-      <c r="I139"/>
-      <c r="J139"/>
-      <c r="K139"/>
-      <c r="L139"/>
+      <c r="C139" s="100"/>
+      <c r="D139" s="100"/>
+      <c r="E139" s="100"/>
+      <c r="F139" s="100"/>
+      <c r="G139" s="100"/>
+      <c r="H139" s="100"/>
+      <c r="I139" s="100"/>
+      <c r="J139" s="100"/>
+      <c r="K139" s="100"/>
+      <c r="L139" s="100"/>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140"/>
       <c r="B140"/>
-      <c r="C140"/>
-      <c r="D140"/>
-      <c r="E140"/>
-      <c r="F140"/>
-      <c r="G140"/>
-      <c r="H140"/>
-      <c r="I140"/>
-      <c r="J140"/>
-      <c r="K140"/>
-      <c r="L140"/>
-    </row>
-    <row r="141">
+      <c r="C140" s="100"/>
+      <c r="D140" s="100"/>
+      <c r="E140" s="100"/>
+      <c r="F140" s="100"/>
+      <c r="G140" s="100"/>
+      <c r="H140" s="100"/>
+      <c r="I140" s="100"/>
+      <c r="J140" s="100"/>
+      <c r="K140" s="100"/>
+      <c r="L140" s="100"/>
+    </row>
+    <row r="141" ht="20" customHeight="1">
       <c r="A141"/>
       <c r="B141"/>
-      <c r="C141"/>
-      <c r="D141"/>
-      <c r="E141"/>
-      <c r="F141"/>
-      <c r="G141"/>
-      <c r="H141"/>
-      <c r="I141"/>
-      <c r="J141"/>
-      <c r="K141"/>
-      <c r="L141"/>
-    </row>
-    <row r="142">
+      <c r="C141" s="100"/>
+      <c r="D141" s="100"/>
+      <c r="E141" s="100"/>
+      <c r="F141" s="100"/>
+      <c r="G141" s="100"/>
+      <c r="H141" s="100"/>
+      <c r="I141" s="100"/>
+      <c r="J141" s="100"/>
+      <c r="K141" s="100"/>
+      <c r="L141" s="100"/>
+    </row>
+    <row r="142" ht="20" customHeight="1">
       <c r="A142"/>
       <c r="B142"/>
-      <c r="C142"/>
-      <c r="D142"/>
-      <c r="E142"/>
-      <c r="F142"/>
-      <c r="G142"/>
-      <c r="H142"/>
-      <c r="I142"/>
-      <c r="J142"/>
-      <c r="K142"/>
-      <c r="L142"/>
-    </row>
-    <row r="143">
+      <c r="C142" s="100"/>
+      <c r="D142" s="100"/>
+      <c r="E142" s="100"/>
+      <c r="F142" s="100"/>
+      <c r="G142" s="100"/>
+      <c r="H142" s="100"/>
+      <c r="I142" s="100"/>
+      <c r="J142" s="100"/>
+      <c r="K142" s="100"/>
+      <c r="L142" s="100"/>
+    </row>
+    <row r="143" ht="20" customHeight="1">
       <c r="A143"/>
       <c r="B143"/>
-      <c r="C143"/>
-      <c r="D143"/>
-      <c r="E143"/>
-      <c r="F143"/>
-      <c r="G143"/>
-      <c r="H143"/>
-      <c r="I143"/>
-      <c r="J143"/>
-      <c r="K143"/>
-      <c r="L143"/>
-    </row>
-    <row r="144">
+      <c r="C143" s="100"/>
+      <c r="D143" s="100"/>
+      <c r="E143" s="100"/>
+      <c r="F143" s="100"/>
+      <c r="G143" s="100"/>
+      <c r="H143" s="100"/>
+      <c r="I143" s="100"/>
+      <c r="J143" s="100"/>
+      <c r="K143" s="100"/>
+      <c r="L143" s="100"/>
+    </row>
+    <row r="144" ht="20" customHeight="1">
       <c r="A144"/>
       <c r="B144"/>
-      <c r="C144"/>
-      <c r="D144"/>
-      <c r="E144"/>
-      <c r="F144"/>
-      <c r="G144"/>
-      <c r="H144"/>
-      <c r="I144"/>
-      <c r="J144"/>
-      <c r="K144"/>
-      <c r="L144"/>
-    </row>
-    <row r="145">
+      <c r="C144" s="100"/>
+      <c r="D144" s="100"/>
+      <c r="E144" s="100"/>
+      <c r="F144" s="100"/>
+      <c r="G144" s="100"/>
+      <c r="H144" s="100"/>
+      <c r="I144" s="100"/>
+      <c r="J144" s="100"/>
+      <c r="K144" s="100"/>
+      <c r="L144" s="100"/>
+    </row>
+    <row r="145" ht="20" customHeight="1">
       <c r="A145"/>
       <c r="B145"/>
-      <c r="C145"/>
-      <c r="D145"/>
-      <c r="E145"/>
-      <c r="F145"/>
-      <c r="G145"/>
-      <c r="H145"/>
-      <c r="I145"/>
-      <c r="J145"/>
-      <c r="K145"/>
-      <c r="L145"/>
-    </row>
-    <row r="146">
+      <c r="C145" s="100"/>
+      <c r="D145" s="100"/>
+      <c r="E145" s="100"/>
+      <c r="F145" s="100"/>
+      <c r="G145" s="100"/>
+      <c r="H145" s="100"/>
+      <c r="I145" s="100"/>
+      <c r="J145" s="100"/>
+      <c r="K145" s="100"/>
+      <c r="L145" s="100"/>
+    </row>
+    <row r="146" ht="20" customHeight="1">
       <c r="A146"/>
       <c r="B146"/>
-      <c r="C146"/>
-      <c r="D146"/>
-      <c r="E146"/>
-      <c r="F146"/>
-      <c r="G146"/>
-      <c r="H146"/>
-      <c r="I146"/>
-      <c r="J146"/>
-      <c r="K146"/>
-      <c r="L146"/>
-    </row>
-    <row r="147">
+      <c r="C146" s="100"/>
+      <c r="D146" s="100"/>
+      <c r="E146" s="100"/>
+      <c r="F146" s="100"/>
+      <c r="G146" s="100"/>
+      <c r="H146" s="100"/>
+      <c r="I146" s="100"/>
+      <c r="J146" s="100"/>
+      <c r="K146" s="100"/>
+      <c r="L146" s="100"/>
+    </row>
+    <row r="147" ht="20" customHeight="1">
       <c r="A147"/>
       <c r="B147"/>
-      <c r="C147"/>
-      <c r="D147"/>
-      <c r="E147"/>
-      <c r="F147"/>
-      <c r="G147"/>
-      <c r="H147"/>
-      <c r="I147"/>
-      <c r="J147"/>
-      <c r="K147"/>
-      <c r="L147"/>
-    </row>
-    <row r="148">
+      <c r="C147" s="100"/>
+      <c r="D147" s="100"/>
+      <c r="E147" s="100"/>
+      <c r="F147" s="100"/>
+      <c r="G147" s="100"/>
+      <c r="H147" s="100"/>
+      <c r="I147" s="100"/>
+      <c r="J147" s="100"/>
+      <c r="K147" s="100"/>
+      <c r="L147" s="100"/>
+    </row>
+    <row r="148" ht="20" customHeight="1">
       <c r="A148"/>
       <c r="B148"/>
-      <c r="C148"/>
-      <c r="D148"/>
-      <c r="E148"/>
-      <c r="F148"/>
-      <c r="G148"/>
-      <c r="H148"/>
-      <c r="I148"/>
-      <c r="J148"/>
-      <c r="K148"/>
-      <c r="L148"/>
-    </row>
-    <row r="149">
+      <c r="C148" s="100"/>
+      <c r="D148" s="100"/>
+      <c r="E148" s="100"/>
+      <c r="F148" s="100"/>
+      <c r="G148" s="100"/>
+      <c r="H148" s="100"/>
+      <c r="I148" s="100"/>
+      <c r="J148" s="100"/>
+      <c r="K148" s="100"/>
+      <c r="L148" s="100"/>
+    </row>
+    <row r="149" ht="20" customHeight="1">
       <c r="A149"/>
       <c r="B149"/>
-      <c r="C149"/>
-      <c r="D149"/>
-      <c r="E149"/>
-      <c r="F149"/>
-      <c r="G149"/>
-      <c r="H149"/>
-      <c r="I149"/>
-      <c r="J149"/>
-      <c r="K149"/>
-      <c r="L149"/>
-    </row>
-    <row r="150">
+      <c r="C149" s="100"/>
+      <c r="D149" s="100"/>
+      <c r="E149" s="100"/>
+      <c r="F149" s="100"/>
+      <c r="G149" s="100"/>
+      <c r="H149" s="100"/>
+      <c r="I149" s="100"/>
+      <c r="J149" s="100"/>
+      <c r="K149" s="100"/>
+      <c r="L149" s="100"/>
+    </row>
+    <row r="150" ht="20" customHeight="1">
       <c r="A150"/>
       <c r="B150"/>
-      <c r="C150"/>
-      <c r="D150"/>
-      <c r="E150"/>
-      <c r="F150"/>
-      <c r="G150"/>
-      <c r="H150"/>
-      <c r="I150"/>
-      <c r="J150"/>
-      <c r="K150"/>
-      <c r="L150"/>
+      <c r="C150" s="100"/>
+      <c r="D150" s="100"/>
+      <c r="E150" s="100"/>
+      <c r="F150" s="100"/>
+      <c r="G150" s="100"/>
+      <c r="H150" s="100"/>
+      <c r="I150" s="100"/>
+      <c r="J150" s="100"/>
+      <c r="K150" s="100"/>
+      <c r="L150" s="100"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>

<commit_message>
Remove secondary metadata from Excel results panel
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Rb68aa64bfa934638"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R639d5daa445c4a97"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R2dcc5bc14b1644b1"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R38df040599604895"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="143">
+  <x:cellXfs count="145">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -584,12 +584,18 @@
     </x:xf>
     <x:xf numFmtId="208" fontId="11" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="23">
+  <x:dxfs count="27">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -722,6 +728,50 @@
     </x:dxf>
     <x:dxf>
       <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7D2638"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7D2638"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7D2638"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7D2638"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFDE8E7"/>
+        </x:patternFill>
+      </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
@@ -1246,7 +1296,7 @@
         <v>建议 Quote 资金</v>
       </c>
       <c r="D18" s="114">
-        <f>IF(ISNUMBER($D$26),(IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($D$22="","",SUM($D$22,$D$23,$D$24,$D$25))))+$D$26,"")</f>
+        <f>IF(ISNUMBER($D$26),(IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($D$22="","",SUM($D$22,$D$23,$D$24,$D$25))))+$D$26,"")</f>
       </c>
       <c r="E18" s="58">
         <f>$D$7</f>
@@ -1255,7 +1305,7 @@
         <v>原生币 Gas 储备</v>
       </c>
       <c r="G18" s="68">
-        <f>$D$32*MAX(0,$G$11)</f>
+        <f>$D$53*MAX(0,$G$11)</f>
       </c>
       <c r="H18" s="58" t="str">
         <v>BNB</v>
@@ -1278,7 +1328,7 @@
         <v>Quote 折算 / USDT</v>
       </c>
       <c r="D19" s="115">
-        <f>IF(ISNUMBER($D$18),IF($D$18=0,0,IF($D$33&gt;0,$D$18*$D$33,"")),"")</f>
+        <f>IF(ISNUMBER($D$18),IF($D$18=0,0,IF($D$55&gt;0,$D$18*$D$55,"")),"")</f>
       </c>
       <c r="E19" s="100" t="str">
         <v>USDT</v>
@@ -1296,7 +1346,7 @@
         <v>原生币价格 / USDT</v>
       </c>
       <c r="J19" s="116">
-        <f>IF($D$7="BNB",$D$33,IF('Quote参数'!$P$7&gt;0,'Quote参数'!$P$7,""))</f>
+        <f>IF($D$7="BNB",$D$55,IF('Quote参数'!$P$7&gt;0,'Quote参数'!$P$7,""))</f>
       </c>
       <c r="K19" s="100"/>
       <c r="L19" s="100"/>
@@ -1337,10 +1387,10 @@
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="100">
-        <f>"预算 "&amp;TEXT($D$31,"0%")&amp;" 理论资金"</f>
+        <f>"预算 "&amp;TEXT($D$52,"0%")&amp;" 理论资金"</f>
       </c>
       <c r="D22" s="115">
-        <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($J$45="","",$J$41+$J$45))</f>
+        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($J$45="","",$J$41+$J$45))</f>
       </c>
       <c r="E22" s="100">
         <f>$D$7</f>
@@ -1362,7 +1412,7 @@
         <v>额外内盘资金</v>
       </c>
       <c r="D23" s="115">
-        <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",$J$41*MAX(0,$G$7-1))</f>
+        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",$J$41*MAX(0,$G$7-1))</f>
       </c>
       <c r="E23" s="100">
         <f>$D$7</f>
@@ -1386,7 +1436,7 @@
         <v>洗筹损耗</v>
       </c>
       <c r="D24" s="115">
-        <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",IF($J$46="","",$J$46*$J$47))</f>
+        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($J$46="","",$J$46*$J$47))</f>
       </c>
       <c r="E24" s="100">
         <f>$D$7</f>
@@ -1434,7 +1484,7 @@
         <v>恢复目标控筹资金</v>
       </c>
       <c r="D26" s="115">
-        <f>IF(LEFT($D$30,2)&lt;&gt;"可达","",MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)))</f>
+        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)))</f>
       </c>
       <c r="E26" s="100">
         <f>$D$7</f>
@@ -1514,16 +1564,12 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="101" t="str">
-        <v>目标是否可达</v>
-      </c>
-      <c r="D30" s="101">
-        <f>IF($J$51&lt;&gt;"参数有效",$J$51,IF(OR($D$8&lt;80%,$D$8&gt;=100%),"目标控筹率无效",IF(OR($J$7&lt;0,$J$7&gt;10%,$J$8&lt;0,$J$8&gt;10%),"税率无效",IF($D$31&gt;=$G$32,"目标+1%不可达","可达"))))</f>
-      </c>
-      <c r="E30" s="100"/>
-      <c r="F30" s="100"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
       <c r="I30" s="101" t="str">
         <v>卖出含税费率</v>
       </c>
@@ -1533,97 +1579,71 @@
       <c r="K30" s="100"/>
       <c r="L30" s="100"/>
     </row>
-    <row r="31" ht="20" customHeight="1">
+    <row r="31" customHeight="1" hidden="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="101" t="str">
-        <v>预算使用控筹率</v>
-      </c>
-      <c r="D31" s="117">
-        <f>$D$8+1%</f>
-      </c>
-      <c r="E31" s="100"/>
-      <c r="F31" s="100"/>
-      <c r="G31" s="100"/>
-      <c r="H31" s="100"/>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31"/>
+      <c r="F31"/>
+      <c r="G31"/>
+      <c r="H31"/>
       <c r="I31" s="100"/>
       <c r="J31" s="100"/>
       <c r="K31" s="100"/>
       <c r="L31" s="100"/>
     </row>
-    <row r="32" ht="20" customHeight="1">
+    <row r="32" customHeight="1" hidden="1">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="101" t="str">
-        <v>地址总数</v>
-      </c>
-      <c r="D32" s="115">
-        <f>MAX(0,$G$8)*MAX(0,$G$7)+MAX(0,$G$9)+MAX(0,$G$10)</f>
-      </c>
-      <c r="E32" s="100"/>
-      <c r="F32" s="101" t="str">
-        <v>当前控筹上限</v>
-      </c>
-      <c r="G32" s="117">
-        <f>$G$43+(1-$J$7)*$G$48/1000000000</f>
-      </c>
-      <c r="H32" s="100"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="H32"/>
       <c r="I32" s="100"/>
       <c r="J32" s="100"/>
       <c r="K32" s="100"/>
       <c r="L32" s="100"/>
     </row>
-    <row r="33" ht="20" customHeight="1">
+    <row r="33" customHeight="1" hidden="1">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="101" t="str">
-        <v>Quote 价格 / USDT</v>
-      </c>
-      <c r="D33" s="116">
-        <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE),""))</f>
-      </c>
-      <c r="E33" s="100"/>
-      <c r="F33" s="100"/>
-      <c r="G33" s="100"/>
-      <c r="H33" s="100"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
       <c r="I33" s="100"/>
       <c r="J33" s="100"/>
       <c r="K33" s="100"/>
       <c r="L33" s="100"/>
     </row>
-    <row r="34" ht="20" customHeight="1">
+    <row r="34" customHeight="1" hidden="1">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="101" t="str">
-        <v>行情时间 / UTC</v>
-      </c>
-      <c r="D34" s="119">
-        <f>IF(VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE))</f>
-      </c>
-      <c r="E34" s="100"/>
-      <c r="F34" s="100"/>
-      <c r="G34" s="100"/>
-      <c r="H34" s="100"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
       <c r="I34" s="100"/>
       <c r="J34" s="100"/>
       <c r="K34" s="100"/>
       <c r="L34" s="100"/>
     </row>
-    <row r="35" ht="20" customHeight="1">
+    <row r="35" customHeight="1" hidden="1">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="101" t="str">
-        <v>价格采用方式</v>
-      </c>
-      <c r="D35" s="100">
-        <f>IF($D$9&lt;&gt;"","手动覆盖","每日行情")</f>
-      </c>
-      <c r="E35" s="100"/>
-      <c r="F35" s="101">
-        <f>IF($D$9&lt;&gt;"",IF($D$33="","手动价格无效","手动价格"),IF($D$33="","缺少价格","每日行情"))</f>
-      </c>
-      <c r="G35" s="101"/>
-      <c r="H35" s="101"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35"/>
+      <c r="F35"/>
+      <c r="G35"/>
+      <c r="H35"/>
       <c r="I35" s="100"/>
       <c r="J35" s="100"/>
       <c r="K35" s="100"/>
@@ -1914,7 +1934,7 @@
         <v>外盘净控筹 TOKEN</v>
       </c>
       <c r="J48" s="102">
-        <f>IF($D$31&lt;$G$32,MAX(0,($D$31-$G$43)*1000000000),"")</f>
+        <f>IF($D$52&lt;$D$54,MAX(0,($D$52-$G$43)*1000000000),"")</f>
       </c>
       <c r="K48" s="101"/>
       <c r="L48" s="101"/>
@@ -1966,8 +1986,12 @@
     <row r="51" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A51"/>
       <c r="B51"/>
-      <c r="C51" s="101"/>
-      <c r="D51" s="102"/>
+      <c r="C51" s="101" t="str">
+        <v>目标是否可达</v>
+      </c>
+      <c r="D51" s="102">
+        <f>IF($J$51&lt;&gt;"参数有效",$J$51,IF(OR($D$8&lt;80%,$D$8&gt;=100%),"目标控筹率无效",IF(OR($J$7&lt;0,$J$7&gt;10%,$J$8&lt;0,$J$8&gt;10%),"税率无效",IF($D$52&gt;=$D$54,"目标+1%不可达","可达"))))</f>
+      </c>
       <c r="E51" s="101"/>
       <c r="F51" s="101" t="str">
         <v>协议来源</v>
@@ -1988,8 +2012,12 @@
     <row r="52" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A52"/>
       <c r="B52"/>
-      <c r="C52" s="101"/>
-      <c r="D52" s="102"/>
+      <c r="C52" s="101" t="str">
+        <v>预算使用控筹率</v>
+      </c>
+      <c r="D52" s="143">
+        <f>$D$8+1%</f>
+      </c>
       <c r="E52" s="101"/>
       <c r="F52" s="101" t="str">
         <v>虚拟 TOKEN h</v>
@@ -2006,8 +2034,12 @@
     <row r="53" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A53"/>
       <c r="B53"/>
-      <c r="C53" s="101"/>
-      <c r="D53" s="102"/>
+      <c r="C53" s="101" t="str">
+        <v>地址总数</v>
+      </c>
+      <c r="D53" s="105">
+        <f>MAX(0,$G$8)*MAX(0,$G$7)+MAX(0,$G$9)+MAX(0,$G$10)</f>
+      </c>
       <c r="E53" s="101"/>
       <c r="F53" s="101" t="str">
         <v>买税方向</v>
@@ -2024,11 +2056,19 @@
     <row r="54" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A54"/>
       <c r="B54"/>
-      <c r="C54" s="101"/>
-      <c r="D54" s="102"/>
+      <c r="C54" s="101" t="str">
+        <v>当前控筹上限</v>
+      </c>
+      <c r="D54" s="143">
+        <f>$G$43+(1-$J$7)*$G$48/1000000000</f>
+      </c>
       <c r="E54" s="101"/>
-      <c r="F54" s="101"/>
-      <c r="G54" s="102"/>
+      <c r="F54" s="101" t="str">
+        <v>价格采用方式</v>
+      </c>
+      <c r="G54" s="102">
+        <f>IF($D$9&lt;&gt;"","手动覆盖","每日行情")</f>
+      </c>
       <c r="H54" s="101"/>
       <c r="I54" s="101" t="str">
         <v>洗后持仓保留比例</v>
@@ -2042,11 +2082,19 @@
     <row r="55" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A55"/>
       <c r="B55"/>
-      <c r="C55" s="101"/>
-      <c r="D55" s="102"/>
+      <c r="C55" s="101" t="str">
+        <v>Quote 价格 / USDT</v>
+      </c>
+      <c r="D55" s="102">
+        <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$14:$P$36,12,FALSE),""))</f>
+      </c>
       <c r="E55" s="101"/>
-      <c r="F55" s="101"/>
-      <c r="G55" s="102"/>
+      <c r="F55" s="101" t="str">
+        <v>价格状态</v>
+      </c>
+      <c r="G55" s="102">
+        <f>IF($D$9&lt;&gt;"",IF($D$55="","手动价格无效","手动价格"),IF($D$55="","缺少价格","每日行情"))</f>
+      </c>
       <c r="H55" s="101"/>
       <c r="I55" s="101" t="str">
         <v>目标外盘 Pool TOKEN</v>
@@ -2060,8 +2108,12 @@
     <row r="56" ht="30" customHeight="1" outlineLevel="1" hidden="1">
       <c r="A56"/>
       <c r="B56"/>
-      <c r="C56" s="101"/>
-      <c r="D56" s="102"/>
+      <c r="C56" s="101" t="str">
+        <v>行情时间 / UTC</v>
+      </c>
+      <c r="D56" s="144">
+        <f>IF(VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE))</f>
+      </c>
       <c r="E56" s="101"/>
       <c r="F56" s="101"/>
       <c r="G56" s="102"/>
@@ -2144,13 +2196,13 @@
         <f>IF(OR(D59="",E59=""),"",E59/D59)</f>
       </c>
       <c r="G59" s="128">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F59))),"",F59*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F59))),"",F59*$D$55)</f>
       </c>
       <c r="H59" s="137">
         <f>IF(NOT(ISNUMBER(F59)),"",F59*$D$45)</f>
       </c>
       <c r="I59" s="137">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H59))),"",H59*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H59))),"",H59*$D$55)</f>
       </c>
       <c r="J59" s="137">
         <f>0</f>
@@ -2178,13 +2230,13 @@
         <f>IF(OR(D60="",E60=""),"",E60/D60)</f>
       </c>
       <c r="G60" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F60))),"",F60*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F60))),"",F60*$D$55)</f>
       </c>
       <c r="H60" s="138">
         <f>IF(NOT(ISNUMBER(F60)),"",F60*$D$45)</f>
       </c>
       <c r="I60" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H60))),"",H60*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H60))),"",H60*$D$55)</f>
       </c>
       <c r="J60" s="138">
         <f>E60-E59</f>
@@ -2212,13 +2264,13 @@
         <f>IF(OR(D61="",E61=""),"",E61/D61)</f>
       </c>
       <c r="G61" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F61))),"",F61*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F61))),"",F61*$D$55)</f>
       </c>
       <c r="H61" s="138">
         <f>IF(NOT(ISNUMBER(F61)),"",F61*$D$45)</f>
       </c>
       <c r="I61" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H61))),"",H61*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H61))),"",H61*$D$55)</f>
       </c>
       <c r="J61" s="138">
         <f>E61-E60</f>
@@ -2246,13 +2298,13 @@
         <f>IF(OR(D62="",E62=""),"",E62/D62)</f>
       </c>
       <c r="G62" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F62))),"",F62*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F62))),"",F62*$D$55)</f>
       </c>
       <c r="H62" s="138">
         <f>IF(NOT(ISNUMBER(F62)),"",F62*$D$45)</f>
       </c>
       <c r="I62" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H62))),"",H62*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H62))),"",H62*$D$55)</f>
       </c>
       <c r="J62" s="138">
         <f>E62-E61</f>
@@ -2280,13 +2332,13 @@
         <f>IF(OR(D63="",E63=""),"",E63/D63)</f>
       </c>
       <c r="G63" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F63))),"",F63*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F63))),"",F63*$D$55)</f>
       </c>
       <c r="H63" s="138">
         <f>IF(NOT(ISNUMBER(F63)),"",F63*$D$45)</f>
       </c>
       <c r="I63" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H63))),"",H63*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H63))),"",H63*$D$55)</f>
       </c>
       <c r="J63" s="138">
         <f>E63-E62</f>
@@ -2314,13 +2366,13 @@
         <f>IF(OR(D64="",E64=""),"",E64/D64)</f>
       </c>
       <c r="G64" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F64))),"",F64*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F64))),"",F64*$D$55)</f>
       </c>
       <c r="H64" s="138">
         <f>IF(NOT(ISNUMBER(F64)),"",F64*$D$45)</f>
       </c>
       <c r="I64" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H64))),"",H64*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H64))),"",H64*$D$55)</f>
       </c>
       <c r="J64" s="138">
         <f>E64-E63</f>
@@ -2348,13 +2400,13 @@
         <f>IF(OR(D65="",E65=""),"",E65/D65)</f>
       </c>
       <c r="G65" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F65))),"",F65*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F65))),"",F65*$D$55)</f>
       </c>
       <c r="H65" s="138">
         <f>IF(NOT(ISNUMBER(F65)),"",F65*$D$45)</f>
       </c>
       <c r="I65" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H65))),"",H65*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H65))),"",H65*$D$55)</f>
       </c>
       <c r="J65" s="138">
         <f>E65-E64</f>
@@ -2382,13 +2434,13 @@
         <f>IF(OR(D66="",E66=""),"",E66/D66)</f>
       </c>
       <c r="G66" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F66))),"",F66*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F66))),"",F66*$D$55)</f>
       </c>
       <c r="H66" s="138">
         <f>IF(NOT(ISNUMBER(F66)),"",F66*$D$45)</f>
       </c>
       <c r="I66" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H66))),"",H66*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H66))),"",H66*$D$55)</f>
       </c>
       <c r="J66" s="138">
         <f>E66-E65</f>
@@ -2416,13 +2468,13 @@
         <f>IF(OR(D67="",E67=""),"",E67/D67)</f>
       </c>
       <c r="G67" s="130">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F67))),"",F67*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F67))),"",F67*$D$55)</f>
       </c>
       <c r="H67" s="139">
         <f>IF(NOT(ISNUMBER(F67)),"",F67*$D$45)</f>
       </c>
       <c r="I67" s="139">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H67))),"",H67*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H67))),"",H67*$D$55)</f>
       </c>
       <c r="J67" s="139">
         <f>E67-E66</f>
@@ -2531,13 +2583,13 @@
         <f>IF(OR(D72="",E72=""),"",E72/D72)</f>
       </c>
       <c r="G72" s="128">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F72))),"",F72*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F72))),"",F72*$D$55)</f>
       </c>
       <c r="H72" s="137">
         <f>IF(NOT(ISNUMBER(F72)),"",F72*$D$45)</f>
       </c>
       <c r="I72" s="137">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H72))),"",H72*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H72))),"",H72*$D$55)</f>
       </c>
       <c r="J72" s="137">
         <f>0</f>
@@ -2556,7 +2608,7 @@
         <v>0.805</v>
       </c>
       <c r="D73" s="138">
-        <f>IF(C73&lt;$G$32,$G$48-MAX(0,(C73-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C73&lt;$D$54,$G$48-MAX(0,(C73-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E73" s="138">
         <f>IF(D73="","",$G$50/D73)</f>
@@ -2565,13 +2617,13 @@
         <f>IF(OR(D73="",E73=""),"",E73/D73)</f>
       </c>
       <c r="G73" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F73))),"",F73*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F73))),"",F73*$D$55)</f>
       </c>
       <c r="H73" s="138">
         <f>IF(NOT(ISNUMBER(F73)),"",F73*$D$45)</f>
       </c>
       <c r="I73" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H73))),"",H73*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H73))),"",H73*$D$55)</f>
       </c>
       <c r="J73" s="138">
         <f>IF(E73="","",MAX(0,E73-$G$44))</f>
@@ -2590,7 +2642,7 @@
         <v>0.81</v>
       </c>
       <c r="D74" s="138">
-        <f>IF(C74&lt;$G$32,$G$48-MAX(0,(C74-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C74&lt;$D$54,$G$48-MAX(0,(C74-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E74" s="138">
         <f>IF(D74="","",$G$50/D74)</f>
@@ -2599,13 +2651,13 @@
         <f>IF(OR(D74="",E74=""),"",E74/D74)</f>
       </c>
       <c r="G74" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F74))),"",F74*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F74))),"",F74*$D$55)</f>
       </c>
       <c r="H74" s="138">
         <f>IF(NOT(ISNUMBER(F74)),"",F74*$D$45)</f>
       </c>
       <c r="I74" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H74))),"",H74*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H74))),"",H74*$D$55)</f>
       </c>
       <c r="J74" s="138">
         <f>IF(E74="","",MAX(0,E74-$G$44))</f>
@@ -2624,7 +2676,7 @@
         <v>0.8150000000000001</v>
       </c>
       <c r="D75" s="138">
-        <f>IF(C75&lt;$G$32,$G$48-MAX(0,(C75-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C75&lt;$D$54,$G$48-MAX(0,(C75-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E75" s="138">
         <f>IF(D75="","",$G$50/D75)</f>
@@ -2633,13 +2685,13 @@
         <f>IF(OR(D75="",E75=""),"",E75/D75)</f>
       </c>
       <c r="G75" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F75))),"",F75*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F75))),"",F75*$D$55)</f>
       </c>
       <c r="H75" s="138">
         <f>IF(NOT(ISNUMBER(F75)),"",F75*$D$45)</f>
       </c>
       <c r="I75" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H75))),"",H75*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H75))),"",H75*$D$55)</f>
       </c>
       <c r="J75" s="138">
         <f>IF(E75="","",MAX(0,E75-$G$44))</f>
@@ -2658,7 +2710,7 @@
         <v>0.8200000000000001</v>
       </c>
       <c r="D76" s="138">
-        <f>IF(C76&lt;$G$32,$G$48-MAX(0,(C76-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C76&lt;$D$54,$G$48-MAX(0,(C76-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E76" s="138">
         <f>IF(D76="","",$G$50/D76)</f>
@@ -2667,13 +2719,13 @@
         <f>IF(OR(D76="",E76=""),"",E76/D76)</f>
       </c>
       <c r="G76" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F76))),"",F76*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F76))),"",F76*$D$55)</f>
       </c>
       <c r="H76" s="138">
         <f>IF(NOT(ISNUMBER(F76)),"",F76*$D$45)</f>
       </c>
       <c r="I76" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H76))),"",H76*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H76))),"",H76*$D$55)</f>
       </c>
       <c r="J76" s="138">
         <f>IF(E76="","",MAX(0,E76-$G$44))</f>
@@ -2692,7 +2744,7 @@
         <v>0.8250000000000001</v>
       </c>
       <c r="D77" s="138">
-        <f>IF(C77&lt;$G$32,$G$48-MAX(0,(C77-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C77&lt;$D$54,$G$48-MAX(0,(C77-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E77" s="138">
         <f>IF(D77="","",$G$50/D77)</f>
@@ -2701,13 +2753,13 @@
         <f>IF(OR(D77="",E77=""),"",E77/D77)</f>
       </c>
       <c r="G77" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F77))),"",F77*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F77))),"",F77*$D$55)</f>
       </c>
       <c r="H77" s="138">
         <f>IF(NOT(ISNUMBER(F77)),"",F77*$D$45)</f>
       </c>
       <c r="I77" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H77))),"",H77*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H77))),"",H77*$D$55)</f>
       </c>
       <c r="J77" s="138">
         <f>IF(E77="","",MAX(0,E77-$G$44))</f>
@@ -2726,7 +2778,7 @@
         <v>0.8300000000000001</v>
       </c>
       <c r="D78" s="138">
-        <f>IF(C78&lt;$G$32,$G$48-MAX(0,(C78-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C78&lt;$D$54,$G$48-MAX(0,(C78-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E78" s="138">
         <f>IF(D78="","",$G$50/D78)</f>
@@ -2735,13 +2787,13 @@
         <f>IF(OR(D78="",E78=""),"",E78/D78)</f>
       </c>
       <c r="G78" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F78))),"",F78*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F78))),"",F78*$D$55)</f>
       </c>
       <c r="H78" s="138">
         <f>IF(NOT(ISNUMBER(F78)),"",F78*$D$45)</f>
       </c>
       <c r="I78" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H78))),"",H78*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H78))),"",H78*$D$55)</f>
       </c>
       <c r="J78" s="138">
         <f>IF(E78="","",MAX(0,E78-$G$44))</f>
@@ -2760,7 +2812,7 @@
         <v>0.8350000000000001</v>
       </c>
       <c r="D79" s="138">
-        <f>IF(C79&lt;$G$32,$G$48-MAX(0,(C79-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C79&lt;$D$54,$G$48-MAX(0,(C79-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E79" s="138">
         <f>IF(D79="","",$G$50/D79)</f>
@@ -2769,13 +2821,13 @@
         <f>IF(OR(D79="",E79=""),"",E79/D79)</f>
       </c>
       <c r="G79" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F79))),"",F79*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F79))),"",F79*$D$55)</f>
       </c>
       <c r="H79" s="138">
         <f>IF(NOT(ISNUMBER(F79)),"",F79*$D$45)</f>
       </c>
       <c r="I79" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H79))),"",H79*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H79))),"",H79*$D$55)</f>
       </c>
       <c r="J79" s="138">
         <f>IF(E79="","",MAX(0,E79-$G$44))</f>
@@ -2794,7 +2846,7 @@
         <v>0.8400000000000001</v>
       </c>
       <c r="D80" s="138">
-        <f>IF(C80&lt;$G$32,$G$48-MAX(0,(C80-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C80&lt;$D$54,$G$48-MAX(0,(C80-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E80" s="138">
         <f>IF(D80="","",$G$50/D80)</f>
@@ -2803,13 +2855,13 @@
         <f>IF(OR(D80="",E80=""),"",E80/D80)</f>
       </c>
       <c r="G80" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F80))),"",F80*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F80))),"",F80*$D$55)</f>
       </c>
       <c r="H80" s="138">
         <f>IF(NOT(ISNUMBER(F80)),"",F80*$D$45)</f>
       </c>
       <c r="I80" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H80))),"",H80*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H80))),"",H80*$D$55)</f>
       </c>
       <c r="J80" s="138">
         <f>IF(E80="","",MAX(0,E80-$G$44))</f>
@@ -2828,7 +2880,7 @@
         <v>0.8450000000000001</v>
       </c>
       <c r="D81" s="138">
-        <f>IF(C81&lt;$G$32,$G$48-MAX(0,(C81-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C81&lt;$D$54,$G$48-MAX(0,(C81-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E81" s="138">
         <f>IF(D81="","",$G$50/D81)</f>
@@ -2837,13 +2889,13 @@
         <f>IF(OR(D81="",E81=""),"",E81/D81)</f>
       </c>
       <c r="G81" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F81))),"",F81*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F81))),"",F81*$D$55)</f>
       </c>
       <c r="H81" s="138">
         <f>IF(NOT(ISNUMBER(F81)),"",F81*$D$45)</f>
       </c>
       <c r="I81" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H81))),"",H81*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H81))),"",H81*$D$55)</f>
       </c>
       <c r="J81" s="138">
         <f>IF(E81="","",MAX(0,E81-$G$44))</f>
@@ -2862,7 +2914,7 @@
         <v>0.8500000000000001</v>
       </c>
       <c r="D82" s="138">
-        <f>IF(C82&lt;$G$32,$G$48-MAX(0,(C82-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C82&lt;$D$54,$G$48-MAX(0,(C82-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E82" s="138">
         <f>IF(D82="","",$G$50/D82)</f>
@@ -2871,13 +2923,13 @@
         <f>IF(OR(D82="",E82=""),"",E82/D82)</f>
       </c>
       <c r="G82" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F82))),"",F82*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F82))),"",F82*$D$55)</f>
       </c>
       <c r="H82" s="138">
         <f>IF(NOT(ISNUMBER(F82)),"",F82*$D$45)</f>
       </c>
       <c r="I82" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H82))),"",H82*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H82))),"",H82*$D$55)</f>
       </c>
       <c r="J82" s="138">
         <f>IF(E82="","",MAX(0,E82-$G$44))</f>
@@ -2896,7 +2948,7 @@
         <v>0.8550000000000001</v>
       </c>
       <c r="D83" s="138">
-        <f>IF(C83&lt;$G$32,$G$48-MAX(0,(C83-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C83&lt;$D$54,$G$48-MAX(0,(C83-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E83" s="138">
         <f>IF(D83="","",$G$50/D83)</f>
@@ -2905,13 +2957,13 @@
         <f>IF(OR(D83="",E83=""),"",E83/D83)</f>
       </c>
       <c r="G83" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F83))),"",F83*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F83))),"",F83*$D$55)</f>
       </c>
       <c r="H83" s="138">
         <f>IF(NOT(ISNUMBER(F83)),"",F83*$D$45)</f>
       </c>
       <c r="I83" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H83))),"",H83*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H83))),"",H83*$D$55)</f>
       </c>
       <c r="J83" s="138">
         <f>IF(E83="","",MAX(0,E83-$G$44))</f>
@@ -2930,7 +2982,7 @@
         <v>0.8600000000000001</v>
       </c>
       <c r="D84" s="138">
-        <f>IF(C84&lt;$G$32,$G$48-MAX(0,(C84-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C84&lt;$D$54,$G$48-MAX(0,(C84-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E84" s="138">
         <f>IF(D84="","",$G$50/D84)</f>
@@ -2939,13 +2991,13 @@
         <f>IF(OR(D84="",E84=""),"",E84/D84)</f>
       </c>
       <c r="G84" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F84))),"",F84*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F84))),"",F84*$D$55)</f>
       </c>
       <c r="H84" s="138">
         <f>IF(NOT(ISNUMBER(F84)),"",F84*$D$45)</f>
       </c>
       <c r="I84" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H84))),"",H84*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H84))),"",H84*$D$55)</f>
       </c>
       <c r="J84" s="138">
         <f>IF(E84="","",MAX(0,E84-$G$44))</f>
@@ -2964,7 +3016,7 @@
         <v>0.865</v>
       </c>
       <c r="D85" s="138">
-        <f>IF(C85&lt;$G$32,$G$48-MAX(0,(C85-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C85&lt;$D$54,$G$48-MAX(0,(C85-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E85" s="138">
         <f>IF(D85="","",$G$50/D85)</f>
@@ -2973,13 +3025,13 @@
         <f>IF(OR(D85="",E85=""),"",E85/D85)</f>
       </c>
       <c r="G85" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F85))),"",F85*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F85))),"",F85*$D$55)</f>
       </c>
       <c r="H85" s="138">
         <f>IF(NOT(ISNUMBER(F85)),"",F85*$D$45)</f>
       </c>
       <c r="I85" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H85))),"",H85*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H85))),"",H85*$D$55)</f>
       </c>
       <c r="J85" s="138">
         <f>IF(E85="","",MAX(0,E85-$G$44))</f>
@@ -2998,7 +3050,7 @@
         <v>0.8700000000000001</v>
       </c>
       <c r="D86" s="138">
-        <f>IF(C86&lt;$G$32,$G$48-MAX(0,(C86-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C86&lt;$D$54,$G$48-MAX(0,(C86-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E86" s="138">
         <f>IF(D86="","",$G$50/D86)</f>
@@ -3007,13 +3059,13 @@
         <f>IF(OR(D86="",E86=""),"",E86/D86)</f>
       </c>
       <c r="G86" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F86))),"",F86*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F86))),"",F86*$D$55)</f>
       </c>
       <c r="H86" s="138">
         <f>IF(NOT(ISNUMBER(F86)),"",F86*$D$45)</f>
       </c>
       <c r="I86" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H86))),"",H86*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H86))),"",H86*$D$55)</f>
       </c>
       <c r="J86" s="138">
         <f>IF(E86="","",MAX(0,E86-$G$44))</f>
@@ -3032,7 +3084,7 @@
         <v>0.875</v>
       </c>
       <c r="D87" s="138">
-        <f>IF(C87&lt;$G$32,$G$48-MAX(0,(C87-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C87&lt;$D$54,$G$48-MAX(0,(C87-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E87" s="138">
         <f>IF(D87="","",$G$50/D87)</f>
@@ -3041,13 +3093,13 @@
         <f>IF(OR(D87="",E87=""),"",E87/D87)</f>
       </c>
       <c r="G87" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F87))),"",F87*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F87))),"",F87*$D$55)</f>
       </c>
       <c r="H87" s="138">
         <f>IF(NOT(ISNUMBER(F87)),"",F87*$D$45)</f>
       </c>
       <c r="I87" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H87))),"",H87*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H87))),"",H87*$D$55)</f>
       </c>
       <c r="J87" s="138">
         <f>IF(E87="","",MAX(0,E87-$G$44))</f>
@@ -3066,7 +3118,7 @@
         <v>0.88</v>
       </c>
       <c r="D88" s="138">
-        <f>IF(C88&lt;$G$32,$G$48-MAX(0,(C88-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C88&lt;$D$54,$G$48-MAX(0,(C88-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E88" s="138">
         <f>IF(D88="","",$G$50/D88)</f>
@@ -3075,13 +3127,13 @@
         <f>IF(OR(D88="",E88=""),"",E88/D88)</f>
       </c>
       <c r="G88" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F88))),"",F88*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F88))),"",F88*$D$55)</f>
       </c>
       <c r="H88" s="138">
         <f>IF(NOT(ISNUMBER(F88)),"",F88*$D$45)</f>
       </c>
       <c r="I88" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H88))),"",H88*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H88))),"",H88*$D$55)</f>
       </c>
       <c r="J88" s="138">
         <f>IF(E88="","",MAX(0,E88-$G$44))</f>
@@ -3100,7 +3152,7 @@
         <v>0.885</v>
       </c>
       <c r="D89" s="138">
-        <f>IF(C89&lt;$G$32,$G$48-MAX(0,(C89-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C89&lt;$D$54,$G$48-MAX(0,(C89-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E89" s="138">
         <f>IF(D89="","",$G$50/D89)</f>
@@ -3109,13 +3161,13 @@
         <f>IF(OR(D89="",E89=""),"",E89/D89)</f>
       </c>
       <c r="G89" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F89))),"",F89*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F89))),"",F89*$D$55)</f>
       </c>
       <c r="H89" s="138">
         <f>IF(NOT(ISNUMBER(F89)),"",F89*$D$45)</f>
       </c>
       <c r="I89" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H89))),"",H89*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H89))),"",H89*$D$55)</f>
       </c>
       <c r="J89" s="138">
         <f>IF(E89="","",MAX(0,E89-$G$44))</f>
@@ -3134,7 +3186,7 @@
         <v>0.89</v>
       </c>
       <c r="D90" s="138">
-        <f>IF(C90&lt;$G$32,$G$48-MAX(0,(C90-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C90&lt;$D$54,$G$48-MAX(0,(C90-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E90" s="138">
         <f>IF(D90="","",$G$50/D90)</f>
@@ -3143,13 +3195,13 @@
         <f>IF(OR(D90="",E90=""),"",E90/D90)</f>
       </c>
       <c r="G90" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F90))),"",F90*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F90))),"",F90*$D$55)</f>
       </c>
       <c r="H90" s="138">
         <f>IF(NOT(ISNUMBER(F90)),"",F90*$D$45)</f>
       </c>
       <c r="I90" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H90))),"",H90*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H90))),"",H90*$D$55)</f>
       </c>
       <c r="J90" s="138">
         <f>IF(E90="","",MAX(0,E90-$G$44))</f>
@@ -3168,7 +3220,7 @@
         <v>0.895</v>
       </c>
       <c r="D91" s="138">
-        <f>IF(C91&lt;$G$32,$G$48-MAX(0,(C91-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C91&lt;$D$54,$G$48-MAX(0,(C91-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E91" s="138">
         <f>IF(D91="","",$G$50/D91)</f>
@@ -3177,13 +3229,13 @@
         <f>IF(OR(D91="",E91=""),"",E91/D91)</f>
       </c>
       <c r="G91" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F91))),"",F91*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F91))),"",F91*$D$55)</f>
       </c>
       <c r="H91" s="138">
         <f>IF(NOT(ISNUMBER(F91)),"",F91*$D$45)</f>
       </c>
       <c r="I91" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H91))),"",H91*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H91))),"",H91*$D$55)</f>
       </c>
       <c r="J91" s="138">
         <f>IF(E91="","",MAX(0,E91-$G$44))</f>
@@ -3202,7 +3254,7 @@
         <v>0.9</v>
       </c>
       <c r="D92" s="138">
-        <f>IF(C92&lt;$G$32,$G$48-MAX(0,(C92-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C92&lt;$D$54,$G$48-MAX(0,(C92-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E92" s="138">
         <f>IF(D92="","",$G$50/D92)</f>
@@ -3211,13 +3263,13 @@
         <f>IF(OR(D92="",E92=""),"",E92/D92)</f>
       </c>
       <c r="G92" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F92))),"",F92*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F92))),"",F92*$D$55)</f>
       </c>
       <c r="H92" s="138">
         <f>IF(NOT(ISNUMBER(F92)),"",F92*$D$45)</f>
       </c>
       <c r="I92" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H92))),"",H92*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H92))),"",H92*$D$55)</f>
       </c>
       <c r="J92" s="138">
         <f>IF(E92="","",MAX(0,E92-$G$44))</f>
@@ -3236,7 +3288,7 @@
         <v>0.905</v>
       </c>
       <c r="D93" s="138">
-        <f>IF(C93&lt;$G$32,$G$48-MAX(0,(C93-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C93&lt;$D$54,$G$48-MAX(0,(C93-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E93" s="138">
         <f>IF(D93="","",$G$50/D93)</f>
@@ -3245,13 +3297,13 @@
         <f>IF(OR(D93="",E93=""),"",E93/D93)</f>
       </c>
       <c r="G93" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F93))),"",F93*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F93))),"",F93*$D$55)</f>
       </c>
       <c r="H93" s="138">
         <f>IF(NOT(ISNUMBER(F93)),"",F93*$D$45)</f>
       </c>
       <c r="I93" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H93))),"",H93*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H93))),"",H93*$D$55)</f>
       </c>
       <c r="J93" s="138">
         <f>IF(E93="","",MAX(0,E93-$G$44))</f>
@@ -3270,7 +3322,7 @@
         <v>0.91</v>
       </c>
       <c r="D94" s="138">
-        <f>IF(C94&lt;$G$32,$G$48-MAX(0,(C94-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C94&lt;$D$54,$G$48-MAX(0,(C94-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E94" s="138">
         <f>IF(D94="","",$G$50/D94)</f>
@@ -3279,13 +3331,13 @@
         <f>IF(OR(D94="",E94=""),"",E94/D94)</f>
       </c>
       <c r="G94" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F94))),"",F94*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F94))),"",F94*$D$55)</f>
       </c>
       <c r="H94" s="138">
         <f>IF(NOT(ISNUMBER(F94)),"",F94*$D$45)</f>
       </c>
       <c r="I94" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H94))),"",H94*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H94))),"",H94*$D$55)</f>
       </c>
       <c r="J94" s="138">
         <f>IF(E94="","",MAX(0,E94-$G$44))</f>
@@ -3304,7 +3356,7 @@
         <v>0.915</v>
       </c>
       <c r="D95" s="138">
-        <f>IF(C95&lt;$G$32,$G$48-MAX(0,(C95-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C95&lt;$D$54,$G$48-MAX(0,(C95-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E95" s="138">
         <f>IF(D95="","",$G$50/D95)</f>
@@ -3313,13 +3365,13 @@
         <f>IF(OR(D95="",E95=""),"",E95/D95)</f>
       </c>
       <c r="G95" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F95))),"",F95*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F95))),"",F95*$D$55)</f>
       </c>
       <c r="H95" s="138">
         <f>IF(NOT(ISNUMBER(F95)),"",F95*$D$45)</f>
       </c>
       <c r="I95" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H95))),"",H95*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H95))),"",H95*$D$55)</f>
       </c>
       <c r="J95" s="138">
         <f>IF(E95="","",MAX(0,E95-$G$44))</f>
@@ -3338,7 +3390,7 @@
         <v>0.92</v>
       </c>
       <c r="D96" s="138">
-        <f>IF(C96&lt;$G$32,$G$48-MAX(0,(C96-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C96&lt;$D$54,$G$48-MAX(0,(C96-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E96" s="138">
         <f>IF(D96="","",$G$50/D96)</f>
@@ -3347,13 +3399,13 @@
         <f>IF(OR(D96="",E96=""),"",E96/D96)</f>
       </c>
       <c r="G96" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F96))),"",F96*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F96))),"",F96*$D$55)</f>
       </c>
       <c r="H96" s="138">
         <f>IF(NOT(ISNUMBER(F96)),"",F96*$D$45)</f>
       </c>
       <c r="I96" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H96))),"",H96*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H96))),"",H96*$D$55)</f>
       </c>
       <c r="J96" s="138">
         <f>IF(E96="","",MAX(0,E96-$G$44))</f>
@@ -3372,7 +3424,7 @@
         <v>0.925</v>
       </c>
       <c r="D97" s="138">
-        <f>IF(C97&lt;$G$32,$G$48-MAX(0,(C97-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C97&lt;$D$54,$G$48-MAX(0,(C97-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E97" s="138">
         <f>IF(D97="","",$G$50/D97)</f>
@@ -3381,13 +3433,13 @@
         <f>IF(OR(D97="",E97=""),"",E97/D97)</f>
       </c>
       <c r="G97" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F97))),"",F97*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F97))),"",F97*$D$55)</f>
       </c>
       <c r="H97" s="138">
         <f>IF(NOT(ISNUMBER(F97)),"",F97*$D$45)</f>
       </c>
       <c r="I97" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H97))),"",H97*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H97))),"",H97*$D$55)</f>
       </c>
       <c r="J97" s="138">
         <f>IF(E97="","",MAX(0,E97-$G$44))</f>
@@ -3406,7 +3458,7 @@
         <v>0.93</v>
       </c>
       <c r="D98" s="138">
-        <f>IF(C98&lt;$G$32,$G$48-MAX(0,(C98-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C98&lt;$D$54,$G$48-MAX(0,(C98-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E98" s="138">
         <f>IF(D98="","",$G$50/D98)</f>
@@ -3415,13 +3467,13 @@
         <f>IF(OR(D98="",E98=""),"",E98/D98)</f>
       </c>
       <c r="G98" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F98))),"",F98*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F98))),"",F98*$D$55)</f>
       </c>
       <c r="H98" s="138">
         <f>IF(NOT(ISNUMBER(F98)),"",F98*$D$45)</f>
       </c>
       <c r="I98" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H98))),"",H98*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H98))),"",H98*$D$55)</f>
       </c>
       <c r="J98" s="138">
         <f>IF(E98="","",MAX(0,E98-$G$44))</f>
@@ -3440,7 +3492,7 @@
         <v>0.935</v>
       </c>
       <c r="D99" s="138">
-        <f>IF(C99&lt;$G$32,$G$48-MAX(0,(C99-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C99&lt;$D$54,$G$48-MAX(0,(C99-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E99" s="138">
         <f>IF(D99="","",$G$50/D99)</f>
@@ -3449,13 +3501,13 @@
         <f>IF(OR(D99="",E99=""),"",E99/D99)</f>
       </c>
       <c r="G99" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F99))),"",F99*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F99))),"",F99*$D$55)</f>
       </c>
       <c r="H99" s="138">
         <f>IF(NOT(ISNUMBER(F99)),"",F99*$D$45)</f>
       </c>
       <c r="I99" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H99))),"",H99*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H99))),"",H99*$D$55)</f>
       </c>
       <c r="J99" s="138">
         <f>IF(E99="","",MAX(0,E99-$G$44))</f>
@@ -3474,7 +3526,7 @@
         <v>0.9400000000000001</v>
       </c>
       <c r="D100" s="138">
-        <f>IF(C100&lt;$G$32,$G$48-MAX(0,(C100-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C100&lt;$D$54,$G$48-MAX(0,(C100-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E100" s="138">
         <f>IF(D100="","",$G$50/D100)</f>
@@ -3483,13 +3535,13 @@
         <f>IF(OR(D100="",E100=""),"",E100/D100)</f>
       </c>
       <c r="G100" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F100))),"",F100*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F100))),"",F100*$D$55)</f>
       </c>
       <c r="H100" s="138">
         <f>IF(NOT(ISNUMBER(F100)),"",F100*$D$45)</f>
       </c>
       <c r="I100" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H100))),"",H100*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H100))),"",H100*$D$55)</f>
       </c>
       <c r="J100" s="138">
         <f>IF(E100="","",MAX(0,E100-$G$44))</f>
@@ -3508,7 +3560,7 @@
         <v>0.9450000000000001</v>
       </c>
       <c r="D101" s="138">
-        <f>IF(C101&lt;$G$32,$G$48-MAX(0,(C101-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C101&lt;$D$54,$G$48-MAX(0,(C101-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E101" s="138">
         <f>IF(D101="","",$G$50/D101)</f>
@@ -3517,13 +3569,13 @@
         <f>IF(OR(D101="",E101=""),"",E101/D101)</f>
       </c>
       <c r="G101" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F101))),"",F101*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F101))),"",F101*$D$55)</f>
       </c>
       <c r="H101" s="138">
         <f>IF(NOT(ISNUMBER(F101)),"",F101*$D$45)</f>
       </c>
       <c r="I101" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H101))),"",H101*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H101))),"",H101*$D$55)</f>
       </c>
       <c r="J101" s="138">
         <f>IF(E101="","",MAX(0,E101-$G$44))</f>
@@ -3542,7 +3594,7 @@
         <v>0.9500000000000001</v>
       </c>
       <c r="D102" s="138">
-        <f>IF(C102&lt;$G$32,$G$48-MAX(0,(C102-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C102&lt;$D$54,$G$48-MAX(0,(C102-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E102" s="138">
         <f>IF(D102="","",$G$50/D102)</f>
@@ -3551,13 +3603,13 @@
         <f>IF(OR(D102="",E102=""),"",E102/D102)</f>
       </c>
       <c r="G102" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F102))),"",F102*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F102))),"",F102*$D$55)</f>
       </c>
       <c r="H102" s="138">
         <f>IF(NOT(ISNUMBER(F102)),"",F102*$D$45)</f>
       </c>
       <c r="I102" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H102))),"",H102*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H102))),"",H102*$D$55)</f>
       </c>
       <c r="J102" s="138">
         <f>IF(E102="","",MAX(0,E102-$G$44))</f>
@@ -3576,7 +3628,7 @@
         <v>0.9550000000000001</v>
       </c>
       <c r="D103" s="138">
-        <f>IF(C103&lt;$G$32,$G$48-MAX(0,(C103-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C103&lt;$D$54,$G$48-MAX(0,(C103-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E103" s="138">
         <f>IF(D103="","",$G$50/D103)</f>
@@ -3585,13 +3637,13 @@
         <f>IF(OR(D103="",E103=""),"",E103/D103)</f>
       </c>
       <c r="G103" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F103))),"",F103*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F103))),"",F103*$D$55)</f>
       </c>
       <c r="H103" s="138">
         <f>IF(NOT(ISNUMBER(F103)),"",F103*$D$45)</f>
       </c>
       <c r="I103" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H103))),"",H103*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H103))),"",H103*$D$55)</f>
       </c>
       <c r="J103" s="138">
         <f>IF(E103="","",MAX(0,E103-$G$44))</f>
@@ -3610,7 +3662,7 @@
         <v>0.9600000000000001</v>
       </c>
       <c r="D104" s="138">
-        <f>IF(C104&lt;$G$32,$G$48-MAX(0,(C104-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C104&lt;$D$54,$G$48-MAX(0,(C104-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E104" s="138">
         <f>IF(D104="","",$G$50/D104)</f>
@@ -3619,13 +3671,13 @@
         <f>IF(OR(D104="",E104=""),"",E104/D104)</f>
       </c>
       <c r="G104" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F104))),"",F104*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F104))),"",F104*$D$55)</f>
       </c>
       <c r="H104" s="138">
         <f>IF(NOT(ISNUMBER(F104)),"",F104*$D$45)</f>
       </c>
       <c r="I104" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H104))),"",H104*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H104))),"",H104*$D$55)</f>
       </c>
       <c r="J104" s="138">
         <f>IF(E104="","",MAX(0,E104-$G$44))</f>
@@ -3644,7 +3696,7 @@
         <v>0.9650000000000001</v>
       </c>
       <c r="D105" s="138">
-        <f>IF(C105&lt;$G$32,$G$48-MAX(0,(C105-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C105&lt;$D$54,$G$48-MAX(0,(C105-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E105" s="138">
         <f>IF(D105="","",$G$50/D105)</f>
@@ -3653,13 +3705,13 @@
         <f>IF(OR(D105="",E105=""),"",E105/D105)</f>
       </c>
       <c r="G105" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F105))),"",F105*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F105))),"",F105*$D$55)</f>
       </c>
       <c r="H105" s="138">
         <f>IF(NOT(ISNUMBER(F105)),"",F105*$D$45)</f>
       </c>
       <c r="I105" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H105))),"",H105*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H105))),"",H105*$D$55)</f>
       </c>
       <c r="J105" s="138">
         <f>IF(E105="","",MAX(0,E105-$G$44))</f>
@@ -3678,7 +3730,7 @@
         <v>0.9700000000000001</v>
       </c>
       <c r="D106" s="138">
-        <f>IF(C106&lt;$G$32,$G$48-MAX(0,(C106-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C106&lt;$D$54,$G$48-MAX(0,(C106-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E106" s="138">
         <f>IF(D106="","",$G$50/D106)</f>
@@ -3687,13 +3739,13 @@
         <f>IF(OR(D106="",E106=""),"",E106/D106)</f>
       </c>
       <c r="G106" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F106))),"",F106*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F106))),"",F106*$D$55)</f>
       </c>
       <c r="H106" s="138">
         <f>IF(NOT(ISNUMBER(F106)),"",F106*$D$45)</f>
       </c>
       <c r="I106" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H106))),"",H106*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H106))),"",H106*$D$55)</f>
       </c>
       <c r="J106" s="138">
         <f>IF(E106="","",MAX(0,E106-$G$44))</f>
@@ -3712,7 +3764,7 @@
         <v>0.9750000000000001</v>
       </c>
       <c r="D107" s="138">
-        <f>IF(C107&lt;$G$32,$G$48-MAX(0,(C107-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C107&lt;$D$54,$G$48-MAX(0,(C107-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E107" s="138">
         <f>IF(D107="","",$G$50/D107)</f>
@@ -3721,13 +3773,13 @@
         <f>IF(OR(D107="",E107=""),"",E107/D107)</f>
       </c>
       <c r="G107" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F107))),"",F107*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F107))),"",F107*$D$55)</f>
       </c>
       <c r="H107" s="138">
         <f>IF(NOT(ISNUMBER(F107)),"",F107*$D$45)</f>
       </c>
       <c r="I107" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H107))),"",H107*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H107))),"",H107*$D$55)</f>
       </c>
       <c r="J107" s="138">
         <f>IF(E107="","",MAX(0,E107-$G$44))</f>
@@ -3746,7 +3798,7 @@
         <v>0.98</v>
       </c>
       <c r="D108" s="138">
-        <f>IF(C108&lt;$G$32,$G$48-MAX(0,(C108-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C108&lt;$D$54,$G$48-MAX(0,(C108-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E108" s="138">
         <f>IF(D108="","",$G$50/D108)</f>
@@ -3755,13 +3807,13 @@
         <f>IF(OR(D108="",E108=""),"",E108/D108)</f>
       </c>
       <c r="G108" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F108))),"",F108*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F108))),"",F108*$D$55)</f>
       </c>
       <c r="H108" s="138">
         <f>IF(NOT(ISNUMBER(F108)),"",F108*$D$45)</f>
       </c>
       <c r="I108" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H108))),"",H108*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H108))),"",H108*$D$55)</f>
       </c>
       <c r="J108" s="138">
         <f>IF(E108="","",MAX(0,E108-$G$44))</f>
@@ -3780,7 +3832,7 @@
         <v>0.9850000000000001</v>
       </c>
       <c r="D109" s="138">
-        <f>IF(C109&lt;$G$32,$G$48-MAX(0,(C109-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C109&lt;$D$54,$G$48-MAX(0,(C109-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E109" s="138">
         <f>IF(D109="","",$G$50/D109)</f>
@@ -3789,13 +3841,13 @@
         <f>IF(OR(D109="",E109=""),"",E109/D109)</f>
       </c>
       <c r="G109" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F109))),"",F109*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F109))),"",F109*$D$55)</f>
       </c>
       <c r="H109" s="138">
         <f>IF(NOT(ISNUMBER(F109)),"",F109*$D$45)</f>
       </c>
       <c r="I109" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H109))),"",H109*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H109))),"",H109*$D$55)</f>
       </c>
       <c r="J109" s="138">
         <f>IF(E109="","",MAX(0,E109-$G$44))</f>
@@ -3814,7 +3866,7 @@
         <v>0.99</v>
       </c>
       <c r="D110" s="138">
-        <f>IF(C110&lt;$G$32,$G$48-MAX(0,(C110-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C110&lt;$D$54,$G$48-MAX(0,(C110-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E110" s="138">
         <f>IF(D110="","",$G$50/D110)</f>
@@ -3823,13 +3875,13 @@
         <f>IF(OR(D110="",E110=""),"",E110/D110)</f>
       </c>
       <c r="G110" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F110))),"",F110*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F110))),"",F110*$D$55)</f>
       </c>
       <c r="H110" s="138">
         <f>IF(NOT(ISNUMBER(F110)),"",F110*$D$45)</f>
       </c>
       <c r="I110" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H110))),"",H110*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H110))),"",H110*$D$55)</f>
       </c>
       <c r="J110" s="138">
         <f>IF(E110="","",MAX(0,E110-$G$44))</f>
@@ -3848,7 +3900,7 @@
         <v>0.9950000000000001</v>
       </c>
       <c r="D111" s="138">
-        <f>IF(C111&lt;$G$32,$G$48-MAX(0,(C111-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C111&lt;$D$54,$G$48-MAX(0,(C111-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E111" s="138">
         <f>IF(D111="","",$G$50/D111)</f>
@@ -3857,13 +3909,13 @@
         <f>IF(OR(D111="",E111=""),"",E111/D111)</f>
       </c>
       <c r="G111" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F111))),"",F111*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F111))),"",F111*$D$55)</f>
       </c>
       <c r="H111" s="138">
         <f>IF(NOT(ISNUMBER(F111)),"",F111*$D$45)</f>
       </c>
       <c r="I111" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H111))),"",H111*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H111))),"",H111*$D$55)</f>
       </c>
       <c r="J111" s="138">
         <f>IF(E111="","",MAX(0,E111-$G$44))</f>
@@ -3882,7 +3934,7 @@
         <v>1</v>
       </c>
       <c r="D112" s="139">
-        <f>IF(C112&lt;$G$32,$G$48-MAX(0,(C112-$G$43)*$D$45)/(1-$J$7),"")</f>
+        <f>IF(C112&lt;$D$54,$G$48-MAX(0,(C112-$G$43)*$D$45)/(1-$J$7),"")</f>
       </c>
       <c r="E112" s="139">
         <f>IF(D112="","",$G$50/D112)</f>
@@ -3891,13 +3943,13 @@
         <f>IF(OR(D112="",E112=""),"",E112/D112)</f>
       </c>
       <c r="G112" s="130">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F112))),"",F112*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F112))),"",F112*$D$55)</f>
       </c>
       <c r="H112" s="139">
         <f>IF(NOT(ISNUMBER(F112)),"",F112*$D$45)</f>
       </c>
       <c r="I112" s="139">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H112))),"",H112*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H112))),"",H112*$D$55)</f>
       </c>
       <c r="J112" s="139">
         <f>IF(E112="","",MAX(0,E112-$G$44))</f>
@@ -3999,13 +4051,13 @@
         <f>IF(OR(D117="",E117=""),"",E117/D117)</f>
       </c>
       <c r="G117" s="128">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F117))),"",F117*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F117))),"",F117*$D$55)</f>
       </c>
       <c r="H117" s="137">
         <f>IF(NOT(ISNUMBER(F117)),"",F117*$D$45)</f>
       </c>
       <c r="I117" s="137">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H117))),"",H117*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H117))),"",H117*$D$55)</f>
       </c>
       <c r="J117" s="125">
         <f>IF($H$117&gt;0,1-H117/$H$117,0)</f>
@@ -4029,13 +4081,13 @@
         <f>IF(OR(D118="",E118=""),"",E118/D118)</f>
       </c>
       <c r="G118" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F118))),"",F118*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F118))),"",F118*$D$55)</f>
       </c>
       <c r="H118" s="138">
         <f>IF(NOT(ISNUMBER(F118)),"",F118*$D$45)</f>
       </c>
       <c r="I118" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H118))),"",H118*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H118))),"",H118*$D$55)</f>
       </c>
       <c r="J118" s="126">
         <f>IF($H$117&gt;0,1-H118/$H$117,0)</f>
@@ -4059,13 +4111,13 @@
         <f>IF(OR(D119="",E119=""),"",E119/D119)</f>
       </c>
       <c r="G119" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F119))),"",F119*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F119))),"",F119*$D$55)</f>
       </c>
       <c r="H119" s="138">
         <f>IF(NOT(ISNUMBER(F119)),"",F119*$D$45)</f>
       </c>
       <c r="I119" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H119))),"",H119*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H119))),"",H119*$D$55)</f>
       </c>
       <c r="J119" s="126">
         <f>IF($H$117&gt;0,1-H119/$H$117,0)</f>
@@ -4089,13 +4141,13 @@
         <f>IF(OR(D120="",E120=""),"",E120/D120)</f>
       </c>
       <c r="G120" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F120))),"",F120*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F120))),"",F120*$D$55)</f>
       </c>
       <c r="H120" s="138">
         <f>IF(NOT(ISNUMBER(F120)),"",F120*$D$45)</f>
       </c>
       <c r="I120" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H120))),"",H120*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H120))),"",H120*$D$55)</f>
       </c>
       <c r="J120" s="126">
         <f>IF($H$117&gt;0,1-H120/$H$117,0)</f>
@@ -4119,13 +4171,13 @@
         <f>IF(OR(D121="",E121=""),"",E121/D121)</f>
       </c>
       <c r="G121" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F121))),"",F121*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F121))),"",F121*$D$55)</f>
       </c>
       <c r="H121" s="138">
         <f>IF(NOT(ISNUMBER(F121)),"",F121*$D$45)</f>
       </c>
       <c r="I121" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H121))),"",H121*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H121))),"",H121*$D$55)</f>
       </c>
       <c r="J121" s="126">
         <f>IF($H$117&gt;0,1-H121/$H$117,0)</f>
@@ -4149,13 +4201,13 @@
         <f>IF(OR(D122="",E122=""),"",E122/D122)</f>
       </c>
       <c r="G122" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F122))),"",F122*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F122))),"",F122*$D$55)</f>
       </c>
       <c r="H122" s="138">
         <f>IF(NOT(ISNUMBER(F122)),"",F122*$D$45)</f>
       </c>
       <c r="I122" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H122))),"",H122*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H122))),"",H122*$D$55)</f>
       </c>
       <c r="J122" s="126">
         <f>IF($H$117&gt;0,1-H122/$H$117,0)</f>
@@ -4179,13 +4231,13 @@
         <f>IF(OR(D123="",E123=""),"",E123/D123)</f>
       </c>
       <c r="G123" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F123))),"",F123*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F123))),"",F123*$D$55)</f>
       </c>
       <c r="H123" s="138">
         <f>IF(NOT(ISNUMBER(F123)),"",F123*$D$45)</f>
       </c>
       <c r="I123" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H123))),"",H123*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H123))),"",H123*$D$55)</f>
       </c>
       <c r="J123" s="126">
         <f>IF($H$117&gt;0,1-H123/$H$117,0)</f>
@@ -4209,13 +4261,13 @@
         <f>IF(OR(D124="",E124=""),"",E124/D124)</f>
       </c>
       <c r="G124" s="129">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F124))),"",F124*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F124))),"",F124*$D$55)</f>
       </c>
       <c r="H124" s="138">
         <f>IF(NOT(ISNUMBER(F124)),"",F124*$D$45)</f>
       </c>
       <c r="I124" s="138">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H124))),"",H124*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H124))),"",H124*$D$55)</f>
       </c>
       <c r="J124" s="126">
         <f>IF($H$117&gt;0,1-H124/$H$117,0)</f>
@@ -4239,13 +4291,13 @@
         <f>IF(OR(D125="",E125=""),"",E125/D125)</f>
       </c>
       <c r="G125" s="130">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(F125))),"",F125*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(F125))),"",F125*$D$55)</f>
       </c>
       <c r="H125" s="139">
         <f>IF(NOT(ISNUMBER(F125)),"",F125*$D$45)</f>
       </c>
       <c r="I125" s="139">
-        <f>IF(OR($D$33="",NOT(ISNUMBER(H125))),"",H125*$D$33)</f>
+        <f>IF(OR($D$55="",NOT(ISNUMBER(H125))),"",H125*$D$55)</f>
       </c>
       <c r="J125" s="127">
         <f>IF($H$117&gt;0,1-H125/$H$117,0)</f>
@@ -4622,8 +4674,7 @@
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="I22:L22"/>
     <mergeCell ref="I27:L27"/>
-    <mergeCell ref="D34:F34"/>
-    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="D56:E56"/>
   </mergeCells>
   <conditionalFormatting sqref="D23:D23">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="不可达"/>
@@ -4632,14 +4683,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J24:J24">
     <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="缺少"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D30:D30">
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="不可达"/>
-    <cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="无效"/>
-    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="缺少"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F35:F35">
-    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="缺少"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:D18">
     <cfRule type="expression" dxfId="8" priority="9">
@@ -4715,6 +4758,14 @@
     <cfRule type="expression" dxfId="22" priority="23">
       <formula>$D$7="BNB"</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D51:D51">
+    <cfRule type="containsText" dxfId="23" priority="24" operator="containsText" text="不可达"/>
+    <cfRule type="containsText" dxfId="24" priority="25" operator="containsText" text="无效"/>
+    <cfRule type="containsText" dxfId="25" priority="26" operator="containsText" text="缺少"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G55:G55">
+    <cfRule type="containsText" dxfId="26" priority="27" operator="containsText" text="缺少"/>
   </conditionalFormatting>
   <dataValidations count="11">
     <dataValidation type="list" sqref="D7">

</xml_diff>

<commit_message>
Unify calculator Excel defaults and daily 10000-USDT reserves
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R2dcc5bc14b1644b1"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R38df040599604895"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R7245ec62e2bb4f70"/>
+    <sheet name="Quote参数" sheetId="2" r:id="Rd65ad75769864cf4"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="145">
+  <x:cellXfs count="147">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -590,6 +590,12 @@
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1118,7 +1124,7 @@
         <v>目标控筹率</v>
       </c>
       <c r="D8" s="50" t="n">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="E8" s="35" t="str">
         <v>预算沿用 +1%</v>
@@ -1127,7 +1133,7 @@
         <v>内盘地址 / 套</v>
       </c>
       <c r="G8" s="49" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="35" t="str">
@@ -1153,7 +1159,7 @@
         <v>外盘地址数</v>
       </c>
       <c r="G9" s="49" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1171,7 +1177,7 @@
         <v>Holder 地址数</v>
       </c>
       <c r="G10" s="49" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -1206,8 +1212,8 @@
       <c r="F12" s="35" t="str">
         <v>资金预留 / Quote</v>
       </c>
-      <c r="G12" s="51" t="n">
-        <v>0</v>
+      <c r="G12" s="146">
+        <f>IF(AND(ISNUMBER($D$55),$D$55&gt;0),ROUNDUP($G$56/$D$55,0),"")</f>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1219,7 +1225,7 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="52" t="str">
-        <v>手动价格只用于 USDT 换算，不改变 Quote 控筹预算。清空覆盖格后恢复自动取价。</v>
+        <v>预留资金 = 10,000 USDT ÷ Quote 价格，向上取整。手动价格会同时调整预留与折算价值；清空后恢复每日价。</v>
       </c>
       <c r="D13" s="52"/>
       <c r="E13" s="52"/>
@@ -2115,8 +2121,12 @@
         <f>IF(VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$14:$Q$36,13,FALSE))</f>
       </c>
       <c r="E56" s="101"/>
-      <c r="F56" s="101"/>
-      <c r="G56" s="102"/>
+      <c r="F56" s="101" t="str">
+        <v>预留预算 / USDT</v>
+      </c>
+      <c r="G56" s="105" t="n">
+        <v>10000</v>
+      </c>
       <c r="H56" s="101"/>
       <c r="I56" s="101" t="str">
         <v>洗后外盘 Pool TOKEN</v>
@@ -5007,14 +5017,14 @@
       <c r="N7" s="35"/>
       <c r="O7" s="35"/>
       <c r="P7" s="44">
-        <v>754.0686961856693</v>
+        <v>754.5107710045597</v>
       </c>
       <c r="Q7" s="45">
-        <v>46283.34975868055</v>
+        <v>46283.37613721065</v>
       </c>
       <c r="R7" s="35" t="inlineStr">
         <is>
-          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin&amp;vs_currencies=usd</t>
+          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether,ethereum,binancecoin,solana,hyperliquid,aster-2&amp;vs_currencies=usd</t>
         </is>
       </c>
       <c r="S7" s="35" t="inlineStr">
@@ -5242,10 +5252,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P14" s="26">
-        <v>155.8372</v>
+        <v>156.0833</v>
       </c>
       <c r="Q14" s="29">
-        <v>46283.3493256713</v>
+        <v>46283.37570457176</v>
       </c>
       <c r="R14" s="32" t="inlineStr">
         <is>
@@ -5301,10 +5311,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P15" s="27">
-        <v>186.7124</v>
+        <v>186.7097</v>
       </c>
       <c r="Q15" s="30">
-        <v>46283.34933046296</v>
+        <v>46283.37570887732</v>
       </c>
       <c r="R15" s="33" t="inlineStr">
         <is>
@@ -5360,10 +5370,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P16" s="27">
-        <v>764.4157</v>
+        <v>764.4747</v>
       </c>
       <c r="Q16" s="30">
-        <v>46283.34933644676</v>
+        <v>46283.375714953705</v>
       </c>
       <c r="R16" s="33" t="inlineStr">
         <is>
@@ -5419,10 +5429,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P17" s="27">
-        <v>4391.7337</v>
+        <v>4392.5405</v>
       </c>
       <c r="Q17" s="30">
-        <v>46283.349342326386</v>
+        <v>46283.375720717595</v>
       </c>
       <c r="R17" s="33" t="inlineStr">
         <is>
@@ -5478,10 +5488,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P18" s="27">
-        <v>721.7453</v>
+        <v>721.08824</v>
       </c>
       <c r="Q18" s="30">
-        <v>46283.34934763889</v>
+        <v>46283.37572564815</v>
       </c>
       <c r="R18" s="33" t="inlineStr">
         <is>
@@ -5537,10 +5547,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P19" s="27">
-        <v>221.7181</v>
+        <v>221.7199</v>
       </c>
       <c r="Q19" s="30">
-        <v>46283.3493534375</v>
+        <v>46283.375732326385</v>
       </c>
       <c r="R19" s="33" t="inlineStr">
         <is>
@@ -5596,10 +5606,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P20" s="27">
-        <v>337.03562</v>
+        <v>337.04141</v>
       </c>
       <c r="Q20" s="30">
-        <v>46283.349359155094</v>
+        <v>46283.37574059028</v>
       </c>
       <c r="R20" s="33" t="inlineStr">
         <is>
@@ -5655,10 +5665,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P21" s="27">
-        <v>369.434</v>
+        <v>369.7037</v>
       </c>
       <c r="Q21" s="30">
-        <v>46283.34936508102</v>
+        <v>46283.375743055556</v>
       </c>
       <c r="R21" s="33" t="inlineStr">
         <is>
@@ -5714,10 +5724,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P22" s="27">
-        <v>498.6768</v>
+        <v>498.6779</v>
       </c>
       <c r="Q22" s="30">
-        <v>46283.349370324075</v>
+        <v>46283.375749467596</v>
       </c>
       <c r="R22" s="33" t="inlineStr">
         <is>
@@ -5773,10 +5783,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P23" s="27">
-        <v>354.4693</v>
+        <v>354.4855</v>
       </c>
       <c r="Q23" s="30">
-        <v>46283.349375972226</v>
+        <v>46283.375755497684</v>
       </c>
       <c r="R23" s="33" t="inlineStr">
         <is>
@@ -5832,10 +5842,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P24" s="27">
-        <v>112.8313</v>
+        <v>113.3925</v>
       </c>
       <c r="Q24" s="30">
-        <v>46283.34938252315</v>
+        <v>46283.37576112269</v>
       </c>
       <c r="R24" s="33" t="inlineStr">
         <is>
@@ -5891,10 +5901,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P25" s="27">
-        <v>111.5313</v>
+        <v>111.4531</v>
       </c>
       <c r="Q25" s="30">
-        <v>46283.3493882176</v>
+        <v>46283.375766261575</v>
       </c>
       <c r="R25" s="33" t="inlineStr">
         <is>
@@ -5950,10 +5960,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P26" s="27">
-        <v>22.8497</v>
+        <v>22.8417</v>
       </c>
       <c r="Q26" s="30">
-        <v>46283.34939391204</v>
+        <v>46283.375775706016</v>
       </c>
       <c r="R26" s="33" t="inlineStr">
         <is>
@@ -6009,10 +6019,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P27" s="27">
-        <v>75.7422</v>
+        <v>75.7326</v>
       </c>
       <c r="Q27" s="30">
-        <v>46283.349399872684</v>
+        <v>46283.375779375</v>
       </c>
       <c r="R27" s="33" t="inlineStr">
         <is>
@@ -6068,10 +6078,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P28" s="27">
-        <v>136.1389</v>
+        <v>137.3979</v>
       </c>
       <c r="Q28" s="30">
-        <v>46283.34940596065</v>
+        <v>46283.3757871875</v>
       </c>
       <c r="R28" s="33" t="inlineStr">
         <is>
@@ -6127,10 +6137,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P29" s="27">
-        <v>8.7341</v>
+        <v>8.7287</v>
       </c>
       <c r="Q29" s="30">
-        <v>46283.34941131945</v>
+        <v>46283.37578998843</v>
       </c>
       <c r="R29" s="33" t="inlineStr">
         <is>
@@ -6186,10 +6196,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P30" s="27">
-        <v>43.4689</v>
+        <v>43.7069</v>
       </c>
       <c r="Q30" s="30">
-        <v>46283.34941725695</v>
+        <v>46283.375795960645</v>
       </c>
       <c r="R30" s="33" t="inlineStr">
         <is>
@@ -6245,10 +6255,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P31" s="27">
-        <v>118.9817</v>
+        <v>118.406</v>
       </c>
       <c r="Q31" s="30">
-        <v>46283.349422071755</v>
+        <v>46283.37580177083</v>
       </c>
       <c r="R31" s="33" t="inlineStr">
         <is>
@@ -6304,10 +6314,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P32" s="27">
-        <v>161.5949</v>
+        <v>161.977</v>
       </c>
       <c r="Q32" s="30">
-        <v>46283.34942886574</v>
+        <v>46283.37581027778</v>
       </c>
       <c r="R32" s="33" t="inlineStr">
         <is>
@@ -6363,10 +6373,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P33" s="27">
-        <v>7.8747</v>
+        <v>7.8752</v>
       </c>
       <c r="Q33" s="30">
-        <v>46283.34943337963</v>
+        <v>46283.375813287035</v>
       </c>
       <c r="R33" s="33" t="inlineStr">
         <is>
@@ -6422,10 +6432,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P34" s="27">
-        <v>34.5871</v>
+        <v>34.5876</v>
       </c>
       <c r="Q34" s="30">
-        <v>46283.349439502315</v>
+        <v>46283.37581939815</v>
       </c>
       <c r="R34" s="33" t="inlineStr">
         <is>
@@ -6481,10 +6491,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P35" s="27">
-        <v>24.6759</v>
+        <v>24.6852</v>
       </c>
       <c r="Q35" s="30">
-        <v>46283.349445266205</v>
+        <v>46283.37582730324</v>
       </c>
       <c r="R35" s="33" t="inlineStr">
         <is>
@@ -6545,7 +6555,7 @@
         </is>
       </c>
       <c r="Q36" s="31">
-        <v>46283.34945219907</v>
+        <v>46283.375830034725</v>
       </c>
       <c r="R36" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Price BNC4 from user-selected USDT pool across web and Excel
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -5017,10 +5017,10 @@
       <c r="N7" s="35"/>
       <c r="O7" s="35"/>
       <c r="P7" s="44">
-        <v>754.1006248142221</v>
+        <v>752.7144296870387</v>
       </c>
       <c r="Q7" s="45">
-        <v>46283.38506050926</v>
+        <v>46283.396544745374</v>
       </c>
       <c r="R7" s="35" t="inlineStr">
         <is>
@@ -5252,10 +5252,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P14" s="26">
-        <v>156.08842</v>
+        <v>156.08477</v>
       </c>
       <c r="Q14" s="29">
-        <v>46283.38462777778</v>
+        <v>46283.39609806713</v>
       </c>
       <c r="R14" s="32" t="inlineStr">
         <is>
@@ -5311,10 +5311,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P15" s="27">
-        <v>186.7088</v>
+        <v>186.5263</v>
       </c>
       <c r="Q15" s="30">
-        <v>46283.38463231481</v>
+        <v>46283.39610212963</v>
       </c>
       <c r="R15" s="33" t="inlineStr">
         <is>
@@ -5370,10 +5370,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P16" s="27">
-        <v>764.357</v>
+        <v>764.05131</v>
       </c>
       <c r="Q16" s="30">
-        <v>46283.38463807871</v>
+        <v>46283.39611925926</v>
       </c>
       <c r="R16" s="33" t="inlineStr">
         <is>
@@ -5429,10 +5429,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P17" s="27">
-        <v>4394.9249</v>
+        <v>4385.5977</v>
       </c>
       <c r="Q17" s="30">
-        <v>46283.38464387731</v>
+        <v>46283.39612380787</v>
       </c>
       <c r="R17" s="33" t="inlineStr">
         <is>
@@ -5488,10 +5488,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P18" s="27">
-        <v>720.9937</v>
+        <v>720.705</v>
       </c>
       <c r="Q18" s="30">
-        <v>46283.38465034722</v>
+        <v>46283.39612625</v>
       </c>
       <c r="R18" s="33" t="inlineStr">
         <is>
@@ -5547,10 +5547,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P19" s="27">
-        <v>221.6962</v>
+        <v>221.6845</v>
       </c>
       <c r="Q19" s="30">
-        <v>46283.38465541667</v>
+        <v>46283.39613197916</v>
       </c>
       <c r="R19" s="33" t="inlineStr">
         <is>
@@ -5606,10 +5606,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P20" s="27">
-        <v>337.02364</v>
+        <v>337.02721</v>
       </c>
       <c r="Q20" s="30">
-        <v>46283.38466121528</v>
+        <v>46283.396137800926</v>
       </c>
       <c r="R20" s="33" t="inlineStr">
         <is>
@@ -5665,10 +5665,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P21" s="27">
-        <v>369.6742</v>
+        <v>369.5238</v>
       </c>
       <c r="Q21" s="30">
-        <v>46283.38466707176</v>
+        <v>46283.39614362268</v>
       </c>
       <c r="R21" s="33" t="inlineStr">
         <is>
@@ -5724,10 +5724,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P22" s="27">
-        <v>498.6777</v>
+        <v>498.6181</v>
       </c>
       <c r="Q22" s="30">
-        <v>46283.3846728125</v>
+        <v>46283.396153217596</v>
       </c>
       <c r="R22" s="33" t="inlineStr">
         <is>
@@ -5783,10 +5783,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P23" s="27">
-        <v>354.7571</v>
+        <v>354.758</v>
       </c>
       <c r="Q23" s="30">
-        <v>46283.384678599534</v>
+        <v>46283.39615923611</v>
       </c>
       <c r="R23" s="33" t="inlineStr">
         <is>
@@ -5842,10 +5842,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P24" s="27">
-        <v>113.5559</v>
+        <v>113.8666</v>
       </c>
       <c r="Q24" s="30">
-        <v>46283.384684375</v>
+        <v>46283.396163923615</v>
       </c>
       <c r="R24" s="33" t="inlineStr">
         <is>
@@ -5901,10 +5901,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P25" s="27">
-        <v>111.4438</v>
+        <v>111.4257</v>
       </c>
       <c r="Q25" s="30">
-        <v>46283.38469018519</v>
+        <v>46283.39616679398</v>
       </c>
       <c r="R25" s="33" t="inlineStr">
         <is>
@@ -5960,10 +5960,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P26" s="27">
-        <v>22.8154</v>
+        <v>22.8109</v>
       </c>
       <c r="Q26" s="30">
-        <v>46283.3846959838</v>
+        <v>46283.39617341435</v>
       </c>
       <c r="R26" s="33" t="inlineStr">
         <is>
@@ -6019,10 +6019,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P27" s="27">
-        <v>74.01945</v>
+        <v>73.8456</v>
       </c>
       <c r="Q27" s="30">
-        <v>46283.38470174769</v>
+        <v>46283.39617832176</v>
       </c>
       <c r="R27" s="33" t="inlineStr">
         <is>
@@ -6078,10 +6078,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P28" s="27">
-        <v>137.8229</v>
+        <v>138.005012</v>
       </c>
       <c r="Q28" s="30">
-        <v>46283.38470755787</v>
+        <v>46283.396187847226</v>
       </c>
       <c r="R28" s="33" t="inlineStr">
         <is>
@@ -6137,10 +6137,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P29" s="27">
-        <v>8.7682</v>
+        <v>8.7136</v>
       </c>
       <c r="Q29" s="30">
-        <v>46283.384713900465</v>
+        <v>46283.39619075231</v>
       </c>
       <c r="R29" s="33" t="inlineStr">
         <is>
@@ -6196,10 +6196,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P30" s="27">
-        <v>43.6176</v>
+        <v>43.6805</v>
       </c>
       <c r="Q30" s="30">
-        <v>46283.38471917824</v>
+        <v>46283.39619640046</v>
       </c>
       <c r="R30" s="33" t="inlineStr">
         <is>
@@ -6255,10 +6255,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P31" s="27">
-        <v>118.2157</v>
+        <v>118.4043</v>
       </c>
       <c r="Q31" s="30">
-        <v>46283.384724999996</v>
+        <v>46283.39620527778</v>
       </c>
       <c r="R31" s="33" t="inlineStr">
         <is>
@@ -6314,10 +6314,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P32" s="27">
-        <v>161.8943</v>
+        <v>161.695</v>
       </c>
       <c r="Q32" s="30">
-        <v>46283.38473100694</v>
+        <v>46283.39620826389</v>
       </c>
       <c r="R32" s="33" t="inlineStr">
         <is>
@@ -6373,10 +6373,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P33" s="27">
-        <v>7.8741</v>
+        <v>7.6772</v>
       </c>
       <c r="Q33" s="30">
-        <v>46283.384736643515</v>
+        <v>46283.39621385417</v>
       </c>
       <c r="R33" s="33" t="inlineStr">
         <is>
@@ -6432,10 +6432,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P34" s="27">
-        <v>34.5918</v>
+        <v>34.5884</v>
       </c>
       <c r="Q34" s="30">
-        <v>46283.38474232639</v>
+        <v>46283.39622255787</v>
       </c>
       <c r="R34" s="33" t="inlineStr">
         <is>
@@ -6491,10 +6491,10 @@
         <v>2026-09-10</v>
       </c>
       <c r="P35" s="27">
-        <v>24.8277</v>
+        <v>24.759</v>
       </c>
       <c r="Q35" s="30">
-        <v>46283.38474876158</v>
+        <v>46283.39622539352</v>
       </c>
       <c r="R35" s="33" t="inlineStr">
         <is>
@@ -6555,7 +6555,7 @@
         </is>
       </c>
       <c r="Q36" s="31">
-        <v>46283.384753900464</v>
+        <v>46283.396232499996</v>
       </c>
       <c r="R36" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Classify external fee assets in control workbooks
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R7245ec62e2bb4f70"/>
-    <sheet name="Quote参数" sheetId="2" r:id="Rd65ad75769864cf4"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rb0b511ce09834359"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R1a974b74ae194c3a"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -163,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="147">
+  <x:cellXfs count="149">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -596,6 +596,12 @@
     </x:xf>
     <x:xf numFmtId="208" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -608,7 +614,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -619,7 +625,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -630,7 +636,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -641,7 +647,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -652,7 +658,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -663,7 +669,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -674,7 +680,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -685,7 +691,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -741,7 +747,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -752,7 +758,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -763,7 +769,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -774,7 +780,7 @@
         <x:color rgb="FF7D2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -1487,7 +1493,7 @@
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="101" t="str">
-        <v>恢复目标控筹资金</v>
+        <v>恢复目标控筹预留</v>
       </c>
       <c r="D26" s="115">
         <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)))</f>
@@ -1585,7 +1591,7 @@
       <c r="K30" s="100"/>
       <c r="L30" s="100"/>
     </row>
-    <row r="31" customHeight="1" hidden="1">
+    <row r="31" hidden="1" customHeight="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31"/>
@@ -1599,7 +1605,7 @@
       <c r="K31" s="100"/>
       <c r="L31" s="100"/>
     </row>
-    <row r="32" customHeight="1" hidden="1">
+    <row r="32" hidden="1" customHeight="1">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32"/>
@@ -1613,7 +1619,7 @@
       <c r="K32" s="100"/>
       <c r="L32" s="100"/>
     </row>
-    <row r="33" customHeight="1" hidden="1">
+    <row r="33" hidden="1" customHeight="1">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33"/>
@@ -1627,7 +1633,7 @@
       <c r="K33" s="100"/>
       <c r="L33" s="100"/>
     </row>
-    <row r="34" customHeight="1" hidden="1">
+    <row r="34" hidden="1" customHeight="1">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34"/>
@@ -1641,7 +1647,7 @@
       <c r="K34" s="100"/>
       <c r="L34" s="100"/>
     </row>
-    <row r="35" customHeight="1" hidden="1">
+    <row r="35" hidden="1" customHeight="1">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35"/>
@@ -1655,11 +1661,11 @@
       <c r="K35" s="100"/>
       <c r="L35" s="100"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="36" customHeight="1">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="108" t="str">
-        <v>目标持仓直接 Quote 洗一轮，无额外路由费。控筹下降为小单固定价近似，补回资金为外盘曲线差额（含买税与 LP）。损耗仍按目标+1% FDV；补回是额外保守预留，非逐笔交易模拟。</v>
+        <v>外盘 Pancake LP 费从输入币收取：卖出腿扣 TOKEN，买入腿扣 Quote；Tax V3 买税扣输出 TOKEN、卖税扣输入 TOKEN。洗后控筹只按实际扣 TOKEN 的一侧 LP 费及买卖税折减，补回按曲线差额估算。</v>
       </c>
       <c r="D36" s="108"/>
       <c r="E36" s="108"/>
@@ -1721,7 +1727,7 @@
       <c r="K39" s="8"/>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="40" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A40"/>
       <c r="B40"/>
       <c r="C40" s="101" t="str">
@@ -1741,7 +1747,7 @@
       <c r="K40" s="101"/>
       <c r="L40" s="101"/>
     </row>
-    <row r="41" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="41" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A41"/>
       <c r="B41"/>
       <c r="C41" s="101" t="str">
@@ -1767,7 +1773,7 @@
       <c r="K41" s="101"/>
       <c r="L41" s="101"/>
     </row>
-    <row r="42" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="42" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A42"/>
       <c r="B42"/>
       <c r="C42" s="101" t="str">
@@ -1793,7 +1799,7 @@
       <c r="K42" s="101"/>
       <c r="L42" s="101"/>
     </row>
-    <row r="43" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="43" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A43"/>
       <c r="B43"/>
       <c r="C43" s="101"/>
@@ -1815,7 +1821,7 @@
       <c r="K43" s="101"/>
       <c r="L43" s="101"/>
     </row>
-    <row r="44" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="44" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A44"/>
       <c r="B44"/>
       <c r="C44" s="101" t="str">
@@ -1841,7 +1847,7 @@
       <c r="K44" s="101"/>
       <c r="L44" s="101"/>
     </row>
-    <row r="45" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="45" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A45"/>
       <c r="B45"/>
       <c r="C45" s="101" t="str">
@@ -1867,7 +1873,7 @@
       <c r="K45" s="101"/>
       <c r="L45" s="101"/>
     </row>
-    <row r="46" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="46" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A46"/>
       <c r="B46"/>
       <c r="C46" s="101" t="str">
@@ -1893,7 +1899,7 @@
       <c r="K46" s="101"/>
       <c r="L46" s="101"/>
     </row>
-    <row r="47" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="47" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A47"/>
       <c r="B47"/>
       <c r="C47" s="101" t="str">
@@ -1919,7 +1925,7 @@
       <c r="K47" s="101"/>
       <c r="L47" s="101"/>
     </row>
-    <row r="48" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="48" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A48"/>
       <c r="B48"/>
       <c r="C48" s="101" t="str">
@@ -1945,7 +1951,7 @@
       <c r="K48" s="101"/>
       <c r="L48" s="101"/>
     </row>
-    <row r="49" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="49" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A49"/>
       <c r="B49"/>
       <c r="C49" s="101" t="str">
@@ -1971,7 +1977,7 @@
       <c r="K49" s="101"/>
       <c r="L49" s="101"/>
     </row>
-    <row r="50" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="50" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A50"/>
       <c r="B50"/>
       <c r="C50" s="101"/>
@@ -1989,7 +1995,7 @@
       <c r="K50" s="101"/>
       <c r="L50" s="101"/>
     </row>
-    <row r="51" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="51" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A51"/>
       <c r="B51"/>
       <c r="C51" s="101" t="str">
@@ -2015,7 +2021,7 @@
       <c r="K51" s="101"/>
       <c r="L51" s="101"/>
     </row>
-    <row r="52" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="52" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A52"/>
       <c r="B52"/>
       <c r="C52" s="101" t="str">
@@ -2037,7 +2043,7 @@
       <c r="K52" s="101"/>
       <c r="L52" s="101"/>
     </row>
-    <row r="53" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="53" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A53"/>
       <c r="B53"/>
       <c r="C53" s="101" t="str">
@@ -2059,7 +2065,7 @@
       <c r="K53" s="101"/>
       <c r="L53" s="101"/>
     </row>
-    <row r="54" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="54" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A54"/>
       <c r="B54"/>
       <c r="C54" s="101" t="str">
@@ -2080,12 +2086,12 @@
         <v>洗后持仓保留比例</v>
       </c>
       <c r="J54" s="106">
-        <f>(1-$J$7)*(1-$J$8)*(1-$G$42)^2</f>
+        <f>(1-$J$7)*(1-$J$8)*(1-$G$42)</f>
       </c>
       <c r="K54" s="101"/>
       <c r="L54" s="101"/>
     </row>
-    <row r="55" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="55" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A55"/>
       <c r="B55"/>
       <c r="C55" s="101" t="str">
@@ -2111,7 +2117,7 @@
       <c r="K55" s="101"/>
       <c r="L55" s="101"/>
     </row>
-    <row r="56" ht="30" customHeight="1" outlineLevel="1" hidden="1">
+    <row r="56" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="A56"/>
       <c r="B56"/>
       <c r="C56" s="101" t="str">
@@ -4840,7 +4846,7 @@
     <col min="13" max="13" width="22" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="18" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="16" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="20" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="46" hidden="0" customWidth="1"/>
     <col min="17" max="17" width="22" hidden="0" customWidth="1"/>
     <col min="18" max="18" width="46" hidden="0" customWidth="1"/>
     <col min="19" max="19" width="30" hidden="0" customWidth="1"/>
@@ -5133,25 +5139,31 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
+      <c r="C12" s="148" t="str">
+        <v>外盘扣费依据</v>
+      </c>
+      <c r="D12" s="148"/>
+      <c r="E12" s="148" t="str">
+        <v>PancakeSwap 交易手续费从输入金额扣除；卖出腿输入为 TOKEN。</v>
+      </c>
+      <c r="F12" s="148"/>
+      <c r="G12" s="148"/>
+      <c r="H12" s="148"/>
+      <c r="I12" s="148"/>
+      <c r="J12" s="148"/>
+      <c r="K12" s="148"/>
+      <c r="L12" s="148"/>
+      <c r="M12" s="148"/>
+      <c r="N12" s="148"/>
+      <c r="O12" s="148"/>
+      <c r="P12" s="148" t="str">
+        <v>https://docs.pancakeswap.finance/trade/pancakeswap-exchange/trade</v>
+      </c>
+      <c r="Q12" s="148"/>
+      <c r="R12" s="148"/>
       <c r="S12" s="2"/>
     </row>
     <row r="13" ht="44" customHeight="1">

</xml_diff>

<commit_message>
Apply quote-leg pricing to Pons outer model
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Rb0b511ce09834359"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R1a974b74ae194c3a"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R460505bc6e094336"/>
+    <sheet name="Quote参数" sheetId="2" r:id="Rda67499a124f4f98"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>

</xml_diff>

<commit_message>
Model self-funded outer-market wash recovery in Excel
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R460505bc6e094336"/>
-    <sheet name="Quote参数" sheetId="2" r:id="Rda67499a124f4f98"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rca26cecaf76542b3"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R2deb1b30251a478e"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1496,7 +1496,7 @@
         <v>恢复目标控筹预留</v>
       </c>
       <c r="D26" s="115">
-        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)))</f>
+        <f>IF($D$51&lt;&gt;"可达","",0)</f>
       </c>
       <c r="E26" s="100">
         <f>$D$7</f>
@@ -1533,7 +1533,7 @@
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="101" t="str">
-        <v>补回目标控筹率</v>
+        <v>原目标控筹率</v>
       </c>
       <c r="D28" s="117">
         <f>$D$8</f>
@@ -1665,7 +1665,7 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="108" t="str">
-        <v>外盘 Pancake LP 费从输入币收取：卖出腿扣 TOKEN，买入腿扣 Quote；Tax V3 买税扣输出 TOKEN、卖税扣输入 TOKEN。洗后控筹只按实际扣 TOKEN 的一侧 LP 费及买卖税折减，补回按曲线差额估算。</v>
+        <v>外盘一卖一买：卖出所得 Quote 全额用于回买，不额外补 Quote。洗后控筹按卖出、买入两腿含税费率同价估算；实际成交量、滑点与价格冲击未计入。洗筹损耗另按预算 FDV × 双边费率列示。</v>
       </c>
       <c r="D36" s="108"/>
       <c r="E36" s="108"/>
@@ -2086,7 +2086,7 @@
         <v>洗后持仓保留比例</v>
       </c>
       <c r="J54" s="106">
-        <f>(1-$J$7)*(1-$J$8)*(1-$G$42)</f>
+        <f>MAX(0,1-$J$29)*MAX(0,1-$J$30)</f>
       </c>
       <c r="K54" s="101"/>
       <c r="L54" s="101"/>
@@ -5120,7 +5120,9 @@
       <c r="C11" s="35" t="str">
         <v>税率口径</v>
       </c>
-      <c r="D11" s="35"/>
+      <c r="D11" s="35" t="str">
+        <v>外盘卖出所得 Quote 用于回买，不额外补 Quote；双边 LP 费和买卖税降低洗后持币，预留为 0。</v>
+      </c>
       <c r="E11" s="35" t="str">
         <v>​Tax V3 买税/卖税逐币设置。内盘税作为额外 Quote 费；DEX 买税从 TOKEN 输出扣除。</v>
       </c>

</xml_diff>

<commit_message>
Reserve quote to restore post-wash control target
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Rca26cecaf76542b3"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R2deb1b30251a478e"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Ree9c4e9602624388"/>
+    <sheet name="Quote参数" sheetId="2" r:id="Rff154de45f2d40ad"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1496,7 +1496,7 @@
         <v>恢复目标控筹预留</v>
       </c>
       <c r="D26" s="115">
-        <f>IF($D$51&lt;&gt;"可达","",0)</f>
+        <f>IF($D$51&lt;&gt;"可达","",IF(AND($J$55&gt;0,$J$56&gt;0),MAX(0,($G$50/$J$55-$G$50/$J$56)*(1+$G$42)),""))</f>
       </c>
       <c r="E26" s="100">
         <f>$D$7</f>
@@ -1665,7 +1665,7 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="108" t="str">
-        <v>外盘一卖一买：卖出所得 Quote 全额用于回买，不额外补 Quote。洗后控筹按卖出、买入两腿含税费率同价估算；实际成交量、滑点与价格冲击未计入。洗筹损耗另按预算 FDV × 双边费率列示。</v>
+        <v>外盘一卖一买使用卖出所得 Quote 回买；洗后若低于目标，再按外盘曲线差额及买入费预留恢复所需 Quote。洗筹损耗另列；未模拟成交量、滑点与价格冲击。</v>
       </c>
       <c r="D36" s="108"/>
       <c r="E36" s="108"/>
@@ -5121,7 +5121,7 @@
         <v>税率口径</v>
       </c>
       <c r="D11" s="35" t="str">
-        <v>外盘卖出所得 Quote 用于回买，不额外补 Quote；双边 LP 费和买卖税降低洗后持币，预留为 0。</v>
+        <v>外盘卖出所得 Quote 用于回买；双边 LP 费与买卖税降低持币。恢复目标按外盘曲线差额及买入费另列。</v>
       </c>
       <c r="E11" s="35" t="str">
         <v>​Tax V3 买税/卖税逐币设置。内盘税作为额外 Quote 费；DEX 买税从 TOKEN 输出扣除。</v>

</xml_diff>

<commit_message>
Regenerate recovery-only downloads with current prices
</commit_message>
<xml_diff>
--- a/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/latest/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="Ree9c4e9602624388"/>
-    <sheet name="Quote参数" sheetId="2" r:id="Rff154de45f2d40ad"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rdfcf5d9f72a04e52"/>
+    <sheet name="Quote参数" sheetId="2" r:id="Rc51882bdca6f4145"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="10">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
@@ -26,6 +26,7 @@
     <x:numFmt numFmtId="207" formatCode="0.0000%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0.0000000000"/>
+    <x:numFmt numFmtId="210" formatCode=";;;"/>
   </x:numFmts>
   <x:fonts count="12">
     <x:font>
@@ -163,7 +164,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="149">
+  <x:cellXfs count="150">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -602,6 +603,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1308,7 +1312,7 @@
         <v>建议 Quote 资金</v>
       </c>
       <c r="D18" s="114">
-        <f>IF(ISNUMBER($D$26),(IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($D$22="","",SUM($D$22,$D$23,$D$24,$D$25))))+$D$26,"")</f>
+        <f>IF(AND(LEFT($D$51,2)="可达",ISNUMBER($D$22),ISNUMBER($D$23),ISNUMBER($D$25),ISNUMBER($D$26)),SUM($D$22:$D$23,$D$25:$D$26),"")</f>
       </c>
       <c r="E18" s="58">
         <f>$D$7</f>
@@ -1441,15 +1445,11 @@
       <c r="K23" s="100"/>
       <c r="L23" s="100"/>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" customHeight="1" hidden="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="101" t="str">
-        <v>洗筹损耗</v>
-      </c>
-      <c r="D24" s="115">
-        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($J$46="","",$J$46*$J$47))</f>
-      </c>
+      <c r="C24" s="101"/>
+      <c r="D24" s="149"/>
       <c r="E24" s="100">
         <f>$D$7</f>
       </c>
@@ -1665,7 +1665,7 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="108" t="str">
-        <v>外盘一卖一买使用卖出所得 Quote 回买；洗后若低于目标，再按外盘曲线差额及买入费预留恢复所需 Quote。洗筹损耗另列；未模拟成交量、滑点与价格冲击。</v>
+        <v>外盘一卖一买使用卖出所得 Quote 回买；手续费仅降低洗后持币，不另列资金。洗后若低于目标，再按外盘曲线差额及买入费预留恢复所需 Quote；未模拟成交量、滑点与价格冲击。</v>
       </c>
       <c r="D36" s="108"/>
       <c r="E36" s="108"/>

</xml_diff>